<commit_message>
Add DTOs and repository methods for financial reporting
- Created WorkingAdministrativeExpenseDto, WorkingAssetsDto, and WorkingEPFETFDto for handling administrative expenses, assets, and EPF/ETF data respectively.
- Introduced WORKING DTO to aggregate financial data including interest income, administrative expenses, assets, and EPF/ETF contributions.
- Implemented new methods in LoanRepository and PettyCashRepository to fetch approved loans and petty cash transactions within a date range.
- Added a method in SalaryRepository to retrieve EPF contributions over a specified date range.
- Updated FinancialStatementService and its implementation to generate financial reports, including the new working report.
- Refactored existing code to accommodate the new data structures and ensure proper data aggregation for financial reporting.
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193420E6-1C9F-4B43-AF6D-66B78887498E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F11B7C-4E3E-4FA2-A322-DBD248476C6B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPE" sheetId="24" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="200">
   <si>
     <t>STATEMENT OF FINANCIAL POSITION</t>
   </si>
@@ -549,37 +549,13 @@
     <t>TIN NO. 111350027</t>
   </si>
   <si>
-    <t xml:space="preserve">Expenses </t>
-  </si>
-  <si>
     <t>Advertisment &amp; Sales Promotion</t>
   </si>
   <si>
     <t>Bad Debts</t>
   </si>
   <si>
-    <t>Commission</t>
-  </si>
-  <si>
-    <t>EPF &amp; Etf</t>
-  </si>
-  <si>
-    <t>Rent</t>
-  </si>
-  <si>
-    <t>Maintance &amp; Repair</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phone &amp; Internet bills </t>
-  </si>
-  <si>
-    <t>Company Incorporation fees</t>
-  </si>
-  <si>
     <t>Insurance</t>
-  </si>
-  <si>
-    <t>Stationery &amp; Documents</t>
   </si>
   <si>
     <t>Income</t>
@@ -692,6 +668,12 @@
   <si>
     <t>Kuruwita</t>
   </si>
+  <si>
+    <t>Administrative Expenses</t>
+  </si>
+  <si>
+    <t>EPF ETF</t>
+  </si>
 </sst>
 </file>
 
@@ -703,7 +685,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -863,6 +845,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -976,7 +966,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="240">
+  <cellXfs count="241">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1472,6 +1462,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1958,7 +1949,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.109375" style="44" bestFit="1" customWidth="1"/>
@@ -1996,7 +1987,7 @@
         <v>123</v>
       </c>
       <c r="F3" s="143" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="G3" s="143" t="s">
         <v>124</v>
@@ -2019,7 +2010,7 @@
         <v>45728</v>
       </c>
       <c r="F4" s="146">
-        <f t="shared" ref="F4:F5" si="0">E4-B4</f>
+        <f t="shared" ref="F4" si="0">E4-B4</f>
         <v>343</v>
       </c>
       <c r="G4" s="147">
@@ -2029,47 +2020,22 @@
       <c r="I4" s="176"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B5" s="145">
-        <v>45388</v>
-      </c>
-      <c r="C5" s="181">
-        <v>5</v>
-      </c>
-      <c r="D5" s="146">
-        <v>4600</v>
-      </c>
-      <c r="E5" s="145">
-        <v>45728</v>
-      </c>
-      <c r="F5" s="146">
-        <f t="shared" si="0"/>
-        <v>340</v>
-      </c>
-      <c r="G5" s="147">
-        <f>(D5/C5)*(F5/365)</f>
-        <v>856.98630136986299</v>
+      <c r="A5" s="144"/>
+      <c r="B5" s="144"/>
+      <c r="C5" s="144"/>
+      <c r="D5" s="148">
+        <f>SUM(D4:D4)</f>
+        <v>153700</v>
+      </c>
+      <c r="E5" s="144"/>
+      <c r="F5" s="144"/>
+      <c r="G5" s="148">
+        <f>SUM(G4:G4)</f>
+        <v>28887.178082191782</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="144"/>
-      <c r="B6" s="144"/>
-      <c r="C6" s="144"/>
-      <c r="D6" s="148">
-        <f>SUM(D4:D5)</f>
-        <v>158300</v>
-      </c>
-      <c r="E6" s="144"/>
-      <c r="F6" s="144"/>
-      <c r="G6" s="148">
-        <f>SUM(G4:G5)</f>
-        <v>29744.164383561645</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D8" s="176"/>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D7" s="176"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2331,29 +2297,29 @@
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="118" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C20" s="58"/>
       <c r="D20" s="58"/>
       <c r="H20" s="38"/>
       <c r="I20" s="17"/>
-      <c r="J20" s="139">
+      <c r="J20" s="139" t="e">
         <f>TB!C19</f>
-        <v>4200</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="118" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C21" s="58"/>
       <c r="D21" s="58"/>
       <c r="H21" s="38"/>
       <c r="I21" s="17"/>
-      <c r="J21" s="139">
+      <c r="J21" s="139" t="e">
         <f>TB!C20</f>
-        <v>630</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -2388,9 +2354,9 @@
       <c r="A24" s="57"/>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
-      <c r="J24" s="137">
+      <c r="J24" s="137" t="e">
         <f>SUM(J20:J23)</f>
-        <v>44830</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -2698,7 +2664,7 @@
       </c>
       <c r="E17" s="104"/>
       <c r="H17" s="140" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
@@ -2902,9 +2868,9 @@
         <f>+'P10'!B7</f>
         <v>Office Equipment</v>
       </c>
-      <c r="B36" s="189">
+      <c r="B36" s="189" t="e">
         <f>+'P10'!G7</f>
-        <v>4600</v>
+        <v>#REF!</v>
       </c>
       <c r="C36" s="65">
         <v>5</v>
@@ -2912,18 +2878,18 @@
       <c r="D36" s="227">
         <v>0</v>
       </c>
-      <c r="E36" s="225">
+      <c r="E36" s="225" t="e">
         <f t="shared" ref="E36:E40" si="0">B36/C36</f>
-        <v>920</v>
-      </c>
-      <c r="F36" s="225">
+        <v>#REF!</v>
+      </c>
+      <c r="F36" s="225" t="e">
         <f t="shared" ref="F36:F40" si="1">D36+E36</f>
-        <v>920</v>
+        <v>#REF!</v>
       </c>
       <c r="G36" s="114"/>
-      <c r="H36" s="229">
+      <c r="H36" s="229" t="e">
         <f t="shared" ref="H36:H40" si="2">B36-F36</f>
-        <v>3680</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
@@ -3091,12 +3057,12 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="212" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="207" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="H46" s="186">
         <v>0</v>
@@ -3104,7 +3070,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="207" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="H47" s="235" t="e">
         <f>-H15</f>
@@ -3123,12 +3089,12 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="207" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="207" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="H51" s="186">
         <v>0</v>
@@ -3136,7 +3102,7 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="207" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="H52" s="186">
         <v>0</v>
@@ -3144,7 +3110,7 @@
     </row>
     <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="207" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="H53" s="236" t="e">
         <f>SUM(H48:H52)</f>
@@ -3161,7 +3127,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2A291A8-AC8E-4BB6-A21B-06A29BC55837}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A2:D34"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.6640625" bestFit="1" customWidth="1"/>
@@ -3169,7 +3135,12 @@
     <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="239" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>111</v>
       </c>
@@ -3177,314 +3148,104 @@
         <v>2328236</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B3" s="175"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>158</v>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="239" t="s">
+        <v>198</v>
       </c>
       <c r="B4" s="175"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B5" s="180">
         <v>99975</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>160</v>
-      </c>
-      <c r="B6" s="175">
-        <v>163480</v>
-      </c>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="175"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>161</v>
-      </c>
-      <c r="B7" s="180">
-        <v>11000</v>
-      </c>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="175"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>141</v>
-      </c>
-      <c r="B8" s="180">
-        <v>900750</v>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="239" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>163</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>162</v>
-      </c>
-      <c r="B9" s="175">
-        <v>16522</v>
-      </c>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B9" s="175"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>163</v>
-      </c>
-      <c r="B10" s="180">
-        <v>171150</v>
-      </c>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B10" s="175"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>164</v>
-      </c>
-      <c r="B11" s="180">
-        <v>71672.5</v>
-      </c>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="239" t="s">
+        <v>199</v>
+      </c>
+      <c r="B11" s="175"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>102</v>
-      </c>
-      <c r="B12" s="180">
-        <v>13070</v>
+        <v>167</v>
+      </c>
+      <c r="B12" t="s">
+        <v>168</v>
+      </c>
+      <c r="C12" t="s">
+        <v>169</v>
+      </c>
+      <c r="D12" t="s">
+        <v>170</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>165</v>
-      </c>
-      <c r="B13" s="180">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="177">
         <v>45597</v>
       </c>
+      <c r="B13" s="175">
+        <v>4200</v>
+      </c>
+      <c r="C13" s="175">
+        <f>B13*12/20</f>
+        <v>2520</v>
+      </c>
+      <c r="D13" s="175">
+        <f>C13*3/12</f>
+        <v>630</v>
+      </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>166</v>
-      </c>
-      <c r="B14" s="180">
-        <v>60000</v>
+        <v>28</v>
+      </c>
+      <c r="B14" s="178">
+        <f>SUM(B13:B13)</f>
+        <v>4200</v>
+      </c>
+      <c r="C14" s="179">
+        <f>SUM(C13:C13)</f>
+        <v>2520</v>
+      </c>
+      <c r="D14" s="179">
+        <f>SUM(D13:D13)</f>
+        <v>630</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>167</v>
-      </c>
-      <c r="B15" s="180">
-        <v>10500</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>168</v>
-      </c>
-      <c r="B16" s="180">
-        <v>94812</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="175"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="175"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C19" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="str">
-        <f>+PPE!A4</f>
-        <v>Furniture &amp; Fittings</v>
-      </c>
-      <c r="B20" s="175">
-        <f>+PPE!D4</f>
-        <v>153700</v>
-      </c>
-      <c r="C20">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="str">
-        <f>+PPE!A5</f>
-        <v>Office Equipment</v>
-      </c>
-      <c r="B21" s="175">
-        <f>+PPE!D5</f>
-        <v>4600</v>
-      </c>
-      <c r="C21">
-        <v>1019</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>172</v>
-      </c>
-      <c r="B22" s="175">
-        <v>35000</v>
-      </c>
-      <c r="C22">
-        <v>1039</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>116</v>
-      </c>
-      <c r="B23" s="175">
-        <v>82500</v>
-      </c>
-      <c r="C23">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>173</v>
-      </c>
-      <c r="B24" s="175">
-        <v>36340</v>
-      </c>
-      <c r="C24">
-        <v>1020</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>174</v>
-      </c>
-      <c r="B25" s="175">
-        <f>3990+16500+3200</f>
-        <v>23690</v>
-      </c>
-      <c r="C25">
-        <v>1039</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B26" s="175"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>175</v>
-      </c>
-      <c r="B27" t="s">
-        <v>176</v>
-      </c>
-      <c r="C27" t="s">
-        <v>177</v>
-      </c>
-      <c r="D27" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="177">
-        <v>45597</v>
-      </c>
-      <c r="B28" s="175">
-        <v>4200</v>
-      </c>
-      <c r="C28" s="175">
-        <f>B28*12/20</f>
-        <v>2520</v>
-      </c>
-      <c r="D28" s="175">
-        <f>C28*3/12</f>
-        <v>630</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="177">
-        <v>45627</v>
-      </c>
-      <c r="B29" s="175">
-        <v>4200</v>
-      </c>
-      <c r="C29" s="175">
-        <f>B29*12/20</f>
-        <v>2520</v>
-      </c>
-      <c r="D29" s="175">
-        <f>C29*3/12</f>
-        <v>630</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="177">
-        <v>45658</v>
-      </c>
-      <c r="B30" s="175">
-        <v>4200</v>
-      </c>
-      <c r="C30" s="175">
-        <f>B30*12/20</f>
-        <v>2520</v>
-      </c>
-      <c r="D30" s="175">
-        <f>C30*3/12</f>
-        <v>630</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="177">
-        <v>45689</v>
-      </c>
-      <c r="B31" s="175">
-        <v>4200</v>
-      </c>
-      <c r="C31" s="175">
-        <f>B31*12/20</f>
-        <v>2520</v>
-      </c>
-      <c r="D31" s="175">
-        <f>C31*3/12</f>
-        <v>630</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="177">
-        <v>45717</v>
-      </c>
-      <c r="B32" s="180">
-        <v>4200</v>
-      </c>
-      <c r="C32" s="175">
-        <f>B32*12/20</f>
-        <v>2520</v>
-      </c>
-      <c r="D32" s="180">
-        <f>C32*3/12</f>
-        <v>630</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>28</v>
-      </c>
-      <c r="B33" s="178">
-        <f>SUM(B28:B32)</f>
-        <v>21000</v>
-      </c>
-      <c r="C33" s="179">
-        <f>SUM(C28:C32)</f>
-        <v>12600</v>
-      </c>
-      <c r="D33" s="179">
-        <f>SUM(D28:D32)</f>
-        <v>3150</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="175"/>
-      <c r="C34" s="175"/>
-      <c r="D34" s="175"/>
+    <row r="15" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="175"/>
+      <c r="C15" s="175"/>
+      <c r="D15" s="175"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3504,25 +3265,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="239" t="s">
+      <c r="A1" s="240" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="239"/>
-      <c r="C1" s="239"/>
+      <c r="B1" s="240"/>
+      <c r="C1" s="240"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="240" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="239"/>
-      <c r="C2" s="239"/>
+      <c r="B2" s="240"/>
+      <c r="C2" s="240"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="239" t="s">
+      <c r="A3" s="240" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="239"/>
-      <c r="C3" s="239"/>
+      <c r="B3" s="240"/>
+      <c r="C3" s="240"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="167"/>
@@ -3575,18 +3336,18 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="170" t="s">
-        <v>170</v>
-      </c>
-      <c r="B10" s="182">
-        <f>+PPE!D5</f>
-        <v>4600</v>
+        <v>162</v>
+      </c>
+      <c r="B10" s="182" t="e">
+        <f>+PPE!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C10" s="89"/>
       <c r="J10" s="171"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="170" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B11" s="182" t="e">
         <f>+PPE!#REF!</f>
@@ -3606,7 +3367,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="170" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="B13" s="182" t="e">
         <f>+PPE!#REF!</f>
@@ -3616,7 +3377,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="170" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="B14" s="182" t="e">
         <f>+PPE!#REF!</f>
@@ -3630,8 +3391,8 @@
       </c>
       <c r="B15" s="89"/>
       <c r="C15" s="182">
-        <f>+PPE!G6</f>
-        <v>29744.164383561645</v>
+        <f>+PPE!G5</f>
+        <v>28887.178082191782</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -3661,26 +3422,26 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="170" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="B19" s="89"/>
-      <c r="C19" s="182">
-        <f>Working!B32</f>
-        <v>4200</v>
+      <c r="C19" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="170" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="B20" s="89"/>
-      <c r="C20" s="182">
-        <f>Working!D32</f>
-        <v>630</v>
-      </c>
-      <c r="E20" s="174">
+      <c r="C20" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="E20" s="174" t="e">
         <f>C20*20/3</f>
-        <v>4200</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -3699,7 +3460,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="170" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="B23" s="89"/>
       <c r="C23" s="214">
@@ -3718,7 +3479,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="173" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B26" s="193">
         <v>112919.5</v>
@@ -3727,7 +3488,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="170" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="B27" s="89"/>
       <c r="C27" s="183">
@@ -3746,15 +3507,15 @@
       <c r="A29" s="170" t="s">
         <v>141</v>
       </c>
-      <c r="B29" s="182">
-        <f>Working!B8</f>
-        <v>900750</v>
+      <c r="B29" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C29" s="89"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="170" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="B30" s="182">
         <v>1220000</v>
@@ -3763,7 +3524,7 @@
     </row>
     <row r="31" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B31" s="182">
         <f>Working!B5</f>
@@ -3773,11 +3534,11 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="B32" s="182">
-        <f>Working!B7</f>
-        <v>11000</v>
+        <v>174</v>
+      </c>
+      <c r="B32" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C32" s="89"/>
     </row>
@@ -3785,39 +3546,39 @@
       <c r="A33" s="170" t="s">
         <v>113</v>
       </c>
-      <c r="B33" s="182">
-        <f>Working!B10</f>
-        <v>171150</v>
+      <c r="B33" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C33" s="89"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="170" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="B34" s="182">
-        <f>+Working!C33</f>
-        <v>12600</v>
+        <f>+Working!C14</f>
+        <v>2520</v>
       </c>
       <c r="C34" s="89"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="170" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="B35" s="182">
-        <f>Working!D33</f>
-        <v>3150</v>
+        <f>Working!D14</f>
+        <v>630</v>
       </c>
       <c r="C35" s="89"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="170" t="s">
-        <v>183</v>
-      </c>
-      <c r="B36" s="182">
-        <f>Working!B11</f>
-        <v>71672.5</v>
+        <v>175</v>
+      </c>
+      <c r="B36" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C36" s="89"/>
     </row>
@@ -3825,9 +3586,9 @@
       <c r="A37" s="170" t="s">
         <v>101</v>
       </c>
-      <c r="B37" s="182">
-        <f>Working!B14</f>
-        <v>60000</v>
+      <c r="B37" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C37" s="89"/>
     </row>
@@ -3835,9 +3596,9 @@
       <c r="A38" s="170" t="s">
         <v>102</v>
       </c>
-      <c r="B38" s="182">
-        <f>Working!B12</f>
-        <v>13070</v>
+      <c r="B38" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C38" s="89"/>
     </row>
@@ -3845,9 +3606,9 @@
       <c r="A39" s="170" t="s">
         <v>110</v>
       </c>
-      <c r="B39" s="182">
-        <f>Working!B13</f>
-        <v>45597</v>
+      <c r="B39" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C39" s="89"/>
     </row>
@@ -3860,7 +3621,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="170" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B41" s="214">
         <v>163480</v>
@@ -3869,11 +3630,11 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="170" t="s">
-        <v>167</v>
-      </c>
-      <c r="B42" s="182">
-        <f>+Working!B15</f>
-        <v>10500</v>
+        <v>160</v>
+      </c>
+      <c r="B42" s="182" t="e">
+        <f>+Working!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C42" s="89"/>
     </row>
@@ -3888,9 +3649,9 @@
       <c r="A44" s="170" t="s">
         <v>100</v>
       </c>
-      <c r="B44" s="182">
-        <f>Working!B16</f>
-        <v>94812</v>
+      <c r="B44" s="182" t="e">
+        <f>Working!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C44" s="89"/>
     </row>
@@ -3935,9 +3696,9 @@
         <f>SUM(B5:B48)</f>
         <v>#REF!</v>
       </c>
-      <c r="C49" s="90">
+      <c r="C49" s="90" t="e">
         <f>SUM(C5:C48)</f>
-        <v>3408810.1643835614</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="14.4" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -4100,7 +3861,7 @@
     </row>
     <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="12" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="D16" s="128" t="e">
         <f>SUM(D12:D14)</f>
@@ -5247,7 +5008,7 @@
     </row>
     <row r="12" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A12" s="155" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B12" s="155"/>
       <c r="C12" s="237"/>
@@ -19308,9 +19069,9 @@
         <v>11</v>
       </c>
       <c r="D26" s="3"/>
-      <c r="E26" s="73">
+      <c r="E26" s="73" t="e">
         <f>+'P11'!J24</f>
-        <v>44830</v>
+        <v>#REF!</v>
       </c>
       <c r="F26" s="156"/>
       <c r="J26" s="13"/>
@@ -21317,9 +21078,9 @@
       <c r="A28" s="161" t="s">
         <v>42</v>
       </c>
-      <c r="E28" s="130">
+      <c r="E28" s="130" t="e">
         <f>SUM(E26:E27)</f>
-        <v>1044830</v>
+        <v>#REF!</v>
       </c>
       <c r="F28" s="156"/>
       <c r="J28" s="13"/>
@@ -22321,9 +22082,9 @@
       <c r="A29" s="161" t="s">
         <v>43</v>
       </c>
-      <c r="E29" s="132">
+      <c r="E29" s="132" t="e">
         <f>E28+E23</f>
-        <v>1044830</v>
+        <v>#REF!</v>
       </c>
       <c r="F29" s="156"/>
       <c r="J29" s="13"/>
@@ -41525,7 +41286,7 @@
     </row>
     <row r="50" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A50" s="28" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="B50" s="18"/>
       <c r="C50" s="18"/>
@@ -42532,7 +42293,7 @@
     </row>
     <row r="51" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A51" s="28" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="B51" s="18"/>
       <c r="C51" s="18"/>
@@ -43688,7 +43449,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="E11" s="62">
         <v>0</v>
@@ -43901,7 +43662,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B12" s="195" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="C12" s="195"/>
       <c r="D12" s="195"/>
@@ -43913,14 +43674,14 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B13" s="195" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="C13" s="195"/>
       <c r="D13" s="195"/>
       <c r="F13" s="199"/>
-      <c r="G13" s="221">
+      <c r="G13" s="221" t="e">
         <f>BS!E26</f>
-        <v>44830</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -44184,7 +43945,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
@@ -44274,7 +44035,7 @@
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
       <c r="B11" s="2" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="73">
@@ -44291,9 +44052,9 @@
         <v>141</v>
       </c>
       <c r="C12" s="76"/>
-      <c r="D12" s="124">
+      <c r="D12" s="124" t="e">
         <f>TB!B29</f>
-        <v>900750</v>
+        <v>#REF!</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="38"/>
@@ -44302,12 +44063,12 @@
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
       <c r="B13" s="2" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C13" s="76"/>
       <c r="D13" s="124">
         <f>TB!B34</f>
-        <v>12600</v>
+        <v>2520</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="38"/>
@@ -44316,12 +44077,12 @@
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C14" s="76"/>
       <c r="D14" s="124">
         <f>TB!B35</f>
-        <v>3150</v>
+        <v>630</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="38"/>
@@ -44333,9 +44094,9 @@
         <v>153</v>
       </c>
       <c r="C15" s="76"/>
-      <c r="D15" s="124">
+      <c r="D15" s="124" t="e">
         <f>+TB!B37</f>
-        <v>60000</v>
+        <v>#REF!</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="38"/>
@@ -44344,12 +44105,12 @@
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="C16" s="76"/>
-      <c r="D16" s="124">
+      <c r="D16" s="124" t="e">
         <f>+TB!B31+TB!B32</f>
-        <v>110975</v>
+        <v>#REF!</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="38"/>
@@ -44361,9 +44122,9 @@
         <v>110</v>
       </c>
       <c r="C17" s="76"/>
-      <c r="D17" s="124">
+      <c r="D17" s="124" t="e">
         <f>TB!B39</f>
-        <v>45597</v>
+        <v>#REF!</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="38"/>
@@ -44375,9 +44136,9 @@
         <v>142</v>
       </c>
       <c r="C18" s="76"/>
-      <c r="D18" s="124">
+      <c r="D18" s="124" t="e">
         <f>TB!B38</f>
-        <v>13070</v>
+        <v>#REF!</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="38"/>
@@ -44389,9 +44150,9 @@
         <v>143</v>
       </c>
       <c r="C19" s="76"/>
-      <c r="D19" s="124">
+      <c r="D19" s="124" t="e">
         <f>TB!B33</f>
-        <v>171150</v>
+        <v>#REF!</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="38"/>
@@ -44400,12 +44161,12 @@
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C20" s="76"/>
-      <c r="D20" s="124">
+      <c r="D20" s="124" t="e">
         <f>TB!B42</f>
-        <v>10500</v>
+        <v>#REF!</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="38"/>
@@ -44414,12 +44175,12 @@
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="C21" s="76"/>
-      <c r="D21" s="124">
+      <c r="D21" s="124" t="e">
         <f>TB!B36</f>
-        <v>71672.5</v>
+        <v>#REF!</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="38"/>
@@ -44445,9 +44206,9 @@
         <v>100</v>
       </c>
       <c r="C23" s="76"/>
-      <c r="D23" s="124">
+      <c r="D23" s="124" t="e">
         <f>TB!B44</f>
-        <v>94812</v>
+        <v>#REF!</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="38"/>
@@ -44509,7 +44270,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B29" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="125">
@@ -44690,15 +44451,15 @@
         <v>0</v>
       </c>
       <c r="F7" s="135"/>
-      <c r="G7" s="135">
+      <c r="G7" s="135" t="e">
         <f>TB!B10</f>
-        <v>4600</v>
+        <v>#REF!</v>
       </c>
       <c r="H7" s="122"/>
       <c r="I7" s="123"/>
-      <c r="J7" s="122">
+      <c r="J7" s="122" t="e">
         <f t="shared" ref="J7:J11" si="0">SUM(E7:G7)</f>
-        <v>4600</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
@@ -44896,15 +44657,15 @@
         <v>0</v>
       </c>
       <c r="F17" s="135"/>
-      <c r="G17" s="122">
-        <f>PPE!G5</f>
-        <v>856.98630136986299</v>
+      <c r="G17" s="122" t="e">
+        <f>PPE!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="H17" s="122"/>
       <c r="I17" s="123"/>
-      <c r="J17" s="149">
+      <c r="J17" s="149" t="e">
         <f t="shared" ref="J17:J21" si="2">SUM(E17:G17)</f>
-        <v>856.98630136986299</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -45058,9 +44819,9 @@
         <f t="shared" si="3"/>
         <v>Office Equipment</v>
       </c>
-      <c r="J26" s="74">
+      <c r="J26" s="74" t="e">
         <f t="shared" si="4"/>
-        <v>3743.0136986301368</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
feat: enhance financial reporting by adding TRIALBALANCE DTO and updating account types
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F11B7C-4E3E-4FA2-A322-DBD248476C6B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B53AE7-D416-4887-994D-BE21CF413D5F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPE" sheetId="24" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="191">
   <si>
     <t>STATEMENT OF FINANCIAL POSITION</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t>Cr</t>
-  </si>
-  <si>
-    <t>ADMINSTRATION EXPENSES</t>
   </si>
   <si>
     <t>Assets</t>
@@ -377,15 +374,6 @@
     <t>Printing &amp; Stationery</t>
   </si>
   <si>
-    <t>Incorporation Fees</t>
-  </si>
-  <si>
-    <t>Electricity</t>
-  </si>
-  <si>
-    <t>Travelling Charges</t>
-  </si>
-  <si>
     <t>Audit Fee</t>
   </si>
   <si>
@@ -411,12 +399,6 @@
   </si>
   <si>
     <t>As at 31st March 2025</t>
-  </si>
-  <si>
-    <t>Rent Expenses</t>
-  </si>
-  <si>
-    <t>Fuel Expenses</t>
   </si>
   <si>
     <t>Amount</t>
@@ -561,19 +543,7 @@
     <t>Income</t>
   </si>
   <si>
-    <t>Office Equipment</t>
-  </si>
-  <si>
     <t>Bill Nu.</t>
-  </si>
-  <si>
-    <t>Computer &amp; Printers</t>
-  </si>
-  <si>
-    <t>Telephone</t>
-  </si>
-  <si>
-    <t>CCTV Camera</t>
   </si>
   <si>
     <t>EPF &amp; ETF</t>
@@ -595,12 +565,6 @@
   </si>
   <si>
     <t>Date</t>
-  </si>
-  <si>
-    <t>Sales Commission</t>
-  </si>
-  <si>
-    <t>Repair &amp; Maintance</t>
   </si>
   <si>
     <t xml:space="preserve">Business Promotion &amp; Marketing Expneses </t>
@@ -674,6 +638,15 @@
   <si>
     <t>EPF ETF</t>
   </si>
+  <si>
+    <t>Liabilities</t>
+  </si>
+  <si>
+    <t>Equity</t>
+  </si>
+  <si>
+    <t>Expenses</t>
+  </si>
 </sst>
 </file>
 
@@ -685,7 +658,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -804,27 +777,8 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -836,11 +790,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -849,6 +798,27 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -964,9 +934,9 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="241">
+  <cellXfs count="237">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1147,16 +1117,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1179,7 +1140,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1206,9 +1167,6 @@
     </xf>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="20" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1255,9 +1213,6 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1319,27 +1274,12 @@
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="43" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1350,13 +1290,6 @@
     <xf numFmtId="43" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="6" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="20" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="23" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -1370,7 +1303,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="43" fontId="19" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="43" fontId="12" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1408,12 +1340,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1423,9 +1349,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="20" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="43" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1447,10 +1370,7 @@
     <xf numFmtId="43" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1462,10 +1382,46 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="23">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1511,7 +1467,7 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="184731" cy="264560"/>
@@ -1966,76 +1922,76 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="37" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C1" s="37"/>
     </row>
     <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="142" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="143" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="142" t="s">
-        <v>125</v>
-      </c>
-      <c r="D3" s="144" t="s">
+      <c r="A3" s="137" t="s">
         <v>115</v>
       </c>
-      <c r="E3" s="143" t="s">
-        <v>123</v>
-      </c>
-      <c r="F3" s="143" t="s">
-        <v>173</v>
-      </c>
-      <c r="G3" s="143" t="s">
-        <v>124</v>
+      <c r="B3" s="138" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" s="137" t="s">
+        <v>119</v>
+      </c>
+      <c r="D3" s="139" t="s">
+        <v>109</v>
+      </c>
+      <c r="E3" s="138" t="s">
+        <v>117</v>
+      </c>
+      <c r="F3" s="138" t="s">
+        <v>163</v>
+      </c>
+      <c r="G3" s="138" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B4" s="145">
+        <v>110</v>
+      </c>
+      <c r="B4" s="140">
         <v>45385</v>
       </c>
-      <c r="C4" s="181">
+      <c r="C4" s="171">
         <v>5</v>
       </c>
-      <c r="D4" s="146">
+      <c r="D4" s="141">
         <v>153700</v>
       </c>
-      <c r="E4" s="145">
+      <c r="E4" s="140">
         <v>45728</v>
       </c>
-      <c r="F4" s="146">
+      <c r="F4" s="141">
         <f t="shared" ref="F4" si="0">E4-B4</f>
         <v>343</v>
       </c>
-      <c r="G4" s="147">
+      <c r="G4" s="142">
         <f>(D4/C4)*(F4/365)</f>
         <v>28887.178082191782</v>
       </c>
-      <c r="I4" s="176"/>
+      <c r="I4" s="166"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="144"/>
-      <c r="B5" s="144"/>
-      <c r="C5" s="144"/>
-      <c r="D5" s="148">
+      <c r="A5" s="139"/>
+      <c r="B5" s="139"/>
+      <c r="C5" s="139"/>
+      <c r="D5" s="143">
         <f>SUM(D4:D4)</f>
         <v>153700</v>
       </c>
-      <c r="E5" s="144"/>
-      <c r="F5" s="144"/>
-      <c r="G5" s="148">
+      <c r="E5" s="139"/>
+      <c r="F5" s="139"/>
+      <c r="G5" s="143">
         <f>SUM(G4:G4)</f>
         <v>28887.178082191782</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D7" s="176"/>
+      <c r="D7" s="166"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2064,7 +2020,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2074,13 +2030,13 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="165" t="s">
-        <v>108</v>
+      <c r="J1" s="160" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="79" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" s="79"/>
       <c r="C2" s="79"/>
@@ -2093,8 +2049,8 @@
       <c r="J2" s="79"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="94" t="s">
-        <v>80</v>
+      <c r="A3" s="91" t="s">
+        <v>79</v>
       </c>
       <c r="B3" s="80"/>
       <c r="C3" s="80"/>
@@ -2145,13 +2101,13 @@
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="56" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="C7" s="56"/>
       <c r="D7" s="56"/>
       <c r="H7" s="51"/>
       <c r="I7" s="51"/>
-      <c r="J7" s="122">
+      <c r="J7" s="118">
         <f>+TB!B6</f>
         <v>12560</v>
       </c>
@@ -2163,7 +2119,7 @@
       <c r="D8" s="53"/>
       <c r="H8" s="52"/>
       <c r="I8" s="46"/>
-      <c r="J8" s="137">
+      <c r="J8" s="133">
         <f>SUM(J7:J7)</f>
         <v>12560</v>
       </c>
@@ -2198,13 +2154,13 @@
       <c r="H11" s="17"/>
       <c r="I11" s="17"/>
       <c r="J11" s="86" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="57"/>
       <c r="B12" s="53" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C12" s="53"/>
       <c r="D12" s="53"/>
@@ -2249,14 +2205,14 @@
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="57"/>
       <c r="B16" s="53" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C16" s="53"/>
       <c r="D16" s="53"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
-      <c r="J16" s="138">
-        <f>+TB!C22</f>
+      <c r="J16" s="134">
+        <f>+TB!C14</f>
         <v>6000</v>
       </c>
     </row>
@@ -2267,7 +2223,7 @@
       <c r="D17" s="53"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
-      <c r="J17" s="137">
+      <c r="J17" s="133">
         <f>SUM(J16)</f>
         <v>6000</v>
       </c>
@@ -2286,7 +2242,7 @@
         <v>11</v>
       </c>
       <c r="B19" s="58" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C19" s="58"/>
       <c r="D19" s="58"/>
@@ -2296,57 +2252,57 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
-      <c r="B20" s="118" t="s">
-        <v>171</v>
+      <c r="B20" s="114" t="s">
+        <v>161</v>
       </c>
       <c r="C20" s="58"/>
       <c r="D20" s="58"/>
       <c r="H20" s="38"/>
       <c r="I20" s="17"/>
-      <c r="J20" s="139" t="e">
-        <f>TB!C19</f>
+      <c r="J20" s="135" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
-      <c r="B21" s="118" t="s">
-        <v>172</v>
+      <c r="B21" s="114" t="s">
+        <v>162</v>
       </c>
       <c r="C21" s="58"/>
       <c r="D21" s="58"/>
       <c r="H21" s="38"/>
       <c r="I21" s="17"/>
-      <c r="J21" s="139" t="e">
-        <f>TB!C20</f>
+      <c r="J21" s="135" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
-      <c r="B22" s="118" t="s">
-        <v>145</v>
+      <c r="B22" s="114" t="s">
+        <v>139</v>
       </c>
       <c r="C22" s="58"/>
       <c r="D22" s="58"/>
       <c r="H22" s="38"/>
       <c r="I22" s="17"/>
-      <c r="J22" s="139">
-        <f>+TB!C17</f>
+      <c r="J22" s="135">
+        <f>+TB!C11</f>
         <v>15000</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
-      <c r="B23" s="118" t="s">
-        <v>104</v>
+      <c r="B23" s="114" t="s">
+        <v>100</v>
       </c>
       <c r="C23" s="58"/>
       <c r="D23" s="58"/>
       <c r="H23" s="38"/>
       <c r="I23" s="17"/>
-      <c r="J23" s="139">
-        <f>+TB!C18</f>
+      <c r="J23" s="135">
+        <f>+TB!C12</f>
         <v>25000</v>
       </c>
     </row>
@@ -2354,7 +2310,7 @@
       <c r="A24" s="57"/>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
-      <c r="J24" s="137" t="e">
+      <c r="J24" s="133" t="e">
         <f>SUM(J20:J23)</f>
         <v>#REF!</v>
       </c>
@@ -2529,44 +2485,44 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B1" s="30"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="97"/>
-      <c r="H1" s="165" t="s">
-        <v>82</v>
+      <c r="F1" s="93"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="160" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B2" s="30"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="30" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B3" s="30"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="30" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="98"/>
-      <c r="B5" s="98"/>
-      <c r="D5" s="99"/>
-      <c r="E5" s="99"/>
-      <c r="H5" s="99" t="s">
+      <c r="A5" s="95"/>
+      <c r="B5" s="95"/>
+      <c r="D5" s="96"/>
+      <c r="E5" s="96"/>
+      <c r="H5" s="96" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="63" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E6" s="21"/>
       <c r="H6" s="21" t="e">
@@ -2575,16 +2531,16 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="100"/>
+      <c r="A7" s="97"/>
       <c r="E7" s="21"/>
       <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="64" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E8" s="21"/>
-      <c r="H8" s="101">
+      <c r="H8" s="98">
         <v>0</v>
       </c>
     </row>
@@ -2597,7 +2553,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="30" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B10" s="30"/>
       <c r="E10" s="21"/>
@@ -2605,14 +2561,14 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="D11" s="102"/>
-      <c r="F11" s="216" t="e">
+        <v>129</v>
+      </c>
+      <c r="D11" s="99"/>
+      <c r="F11" s="200" t="e">
         <f>'P10'!G22</f>
         <v>#REF!</v>
       </c>
-      <c r="H11" s="232" t="e">
+      <c r="H11" s="214" t="e">
         <f>+F11</f>
         <v>#REF!</v>
       </c>
@@ -2626,7 +2582,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="30" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B13" s="30"/>
       <c r="E13" s="21"/>
@@ -2634,131 +2590,131 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F14" s="65" t="s">
-        <v>146</v>
-      </c>
-      <c r="H14" s="101" t="e">
+        <v>140</v>
+      </c>
+      <c r="H14" s="98" t="e">
         <f>-E42</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E15" s="21"/>
-      <c r="H15" s="103" t="e">
+      <c r="H15" s="100" t="e">
         <f>SUM(H12:H14)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="E16" s="104"/>
-      <c r="H16" s="104"/>
+      <c r="E16" s="101"/>
+      <c r="H16" s="101"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="E17" s="104"/>
-      <c r="H17" s="140" t="s">
-        <v>186</v>
+        <v>88</v>
+      </c>
+      <c r="E17" s="101"/>
+      <c r="H17" s="136" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="E18" s="104"/>
-      <c r="H18" s="104"/>
+      <c r="E18" s="101"/>
+      <c r="H18" s="101"/>
     </row>
     <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="105" t="s">
+      <c r="A19" s="102" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="103" t="s">
         <v>90</v>
-      </c>
-      <c r="E19" s="106" t="s">
-        <v>91</v>
       </c>
       <c r="F19" s="32" t="str">
         <f>+H17</f>
         <v>Loss</v>
       </c>
-      <c r="H19" s="104" t="e">
+      <c r="H19" s="101" t="e">
         <f>F19*0.3</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
-      <c r="E20" s="104"/>
-      <c r="H20" s="104"/>
+      <c r="E20" s="101"/>
+      <c r="H20" s="101"/>
     </row>
     <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="107" t="s">
-        <v>92</v>
-      </c>
-      <c r="E21" s="104"/>
-      <c r="H21" s="104"/>
+      <c r="A21" s="104" t="s">
+        <v>91</v>
+      </c>
+      <c r="E21" s="101"/>
+      <c r="H21" s="101"/>
     </row>
     <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="13" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="E22" s="65">
         <v>24252</v>
       </c>
-      <c r="F22" s="109">
+      <c r="F22" s="106">
         <v>0</v>
       </c>
-      <c r="G22" s="108"/>
-      <c r="H22" s="109">
+      <c r="G22" s="105"/>
+      <c r="H22" s="106">
         <f>-SUM(F22:F22)</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="3.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D23" s="65"/>
-      <c r="E23" s="104"/>
-      <c r="F23" s="104"/>
-      <c r="G23" s="108"/>
-      <c r="H23" s="104"/>
+      <c r="E23" s="101"/>
+      <c r="F23" s="101"/>
+      <c r="G23" s="105"/>
+      <c r="H23" s="101"/>
     </row>
     <row r="24" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="E24" s="104"/>
-      <c r="H24" s="110" t="e">
+        <v>92</v>
+      </c>
+      <c r="E24" s="101"/>
+      <c r="H24" s="107" t="e">
         <f>SUM(H19:H22)</f>
         <v>#VALUE!</v>
       </c>
       <c r="K24" s="29"/>
     </row>
     <row r="25" spans="1:11" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="E25" s="104"/>
-      <c r="H25" s="104"/>
+      <c r="E25" s="101"/>
+      <c r="H25" s="101"/>
     </row>
     <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
-      <c r="E26" s="104"/>
-      <c r="H26" s="104"/>
+      <c r="E26" s="101"/>
+      <c r="H26" s="101"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="63" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B27" s="18"/>
       <c r="C27" s="18"/>
       <c r="D27" s="18"/>
-      <c r="E27" s="104"/>
+      <c r="E27" s="101"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
       <c r="H27" s="18"/>
     </row>
     <row r="28" spans="1:11" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E28" s="104"/>
-      <c r="H28" s="104"/>
+      <c r="E28" s="101"/>
+      <c r="H28" s="101"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="87" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -2779,340 +2735,340 @@
       <c r="H30" s="18"/>
     </row>
     <row r="31" spans="1:11" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="111" t="s">
+      <c r="A31" s="108" t="s">
+        <v>95</v>
+      </c>
+      <c r="B31" s="109" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="96" t="s">
         <v>96</v>
       </c>
-      <c r="B31" s="112" t="s">
-        <v>27</v>
-      </c>
-      <c r="C31" s="99" t="s">
+      <c r="D31" s="110" t="s">
+        <v>131</v>
+      </c>
+      <c r="E31" s="90" t="s">
         <v>97</v>
       </c>
-      <c r="D31" s="113" t="s">
-        <v>137</v>
-      </c>
-      <c r="E31" s="93" t="s">
+      <c r="F31" s="90" t="s">
+        <v>132</v>
+      </c>
+      <c r="G31" s="90"/>
+      <c r="H31" s="96" t="s">
         <v>98</v>
-      </c>
-      <c r="F31" s="93" t="s">
-        <v>138</v>
-      </c>
-      <c r="G31" s="93"/>
-      <c r="H31" s="99" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="111"/>
-      <c r="B32" s="112"/>
+      <c r="A32" s="108"/>
+      <c r="B32" s="109"/>
       <c r="C32" s="65"/>
-      <c r="D32" s="114"/>
-      <c r="E32" s="114"/>
-      <c r="F32" s="114"/>
-      <c r="G32" s="114"/>
+      <c r="D32" s="111"/>
+      <c r="E32" s="111"/>
+      <c r="F32" s="111"/>
+      <c r="G32" s="111"/>
       <c r="H32" s="65"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A33" s="111" t="s">
-        <v>139</v>
-      </c>
-      <c r="B33" s="112"/>
+      <c r="A33" s="108" t="s">
+        <v>133</v>
+      </c>
+      <c r="B33" s="109"/>
       <c r="C33" s="65"/>
-      <c r="D33" s="114"/>
-      <c r="E33" s="114"/>
-      <c r="F33" s="114"/>
-      <c r="G33" s="114"/>
+      <c r="D33" s="111"/>
+      <c r="E33" s="111"/>
+      <c r="F33" s="111"/>
+      <c r="G33" s="111"/>
       <c r="H33" s="65"/>
     </row>
     <row r="34" spans="1:8" ht="5.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="111"/>
-      <c r="B34" s="112"/>
+      <c r="A34" s="108"/>
+      <c r="B34" s="109"/>
       <c r="C34" s="65"/>
-      <c r="D34" s="114"/>
-      <c r="E34" s="114"/>
-      <c r="F34" s="114"/>
-      <c r="G34" s="114"/>
+      <c r="D34" s="111"/>
+      <c r="E34" s="111"/>
+      <c r="F34" s="111"/>
+      <c r="G34" s="111"/>
       <c r="H34" s="65"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" s="111" t="str">
+      <c r="A35" s="108" t="str">
         <f>+'P10'!B6</f>
         <v>Furniture &amp; Fittings</v>
       </c>
-      <c r="B35" s="189">
+      <c r="B35" s="176">
         <f>+'P10'!G6</f>
         <v>153700</v>
       </c>
       <c r="C35" s="65">
         <v>5</v>
       </c>
-      <c r="D35" s="152">
+      <c r="D35" s="147">
         <v>0</v>
       </c>
-      <c r="E35" s="151">
+      <c r="E35" s="146">
         <f>B35/C35</f>
         <v>30740</v>
       </c>
-      <c r="F35" s="151">
+      <c r="F35" s="146">
         <f>D35+E35</f>
         <v>30740</v>
       </c>
-      <c r="G35" s="114"/>
-      <c r="H35" s="154">
+      <c r="G35" s="111"/>
+      <c r="H35" s="149">
         <f>B35-F35</f>
         <v>122960</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" s="217" t="str">
+      <c r="A36" s="201" t="e">
         <f>+'P10'!B7</f>
-        <v>Office Equipment</v>
-      </c>
-      <c r="B36" s="189" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="B36" s="176" t="e">
         <f>+'P10'!G7</f>
         <v>#REF!</v>
       </c>
       <c r="C36" s="65">
         <v>5</v>
       </c>
-      <c r="D36" s="227">
+      <c r="D36" s="210">
         <v>0</v>
       </c>
-      <c r="E36" s="225" t="e">
+      <c r="E36" s="208" t="e">
         <f t="shared" ref="E36:E40" si="0">B36/C36</f>
         <v>#REF!</v>
       </c>
-      <c r="F36" s="225" t="e">
+      <c r="F36" s="208" t="e">
         <f t="shared" ref="F36:F40" si="1">D36+E36</f>
         <v>#REF!</v>
       </c>
-      <c r="G36" s="114"/>
-      <c r="H36" s="229" t="e">
+      <c r="G36" s="111"/>
+      <c r="H36" s="212" t="e">
         <f t="shared" ref="H36:H40" si="2">B36-F36</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" s="217" t="str">
+      <c r="A37" s="201" t="e">
         <f>+'P10'!B8</f>
-        <v>Computer &amp; Printers</v>
-      </c>
-      <c r="B37" s="189" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="B37" s="176" t="e">
         <f>+'P10'!G8</f>
         <v>#REF!</v>
       </c>
       <c r="C37" s="65">
         <v>5</v>
       </c>
-      <c r="D37" s="227">
+      <c r="D37" s="210">
         <v>0</v>
       </c>
-      <c r="E37" s="225" t="e">
+      <c r="E37" s="208" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F37" s="225" t="e">
+      <c r="F37" s="208" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G37" s="114"/>
-      <c r="H37" s="229" t="e">
+      <c r="G37" s="111"/>
+      <c r="H37" s="212" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="205" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="217" t="str">
+    <row r="38" spans="1:8" s="191" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="201" t="e">
         <f>+'P10'!B9</f>
-        <v>Furniture &amp; Fittings</v>
-      </c>
-      <c r="B38" s="189" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="B38" s="176" t="e">
         <f>+'P10'!G9</f>
         <v>#REF!</v>
       </c>
-      <c r="C38" s="211">
+      <c r="C38" s="197">
         <v>5</v>
       </c>
-      <c r="D38" s="227">
+      <c r="D38" s="210">
         <v>0</v>
       </c>
-      <c r="E38" s="225" t="e">
+      <c r="E38" s="208" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F38" s="225" t="e">
+      <c r="F38" s="208" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G38" s="218"/>
-      <c r="H38" s="229" t="e">
+      <c r="G38" s="202"/>
+      <c r="H38" s="212" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="39" spans="1:8" s="205" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="217" t="str">
+    <row r="39" spans="1:8" s="191" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="201" t="e">
         <f>+'P10'!B10</f>
-        <v>Telephone</v>
-      </c>
-      <c r="B39" s="189" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="B39" s="176" t="e">
         <f>+'P10'!G10</f>
         <v>#REF!</v>
       </c>
-      <c r="C39" s="211">
+      <c r="C39" s="197">
         <v>5</v>
       </c>
-      <c r="D39" s="227">
+      <c r="D39" s="210">
         <v>0</v>
       </c>
-      <c r="E39" s="225" t="e">
+      <c r="E39" s="208" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F39" s="225" t="e">
+      <c r="F39" s="208" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G39" s="218"/>
-      <c r="H39" s="229" t="e">
+      <c r="G39" s="202"/>
+      <c r="H39" s="212" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="40" spans="1:8" s="205" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="217" t="str">
+    <row r="40" spans="1:8" s="191" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="201" t="e">
         <f>+'P10'!B11</f>
-        <v>CCTV Camera</v>
-      </c>
-      <c r="B40" s="189" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="B40" s="176" t="e">
         <f>+'P10'!G11</f>
         <v>#REF!</v>
       </c>
-      <c r="C40" s="211">
+      <c r="C40" s="197">
         <v>5</v>
       </c>
-      <c r="D40" s="227">
+      <c r="D40" s="210">
         <v>0</v>
       </c>
-      <c r="E40" s="225" t="e">
+      <c r="E40" s="208" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F40" s="225" t="e">
+      <c r="F40" s="208" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G40" s="218"/>
-      <c r="H40" s="229" t="e">
+      <c r="G40" s="202"/>
+      <c r="H40" s="212" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="41" spans="1:8" s="205" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="217"/>
-      <c r="B41" s="226"/>
-      <c r="C41" s="211"/>
-      <c r="D41" s="227"/>
-      <c r="E41" s="225"/>
-      <c r="F41" s="225"/>
-      <c r="G41" s="218"/>
-      <c r="H41" s="229"/>
+    <row r="41" spans="1:8" s="191" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="201"/>
+      <c r="B41" s="209"/>
+      <c r="C41" s="197"/>
+      <c r="D41" s="210"/>
+      <c r="E41" s="208"/>
+      <c r="F41" s="208"/>
+      <c r="G41" s="202"/>
+      <c r="H41" s="212"/>
     </row>
     <row r="42" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="63" t="s">
-        <v>28</v>
-      </c>
-      <c r="B42" s="153" t="e">
+        <v>27</v>
+      </c>
+      <c r="B42" s="148" t="e">
         <f>SUM(B35:B40)</f>
         <v>#REF!</v>
       </c>
-      <c r="C42" s="116"/>
-      <c r="D42" s="228">
+      <c r="C42" s="113"/>
+      <c r="D42" s="211">
         <f>SUM(D35:D40)</f>
         <v>0</v>
       </c>
-      <c r="E42" s="228" t="e">
+      <c r="E42" s="211" t="e">
         <f t="shared" ref="E42:H42" si="3">SUM(E35:E40)</f>
         <v>#REF!</v>
       </c>
-      <c r="F42" s="228" t="e">
+      <c r="F42" s="211" t="e">
         <f t="shared" si="3"/>
         <v>#REF!</v>
       </c>
-      <c r="G42" s="116"/>
-      <c r="H42" s="228" t="e">
+      <c r="G42" s="113"/>
+      <c r="H42" s="211" t="e">
         <f t="shared" si="3"/>
         <v>#REF!</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A43" s="18"/>
-      <c r="B43" s="115"/>
-      <c r="C43" s="115"/>
-      <c r="D43" s="115"/>
-      <c r="E43" s="115"/>
-      <c r="F43" s="115"/>
-      <c r="G43" s="115"/>
-      <c r="H43" s="115"/>
+      <c r="B43" s="112"/>
+      <c r="C43" s="112"/>
+      <c r="D43" s="112"/>
+      <c r="E43" s="112"/>
+      <c r="F43" s="112"/>
+      <c r="G43" s="112"/>
+      <c r="H43" s="112"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" s="212" t="s">
-        <v>187</v>
+      <c r="A45" s="198" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A46" s="207" t="s">
-        <v>188</v>
-      </c>
-      <c r="H46" s="186">
+      <c r="A46" s="193" t="s">
+        <v>176</v>
+      </c>
+      <c r="H46" s="173">
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A47" s="207" t="s">
-        <v>189</v>
-      </c>
-      <c r="H47" s="235" t="e">
+      <c r="A47" s="193" t="s">
+        <v>177</v>
+      </c>
+      <c r="H47" s="217" t="e">
         <f>-H15</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A48" s="207"/>
-      <c r="H48" s="186" t="e">
+      <c r="A48" s="193"/>
+      <c r="H48" s="173" t="e">
         <f>SUM(H46:H47)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" s="207"/>
+      <c r="A49" s="193"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A50" s="207" t="s">
-        <v>190</v>
+      <c r="A50" s="193" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A51" s="207" t="s">
-        <v>191</v>
-      </c>
-      <c r="H51" s="186">
+      <c r="A51" s="193" t="s">
+        <v>179</v>
+      </c>
+      <c r="H51" s="173">
         <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="207" t="s">
-        <v>192</v>
-      </c>
-      <c r="H52" s="186">
+      <c r="A52" s="193" t="s">
+        <v>180</v>
+      </c>
+      <c r="H52" s="173">
         <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A53" s="207" t="s">
-        <v>193</v>
-      </c>
-      <c r="H53" s="236" t="e">
+      <c r="A53" s="193" t="s">
+        <v>181</v>
+      </c>
+      <c r="H53" s="218" t="e">
         <f>SUM(H48:H52)</f>
         <v>#REF!</v>
       </c>
@@ -3136,112 +3092,112 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="239" t="s">
-        <v>161</v>
+      <c r="A1" s="221" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>111</v>
-      </c>
-      <c r="B2" s="175">
+        <v>107</v>
+      </c>
+      <c r="B2" s="165">
         <v>2328236</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="175"/>
+      <c r="B3" s="165"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="239" t="s">
-        <v>198</v>
-      </c>
-      <c r="B4" s="175"/>
+      <c r="A4" s="221" t="s">
+        <v>186</v>
+      </c>
+      <c r="B4" s="165"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>158</v>
-      </c>
-      <c r="B5" s="180">
+        <v>152</v>
+      </c>
+      <c r="B5" s="170">
         <v>99975</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="175"/>
+      <c r="B6" s="165"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="175"/>
+      <c r="B7" s="165"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="239" t="s">
-        <v>20</v>
+      <c r="A8" s="221" t="s">
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B9" s="175"/>
+      <c r="B9" s="165"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="175"/>
+      <c r="B10" s="165"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="239" t="s">
-        <v>199</v>
-      </c>
-      <c r="B11" s="175"/>
+      <c r="A11" s="221" t="s">
+        <v>187</v>
+      </c>
+      <c r="B11" s="165"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B12" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C12" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D12" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="177">
+      <c r="A13" s="167">
         <v>45597</v>
       </c>
-      <c r="B13" s="175">
+      <c r="B13" s="165">
         <v>4200</v>
       </c>
-      <c r="C13" s="175">
+      <c r="C13" s="165">
         <f>B13*12/20</f>
         <v>2520</v>
       </c>
-      <c r="D13" s="175">
+      <c r="D13" s="165">
         <f>C13*3/12</f>
         <v>630</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="178">
+        <v>27</v>
+      </c>
+      <c r="B14" s="168">
         <f>SUM(B13:B13)</f>
         <v>4200</v>
       </c>
-      <c r="C14" s="179">
+      <c r="C14" s="169">
         <f>SUM(C13:C13)</f>
         <v>2520</v>
       </c>
-      <c r="D14" s="179">
+      <c r="D14" s="169">
         <f>SUM(D13:D13)</f>
         <v>630</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="175"/>
-      <c r="C15" s="175"/>
-      <c r="D15" s="175"/>
+      <c r="B15" s="165"/>
+      <c r="C15" s="165"/>
+      <c r="D15" s="165"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3252,460 +3208,230 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.109375" style="172" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" style="91" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" style="174" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" style="166" bestFit="1" customWidth="1"/>
-    <col min="5" max="9" width="9.109375" style="166"/>
-    <col min="10" max="10" width="11.5546875" style="166" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="166"/>
+    <col min="1" max="1" width="25" style="163" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" style="88" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="164" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" style="161" bestFit="1" customWidth="1"/>
+    <col min="5" max="9" width="9.109375" style="161"/>
+    <col min="10" max="10" width="11.5546875" style="161" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.109375" style="161"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="240" t="s">
-        <v>155</v>
-      </c>
-      <c r="B1" s="240"/>
-      <c r="C1" s="240"/>
+    <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A1" s="222" t="s">
+        <v>149</v>
+      </c>
+      <c r="B1" s="222"/>
+      <c r="C1" s="222"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="240" t="s">
+    <row r="2" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A2" s="222" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="240"/>
-      <c r="C2" s="240"/>
+      <c r="B2" s="222"/>
+      <c r="C2" s="222"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="240" t="s">
-        <v>112</v>
-      </c>
-      <c r="B3" s="240"/>
-      <c r="C3" s="240"/>
+    <row r="3" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A3" s="222" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="222"/>
+      <c r="C3" s="222"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="167"/>
-      <c r="B4" s="168" t="s">
+    <row r="4" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A4" s="223"/>
+      <c r="B4" s="224" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="88" t="s">
+      <c r="C4" s="225" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="169" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="89"/>
-      <c r="C5" s="89"/>
+    <row r="5" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A5" s="226" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="227"/>
+      <c r="C5" s="227"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="170" t="s">
-        <v>126</v>
-      </c>
-      <c r="B6" s="184">
+    <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A6" s="228" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="234">
         <v>12560</v>
       </c>
-      <c r="C6" s="89"/>
+      <c r="C6" s="227"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="170"/>
-      <c r="B7" s="141"/>
-      <c r="C7" s="89"/>
+    <row r="7" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A7" s="226" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="227"/>
+      <c r="C7" s="227"/>
+      <c r="J7" s="162"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="169" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="89"/>
-      <c r="C8" s="89"/>
-      <c r="J8" s="171"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="170" t="s">
-        <v>116</v>
-      </c>
-      <c r="B9" s="182">
+    <row r="8" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A8" s="228" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="227">
         <f>+PPE!D4</f>
         <v>153700</v>
       </c>
-      <c r="C9" s="89"/>
-      <c r="J9" s="171"/>
+      <c r="C8" s="227"/>
+      <c r="J8" s="162"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="170" t="s">
-        <v>162</v>
-      </c>
-      <c r="B10" s="182" t="e">
-        <f>+PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C10" s="89"/>
-      <c r="J10" s="171"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="170" t="s">
-        <v>164</v>
-      </c>
-      <c r="B11" s="182" t="e">
-        <f>+PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C11" s="89"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="170" t="s">
-        <v>116</v>
-      </c>
-      <c r="B12" s="182" t="e">
-        <f>+PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C12" s="89"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="170" t="s">
-        <v>165</v>
-      </c>
-      <c r="B13" s="182" t="e">
-        <f>+PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C13" s="89"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="170" t="s">
-        <v>166</v>
-      </c>
-      <c r="B14" s="182" t="e">
-        <f>+PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C14" s="89"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="170" t="s">
-        <v>128</v>
-      </c>
-      <c r="B15" s="89"/>
-      <c r="C15" s="182">
+    <row r="9" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A9" s="228" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" s="227"/>
+      <c r="C9" s="227">
         <f>+PPE!G5</f>
         <v>28887.178082191782</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="170"/>
-      <c r="B16" s="89"/>
-      <c r="C16" s="89"/>
+    <row r="10" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A10" s="226" t="s">
+        <v>188</v>
+      </c>
+      <c r="B10" s="227"/>
+      <c r="C10" s="227"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="170" t="s">
-        <v>127</v>
-      </c>
-      <c r="B17" s="89"/>
-      <c r="C17" s="182">
-        <f>+B47</f>
+    <row r="11" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A11" s="228" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" s="227"/>
+      <c r="C11" s="227">
+        <f>+B22</f>
         <v>15000</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="170" t="s">
-        <v>104</v>
-      </c>
-      <c r="B18" s="89"/>
-      <c r="C18" s="182">
-        <f>+B48</f>
+    <row r="12" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A12" s="228" t="s">
+        <v>100</v>
+      </c>
+      <c r="B12" s="227"/>
+      <c r="C12" s="227">
+        <f>+B23</f>
         <v>25000</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="170" t="s">
-        <v>171</v>
-      </c>
-      <c r="B19" s="89"/>
-      <c r="C19" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
+    <row r="13" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="221" t="s">
+        <v>189</v>
+      </c>
+      <c r="B13" s="229"/>
+      <c r="C13" s="230"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="170" t="s">
-        <v>172</v>
-      </c>
-      <c r="B20" s="89"/>
-      <c r="C20" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E20" s="174" t="e">
-        <f>C20*20/3</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="166"/>
-      <c r="C21" s="117"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="170" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="89"/>
-      <c r="C22" s="182">
+    <row r="14" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A14" s="228" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="227"/>
+      <c r="C14" s="227">
         <f>1000*6</f>
         <v>6000</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="B23" s="89"/>
-      <c r="C23" s="214">
+    <row r="15" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A15" s="228" t="s">
+        <v>170</v>
+      </c>
+      <c r="B15" s="227"/>
+      <c r="C15" s="227">
         <v>1000000</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="230" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="231"/>
-      <c r="B24" s="213"/>
-      <c r="C24" s="219"/>
+    <row r="16" spans="1:10" s="213" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="226" t="s">
+        <v>155</v>
+      </c>
+      <c r="B16" s="227"/>
+      <c r="C16" s="230"/>
     </row>
-    <row r="25" spans="1:5" s="230" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="231"/>
-      <c r="B25" s="213"/>
-      <c r="C25" s="219"/>
+    <row r="17" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A17" s="231" t="s">
+        <v>171</v>
+      </c>
+      <c r="B17" s="235">
+        <v>112919.5</v>
+      </c>
+      <c r="C17" s="227"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="173" t="s">
-        <v>183</v>
-      </c>
-      <c r="B26" s="193">
-        <v>112919.5</v>
-      </c>
-      <c r="C26" s="89"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="170" t="s">
-        <v>161</v>
-      </c>
-      <c r="B27" s="89"/>
-      <c r="C27" s="183">
+    <row r="18" spans="1:3" s="213" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="228" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="227"/>
+      <c r="C18" s="236">
         <f>+Working!B2</f>
         <v>2328236</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="169" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" s="89"/>
-      <c r="C28" s="89"/>
+    <row r="19" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="221" t="s">
+        <v>190</v>
+      </c>
+      <c r="B19" s="227"/>
+      <c r="C19" s="227"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="170" t="s">
-        <v>141</v>
-      </c>
-      <c r="B29" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C29" s="89"/>
+    <row r="20" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="228" t="s">
+        <v>166</v>
+      </c>
+      <c r="B20" s="227">
+        <v>1220000</v>
+      </c>
+      <c r="C20" s="227"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="170" t="s">
-        <v>178</v>
-      </c>
-      <c r="B30" s="182">
-        <v>1220000</v>
-      </c>
-      <c r="C30" s="89"/>
+    <row r="21" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A21" s="228" t="s">
+        <v>142</v>
+      </c>
+      <c r="B21" s="227"/>
+      <c r="C21" s="227"/>
     </row>
-    <row r="31" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>158</v>
-      </c>
-      <c r="B31" s="182">
-        <f>Working!B5</f>
-        <v>99975</v>
-      </c>
-      <c r="C31" s="89"/>
+    <row r="22" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A22" s="228" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" s="227">
+        <v>15000</v>
+      </c>
+      <c r="C22" s="227"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="170" t="s">
-        <v>174</v>
-      </c>
-      <c r="B32" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C32" s="89"/>
+    <row r="23" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A23" s="228" t="s">
+        <v>100</v>
+      </c>
+      <c r="B23" s="227">
+        <v>25000</v>
+      </c>
+      <c r="C23" s="227"/>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="170" t="s">
-        <v>113</v>
-      </c>
-      <c r="B33" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C33" s="89"/>
+    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="232" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="233">
+        <f>SUM(B5:B23)</f>
+        <v>1539179.5</v>
+      </c>
+      <c r="C24" s="233">
+        <f>SUM(C5:C23)</f>
+        <v>3403123.1780821919</v>
+      </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="170" t="s">
-        <v>171</v>
-      </c>
-      <c r="B34" s="182">
-        <f>+Working!C14</f>
-        <v>2520</v>
-      </c>
-      <c r="C34" s="89"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="170" t="s">
-        <v>172</v>
-      </c>
-      <c r="B35" s="182">
-        <f>Working!D14</f>
-        <v>630</v>
-      </c>
-      <c r="C35" s="89"/>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="170" t="s">
-        <v>175</v>
-      </c>
-      <c r="B36" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C36" s="89"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="170" t="s">
-        <v>101</v>
-      </c>
-      <c r="B37" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C37" s="89"/>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="170" t="s">
-        <v>102</v>
-      </c>
-      <c r="B38" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C38" s="89"/>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="170" t="s">
-        <v>110</v>
-      </c>
-      <c r="B39" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C39" s="89"/>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="170" t="s">
-        <v>114</v>
-      </c>
-      <c r="B40" s="89"/>
-      <c r="C40" s="89"/>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="170" t="s">
-        <v>159</v>
-      </c>
-      <c r="B41" s="214">
-        <v>163480</v>
-      </c>
-      <c r="C41" s="89"/>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="170" t="s">
-        <v>160</v>
-      </c>
-      <c r="B42" s="182" t="e">
-        <f>+Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C42" s="89"/>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="170" t="s">
-        <v>103</v>
-      </c>
-      <c r="B43" s="89"/>
-      <c r="C43" s="89"/>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="170" t="s">
-        <v>100</v>
-      </c>
-      <c r="B44" s="182" t="e">
-        <f>Working!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C44" s="89"/>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="170" t="s">
-        <v>144</v>
-      </c>
-      <c r="B45" s="182" t="e">
-        <f>'P10'!G22</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C45" s="89"/>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="170" t="s">
-        <v>148</v>
-      </c>
-      <c r="B46" s="89"/>
-      <c r="C46" s="89"/>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="170" t="s">
-        <v>127</v>
-      </c>
-      <c r="B47" s="182">
-        <v>15000</v>
-      </c>
-      <c r="C47" s="89"/>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="170" t="s">
-        <v>104</v>
-      </c>
-      <c r="B48" s="182">
-        <v>25000</v>
-      </c>
-      <c r="C48" s="89"/>
-    </row>
-    <row r="49" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="167"/>
-      <c r="B49" s="90" t="e">
-        <f>SUM(B5:B48)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C49" s="90" t="e">
-        <f>SUM(C5:C48)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" ht="14.4" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B51" s="91" t="e">
-        <f>B49-C49</f>
-        <v>#REF!</v>
+    <row r="25" spans="1:3" ht="14.4" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="88">
+        <f>B24-C24</f>
+        <v>-1863943.6780821919</v>
       </c>
     </row>
   </sheetData>
@@ -3737,17 +3463,17 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="165" t="s">
-        <v>29</v>
+      <c r="D1" s="160" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -3755,7 +3481,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -3765,10 +3491,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -3778,13 +3504,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6" s="3">
         <v>4</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="122">
+      <c r="D6" s="118">
         <f>+'P09'!D8</f>
         <v>2328236</v>
       </c>
@@ -3793,7 +3519,7 @@
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B7" s="3"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="122"/>
+      <c r="D7" s="118"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
@@ -3803,7 +3529,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="125" t="e">
+      <c r="D8" s="121" t="e">
         <f>-'P09'!D26</f>
         <v>#REF!</v>
       </c>
@@ -3813,80 +3539,80 @@
       <c r="A9" s="1"/>
       <c r="B9" s="3"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="126"/>
+      <c r="D9" s="122"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B10" s="3">
         <v>6</v>
       </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="127">
+      <c r="D10" s="123" t="e">
         <f>-'P09'!D30</f>
-        <v>-163480</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="D11" s="122"/>
+      <c r="D11" s="118"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="D12" s="123" t="e">
+      <c r="D12" s="119" t="e">
         <f>SUM(D6:D10)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="D13" s="123"/>
+      <c r="D13" s="119"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" s="3">
         <v>7</v>
       </c>
-      <c r="D14" s="127">
+      <c r="D14" s="123">
         <f>-'P09'!D34</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="D15" s="123"/>
+      <c r="D15" s="119"/>
     </row>
     <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="12" t="s">
-        <v>196</v>
-      </c>
-      <c r="D16" s="128" t="e">
+        <v>184</v>
+      </c>
+      <c r="D16" s="124" t="e">
         <f>SUM(D12:D14)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="D17" s="122"/>
+      <c r="D17" s="118"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
-      <c r="D18" s="129"/>
+      <c r="D18" s="125"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D19" s="7"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -3917,13 +3643,13 @@
   <sheetData>
     <row r="1" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="165" t="s">
-        <v>37</v>
+      <c r="E1" s="160" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:1003" x14ac:dyDescent="0.35">
@@ -3937,7 +3663,7 @@
     </row>
     <row r="3" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -3950,7 +3676,7 @@
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="16" t="s">
@@ -3966,40 +3692,40 @@
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="157"/>
+      <c r="B6" s="152"/>
     </row>
     <row r="7" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1"/>
       <c r="E7" s="73"/>
-      <c r="F7" s="156"/>
+      <c r="F7" s="151"/>
     </row>
     <row r="8" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A8" s="18" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C8" s="3">
         <v>8</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="125" t="e">
+      <c r="E8" s="121" t="e">
         <f>+'P10'!J31</f>
         <v>#REF!</v>
       </c>
-      <c r="F8" s="156"/>
+      <c r="F8" s="151"/>
     </row>
     <row r="9" spans="1:1003" x14ac:dyDescent="0.35">
-      <c r="E9" s="130" t="e">
+      <c r="E9" s="126" t="e">
         <f>SUM(E8)</f>
         <v>#REF!</v>
       </c>
-      <c r="F9" s="156"/>
+      <c r="F9" s="151"/>
     </row>
     <row r="10" spans="1:1003" x14ac:dyDescent="0.35">
-      <c r="E10" s="125"/>
-      <c r="F10" s="156"/>
+      <c r="E10" s="121"/>
+      <c r="F10" s="151"/>
     </row>
     <row r="11" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
@@ -4007,7 +3733,7 @@
       </c>
       <c r="B11" s="1"/>
       <c r="E11" s="73"/>
-      <c r="F11" s="104"/>
+      <c r="F11" s="101"/>
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
       <c r="I11" s="13"/>
@@ -5007,17 +4733,17 @@
       <c r="ALO11" s="13"/>
     </row>
     <row r="12" spans="1:1003" x14ac:dyDescent="0.35">
-      <c r="A12" s="155" t="s">
-        <v>183</v>
-      </c>
-      <c r="B12" s="155"/>
-      <c r="C12" s="237"/>
-      <c r="D12" s="237"/>
-      <c r="E12" s="238">
-        <f>TB!B26</f>
+      <c r="A12" s="150" t="s">
+        <v>171</v>
+      </c>
+      <c r="B12" s="150"/>
+      <c r="C12" s="219"/>
+      <c r="D12" s="219"/>
+      <c r="E12" s="220">
+        <f>TB!B17</f>
         <v>112919.5</v>
       </c>
-      <c r="F12" s="104"/>
+      <c r="F12" s="101"/>
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
       <c r="I12" s="13"/>
@@ -6028,7 +5754,7 @@
         <f>+'P11'!J8</f>
         <v>12560</v>
       </c>
-      <c r="F13" s="104"/>
+      <c r="F13" s="101"/>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
       <c r="I13" s="13"/>
@@ -7029,15 +6755,15 @@
     </row>
     <row r="14" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
-      <c r="E14" s="130">
+      <c r="E14" s="126">
         <f>SUM(E12:E13)</f>
         <v>125479.5</v>
       </c>
-      <c r="F14" s="104"/>
+      <c r="F14" s="101"/>
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
@@ -8041,11 +7767,11 @@
         <v>4</v>
       </c>
       <c r="B15" s="1"/>
-      <c r="E15" s="131" t="e">
+      <c r="E15" s="127" t="e">
         <f>SUM(E14+E9)</f>
         <v>#REF!</v>
       </c>
-      <c r="F15" s="104"/>
+      <c r="F15" s="101"/>
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
       <c r="I15" s="13"/>
@@ -9045,8 +8771,8 @@
       <c r="ALO15" s="13"/>
     </row>
     <row r="16" spans="1:1003" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="E16" s="125"/>
-      <c r="F16" s="156"/>
+      <c r="E16" s="121"/>
+      <c r="F16" s="151"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13"/>
       <c r="L16" s="13"/>
@@ -10046,10 +9772,10 @@
       <c r="A17" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="157"/>
+      <c r="B17" s="152"/>
       <c r="E17" s="73"/>
-      <c r="F17" s="156"/>
-      <c r="I17" s="158"/>
+      <c r="F17" s="151"/>
+      <c r="I17" s="153"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13"/>
       <c r="L17" s="13"/>
@@ -11047,11 +10773,11 @@
     </row>
     <row r="18" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="A18" s="19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" s="1"/>
       <c r="E18" s="73"/>
-      <c r="F18" s="156"/>
+      <c r="F18" s="151"/>
       <c r="J18" s="13"/>
       <c r="K18" s="13"/>
       <c r="L18" s="13"/>
@@ -12059,7 +11785,7 @@
         <f>+'P11'!J17</f>
         <v>6000</v>
       </c>
-      <c r="F19" s="156"/>
+      <c r="F19" s="151"/>
       <c r="J19" s="13"/>
       <c r="K19" s="13"/>
       <c r="L19" s="13"/>
@@ -13063,7 +12789,7 @@
         <f>+CE!G13</f>
         <v>#REF!</v>
       </c>
-      <c r="F20" s="156"/>
+      <c r="F20" s="151"/>
       <c r="J20" s="13"/>
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
@@ -14060,11 +13786,11 @@
       <c r="ALO20" s="13"/>
     </row>
     <row r="21" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="E21" s="130" t="e">
+      <c r="E21" s="126" t="e">
         <f>SUM(E19:E20)</f>
         <v>#REF!</v>
       </c>
-      <c r="F21" s="156"/>
+      <c r="F21" s="151"/>
       <c r="J21" s="62"/>
       <c r="K21" s="13"/>
       <c r="L21" s="13"/>
@@ -15061,8 +14787,8 @@
       <c r="ALO21" s="13"/>
     </row>
     <row r="22" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="E22" s="125"/>
-      <c r="F22" s="156"/>
+      <c r="E22" s="121"/>
+      <c r="F22" s="151"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
       <c r="L22" s="13"/>
@@ -16060,12 +15786,12 @@
     </row>
     <row r="23" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E23" s="125">
+        <v>40</v>
+      </c>
+      <c r="E23" s="121">
         <v>0</v>
       </c>
-      <c r="F23" s="156"/>
+      <c r="F23" s="151"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
@@ -17063,7 +16789,7 @@
     </row>
     <row r="24" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="E24" s="73"/>
-      <c r="F24" s="156"/>
+      <c r="F24" s="151"/>
       <c r="J24" s="13"/>
       <c r="K24" s="13"/>
       <c r="L24" s="13"/>
@@ -18065,7 +17791,7 @@
       </c>
       <c r="B25" s="1"/>
       <c r="E25" s="73"/>
-      <c r="F25" s="156"/>
+      <c r="F25" s="151"/>
       <c r="J25" s="13"/>
       <c r="K25" s="13"/>
       <c r="L25" s="13"/>
@@ -19062,8 +18788,8 @@
       <c r="ALO25" s="13"/>
     </row>
     <row r="26" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A26" s="159" t="s">
-        <v>109</v>
+      <c r="A26" s="154" t="s">
+        <v>105</v>
       </c>
       <c r="C26" s="3">
         <v>11</v>
@@ -19073,7 +18799,7 @@
         <f>+'P11'!J24</f>
         <v>#REF!</v>
       </c>
-      <c r="F26" s="156"/>
+      <c r="F26" s="151"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
       <c r="L26" s="13"/>
@@ -20070,15 +19796,15 @@
       <c r="ALO26" s="13"/>
     </row>
     <row r="27" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A27" s="159" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" s="160"/>
+      <c r="A27" s="154" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="155"/>
       <c r="E27" s="73">
-        <f>TB!C23</f>
+        <f>TB!C15</f>
         <v>1000000</v>
       </c>
-      <c r="F27" s="156"/>
+      <c r="F27" s="151"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
@@ -21075,14 +20801,14 @@
       <c r="ALO27" s="13"/>
     </row>
     <row r="28" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A28" s="161" t="s">
-        <v>42</v>
-      </c>
-      <c r="E28" s="130" t="e">
+      <c r="A28" s="156" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" s="126" t="e">
         <f>SUM(E26:E27)</f>
         <v>#REF!</v>
       </c>
-      <c r="F28" s="156"/>
+      <c r="F28" s="151"/>
       <c r="J28" s="13"/>
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
@@ -22079,14 +21805,14 @@
       <c r="ALO28" s="13"/>
     </row>
     <row r="29" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A29" s="161" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="132" t="e">
+      <c r="A29" s="156" t="s">
+        <v>42</v>
+      </c>
+      <c r="E29" s="128" t="e">
         <f>E28+E23</f>
         <v>#REF!</v>
       </c>
-      <c r="F29" s="156"/>
+      <c r="F29" s="151"/>
       <c r="J29" s="13"/>
       <c r="K29" s="13"/>
       <c r="L29" s="13"/>
@@ -23087,11 +22813,11 @@
         <v>9</v>
       </c>
       <c r="B30" s="1"/>
-      <c r="E30" s="131" t="e">
+      <c r="E30" s="127" t="e">
         <f>+E21+E29</f>
         <v>#REF!</v>
       </c>
-      <c r="F30" s="156"/>
+      <c r="F30" s="151"/>
       <c r="G30" s="77" t="e">
         <f>E15-E30</f>
         <v>#REF!</v>
@@ -24092,7 +23818,7 @@
       <c r="ALO30" s="13"/>
     </row>
     <row r="31" spans="1:1012" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="E31" s="125"/>
+      <c r="E31" s="121"/>
       <c r="J31" s="13"/>
       <c r="K31" s="13"/>
       <c r="L31" s="13"/>
@@ -26106,7 +25832,7 @@
     </row>
     <row r="33" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="E33" s="20"/>
-      <c r="G33" s="92"/>
+      <c r="G33" s="89"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
@@ -29128,16 +28854,16 @@
       <c r="ALX35" s="2"/>
     </row>
     <row r="36" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="162" t="s">
-        <v>44</v>
-      </c>
-      <c r="B36" s="162"/>
-      <c r="C36" s="162"/>
-      <c r="D36" s="162"/>
+      <c r="A36" s="157" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="157"/>
+      <c r="C36" s="157"/>
+      <c r="D36" s="157"/>
       <c r="E36" s="24"/>
-      <c r="F36" s="162"/>
-      <c r="G36" s="162"/>
-      <c r="H36" s="162"/>
+      <c r="F36" s="157"/>
+      <c r="G36" s="157"/>
+      <c r="H36" s="157"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
@@ -30143,14 +29869,14 @@
       <c r="ALX36" s="2"/>
     </row>
     <row r="37" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="162"/>
-      <c r="B37" s="162"/>
-      <c r="C37" s="162"/>
-      <c r="D37" s="162"/>
+      <c r="A37" s="157"/>
+      <c r="B37" s="157"/>
+      <c r="C37" s="157"/>
+      <c r="D37" s="157"/>
       <c r="E37" s="24"/>
-      <c r="F37" s="162"/>
-      <c r="G37" s="162"/>
-      <c r="H37" s="162"/>
+      <c r="F37" s="157"/>
+      <c r="G37" s="157"/>
+      <c r="H37" s="157"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
@@ -31156,14 +30882,14 @@
       <c r="ALX37" s="2"/>
     </row>
     <row r="38" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="163"/>
-      <c r="B38" s="163"/>
-      <c r="C38" s="163"/>
-      <c r="D38" s="163"/>
+      <c r="A38" s="158"/>
+      <c r="B38" s="158"/>
+      <c r="C38" s="158"/>
+      <c r="D38" s="158"/>
       <c r="E38" s="25"/>
-      <c r="F38" s="163"/>
-      <c r="G38" s="163"/>
-      <c r="H38" s="163"/>
+      <c r="F38" s="158"/>
+      <c r="G38" s="158"/>
+      <c r="H38" s="158"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
@@ -32170,7 +31896,7 @@
     </row>
     <row r="39" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E39" s="20"/>
       <c r="J39" s="2"/>
@@ -33179,7 +32905,7 @@
     </row>
     <row r="40" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E40" s="20"/>
       <c r="J40" s="2"/>
@@ -35193,16 +34919,16 @@
       <c r="ALX41" s="2"/>
     </row>
     <row r="42" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="162" t="s">
-        <v>47</v>
-      </c>
-      <c r="B42" s="164"/>
-      <c r="C42" s="164"/>
-      <c r="D42" s="164"/>
+      <c r="A42" s="157" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42" s="159"/>
+      <c r="C42" s="159"/>
+      <c r="D42" s="159"/>
       <c r="E42" s="26"/>
-      <c r="F42" s="164"/>
-      <c r="G42" s="164"/>
-      <c r="H42" s="164"/>
+      <c r="F42" s="159"/>
+      <c r="G42" s="159"/>
+      <c r="H42" s="159"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
@@ -36208,16 +35934,16 @@
       <c r="ALX42" s="2"/>
     </row>
     <row r="43" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="162" t="s">
-        <v>48</v>
-      </c>
-      <c r="B43" s="164"/>
-      <c r="C43" s="164"/>
-      <c r="D43" s="164"/>
+      <c r="A43" s="157" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" s="159"/>
+      <c r="C43" s="159"/>
+      <c r="D43" s="159"/>
       <c r="E43" s="26"/>
-      <c r="F43" s="164"/>
-      <c r="G43" s="164"/>
-      <c r="H43" s="164"/>
+      <c r="F43" s="159"/>
+      <c r="G43" s="159"/>
+      <c r="H43" s="159"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
@@ -37223,14 +36949,14 @@
       <c r="ALX43" s="2"/>
     </row>
     <row r="44" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="162"/>
-      <c r="B44" s="164"/>
-      <c r="C44" s="164"/>
-      <c r="D44" s="164"/>
+      <c r="A44" s="157"/>
+      <c r="B44" s="159"/>
+      <c r="C44" s="159"/>
+      <c r="D44" s="159"/>
       <c r="E44" s="26"/>
-      <c r="F44" s="164"/>
-      <c r="G44" s="164"/>
-      <c r="H44" s="164"/>
+      <c r="F44" s="159"/>
+      <c r="G44" s="159"/>
+      <c r="H44" s="159"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
@@ -38236,14 +37962,14 @@
       <c r="ALX44" s="2"/>
     </row>
     <row r="45" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="162"/>
-      <c r="B45" s="164"/>
-      <c r="C45" s="164"/>
-      <c r="D45" s="164"/>
+      <c r="A45" s="157"/>
+      <c r="B45" s="159"/>
+      <c r="C45" s="159"/>
+      <c r="D45" s="159"/>
       <c r="E45" s="26"/>
-      <c r="F45" s="164"/>
-      <c r="G45" s="164"/>
-      <c r="H45" s="164"/>
+      <c r="F45" s="159"/>
+      <c r="G45" s="159"/>
+      <c r="H45" s="159"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
@@ -39261,12 +38987,12 @@
     </row>
     <row r="47" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="A47" s="27" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
       <c r="D47" s="27" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F47" s="18"/>
       <c r="H47" s="18"/>
@@ -39274,12 +39000,12 @@
     </row>
     <row r="48" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="A48" s="28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B48" s="18"/>
       <c r="C48" s="18"/>
       <c r="D48" s="28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F48" s="18"/>
       <c r="H48" s="18"/>
@@ -41286,7 +41012,7 @@
     </row>
     <row r="50" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A50" s="28" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="B50" s="18"/>
       <c r="C50" s="18"/>
@@ -42293,7 +42019,7 @@
     </row>
     <row r="51" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A51" s="28" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="B51" s="18"/>
       <c r="C51" s="18"/>
@@ -43324,7 +43050,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -43333,14 +43059,14 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="165" t="s">
-        <v>51</v>
+      <c r="I1" s="160" t="s">
+        <v>50</v>
       </c>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" s="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -43354,7 +43080,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -43367,16 +43093,16 @@
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.35">
-      <c r="E4" s="93" t="s">
+      <c r="E4" s="90" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="31"/>
+      <c r="G4" s="90" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="31"/>
-      <c r="G4" s="93" t="s">
+      <c r="H4" s="31"/>
+      <c r="I4" s="90" t="s">
         <v>77</v>
-      </c>
-      <c r="H4" s="31"/>
-      <c r="I4" s="93" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -43389,7 +43115,7 @@
       </c>
       <c r="H5" s="31"/>
       <c r="I5" s="31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -43401,7 +43127,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E7" s="84">
         <v>0</v>
@@ -43424,32 +43150,32 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9" s="133">
-        <f>+TB!C22</f>
+        <v>70</v>
+      </c>
+      <c r="E9" s="129">
+        <f>+TB!C14</f>
         <v>6000</v>
       </c>
-      <c r="F9" s="133"/>
-      <c r="G9" s="133">
+      <c r="F9" s="129"/>
+      <c r="G9" s="129">
         <v>0</v>
       </c>
-      <c r="H9" s="133"/>
+      <c r="H9" s="129"/>
       <c r="I9" s="62">
         <f>+E9</f>
         <v>6000</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E10" s="133"/>
-      <c r="F10" s="133"/>
-      <c r="G10" s="133"/>
-      <c r="H10" s="133"/>
+      <c r="E10" s="129"/>
+      <c r="F10" s="129"/>
+      <c r="G10" s="129"/>
+      <c r="H10" s="129"/>
       <c r="I10" s="62"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E11" s="62">
         <v>0</v>
@@ -43474,29 +43200,29 @@
     </row>
     <row r="13" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="E13" s="194">
+        <v>126</v>
+      </c>
+      <c r="E13" s="180">
         <f>SUM(E7:E11)</f>
         <v>6000</v>
       </c>
-      <c r="F13" s="210"/>
-      <c r="G13" s="194" t="e">
+      <c r="F13" s="196"/>
+      <c r="G13" s="180" t="e">
         <f>SUM(G7:G11)</f>
         <v>#REF!</v>
       </c>
-      <c r="H13" s="210"/>
-      <c r="I13" s="194" t="e">
+      <c r="H13" s="196"/>
+      <c r="I13" s="180" t="e">
         <f>SUM(I7:I11)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="E14" s="134"/>
-      <c r="F14" s="134"/>
-      <c r="G14" s="134"/>
-      <c r="H14" s="134"/>
-      <c r="I14" s="134"/>
+      <c r="E14" s="130"/>
+      <c r="F14" s="130"/>
+      <c r="G14" s="130"/>
+      <c r="H14" s="130"/>
+      <c r="I14" s="130"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="E15" s="33"/>
@@ -43535,12 +43261,12 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -43555,344 +43281,344 @@
   <dimension ref="A1:I43"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.88671875" style="190" customWidth="1"/>
-    <col min="2" max="2" width="30.44140625" style="190" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" style="190" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" style="190" customWidth="1"/>
-    <col min="5" max="5" width="9" style="190" customWidth="1"/>
-    <col min="6" max="6" width="0.6640625" style="190" customWidth="1"/>
-    <col min="7" max="7" width="13.109375" style="190" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="190" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" style="190" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="190"/>
+    <col min="1" max="1" width="2.88671875" style="177" customWidth="1"/>
+    <col min="2" max="2" width="30.44140625" style="177" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" style="177" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" style="177" customWidth="1"/>
+    <col min="5" max="5" width="9" style="177" customWidth="1"/>
+    <col min="6" max="6" width="0.6640625" style="177" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" style="177" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="177" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" style="177" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="177"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="192" t="s">
-        <v>156</v>
-      </c>
-      <c r="E1" s="192"/>
-      <c r="F1" s="192"/>
-      <c r="G1" s="233" t="s">
-        <v>65</v>
-      </c>
-      <c r="H1" s="192"/>
+      <c r="A1" s="179" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="179"/>
+      <c r="F1" s="179"/>
+      <c r="G1" s="215" t="s">
+        <v>64</v>
+      </c>
+      <c r="H1" s="179"/>
     </row>
-    <row r="2" spans="1:8" s="187" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="192" t="s">
-        <v>53</v>
-      </c>
-      <c r="E2" s="192"/>
-      <c r="F2" s="192"/>
-      <c r="G2" s="203"/>
-      <c r="H2" s="192"/>
+    <row r="2" spans="1:8" s="174" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="179" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="189"/>
+      <c r="H2" s="179"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="187" t="str">
+      <c r="A3" s="174" t="str">
         <f>+PL!A3</f>
         <v>FOR THE YEAR PERIOD 31ST MARCH</v>
       </c>
-      <c r="B3" s="192"/>
-      <c r="C3" s="192"/>
-      <c r="D3" s="192"/>
-      <c r="E3" s="192"/>
-      <c r="F3" s="192"/>
-      <c r="G3" s="198">
+      <c r="B3" s="179"/>
+      <c r="C3" s="179"/>
+      <c r="D3" s="179"/>
+      <c r="E3" s="179"/>
+      <c r="F3" s="179"/>
+      <c r="G3" s="184">
         <v>2025</v>
       </c>
-      <c r="H3" s="192"/>
+      <c r="H3" s="179"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="G4" s="206" t="s">
+      <c r="G4" s="192" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F5" s="197"/>
+      <c r="F5" s="183"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="187" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="197"/>
-      <c r="G6" s="200"/>
+      <c r="A6" s="174" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="183"/>
+      <c r="G6" s="186"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="191" t="s">
-        <v>55</v>
-      </c>
-      <c r="F7" s="215"/>
-      <c r="G7" s="220" t="e">
+      <c r="A7" s="178" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" s="199"/>
+      <c r="G7" s="203" t="e">
         <f>+PL!D12</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="190" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" s="199"/>
-      <c r="G8" s="221"/>
+      <c r="A8" s="177" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="185"/>
+      <c r="G8" s="204"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B9" s="195" t="s">
-        <v>135</v>
-      </c>
-      <c r="C9" s="195"/>
-      <c r="D9" s="195"/>
-      <c r="F9" s="199"/>
-      <c r="G9" s="221" t="e">
+      <c r="B9" s="181" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" s="181"/>
+      <c r="D9" s="181"/>
+      <c r="F9" s="185"/>
+      <c r="G9" s="204" t="e">
         <f>'P09'!D22</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="187" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="199"/>
-      <c r="G10" s="222" t="e">
+      <c r="A10" s="174" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="185"/>
+      <c r="G10" s="205" t="e">
         <f>SUM(G7:G9)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F11" s="199"/>
-      <c r="G11" s="221"/>
+      <c r="F11" s="185"/>
+      <c r="G11" s="204"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B12" s="195" t="s">
-        <v>185</v>
-      </c>
-      <c r="C12" s="195"/>
-      <c r="D12" s="195"/>
-      <c r="F12" s="199"/>
-      <c r="G12" s="221">
+      <c r="B12" s="181" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" s="181"/>
+      <c r="D12" s="181"/>
+      <c r="F12" s="185"/>
+      <c r="G12" s="204">
         <f>-BS!E12</f>
         <v>-112919.5</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="195" t="s">
-        <v>195</v>
-      </c>
-      <c r="C13" s="195"/>
-      <c r="D13" s="195"/>
-      <c r="F13" s="199"/>
-      <c r="G13" s="221" t="e">
+      <c r="B13" s="181" t="s">
+        <v>183</v>
+      </c>
+      <c r="C13" s="181"/>
+      <c r="D13" s="181"/>
+      <c r="F13" s="185"/>
+      <c r="G13" s="204" t="e">
         <f>BS!E26</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B14" s="195" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="195"/>
-      <c r="D14" s="195"/>
-      <c r="F14" s="199"/>
-      <c r="G14" s="221">
+      <c r="B14" s="181" t="s">
+        <v>102</v>
+      </c>
+      <c r="C14" s="181"/>
+      <c r="D14" s="181"/>
+      <c r="F14" s="185"/>
+      <c r="G14" s="204">
         <f>BS!E27</f>
         <v>1000000</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="187" t="s">
-        <v>57</v>
-      </c>
-      <c r="F15" s="199"/>
-      <c r="G15" s="222" t="e">
+      <c r="A15" s="174" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" s="185"/>
+      <c r="G15" s="205" t="e">
         <f>SUM(G10:G14)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F16" s="199"/>
-      <c r="G16" s="221"/>
+      <c r="F16" s="185"/>
+      <c r="G16" s="204"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B17" s="190" t="s">
-        <v>25</v>
-      </c>
-      <c r="F17" s="199"/>
-      <c r="G17" s="221">
+      <c r="B17" s="177" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="185"/>
+      <c r="G17" s="204">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F18" s="199"/>
-      <c r="G18" s="223">
+      <c r="F18" s="185"/>
+      <c r="G18" s="206">
         <f>SUM(G17:G17)</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="187" t="s">
-        <v>58</v>
-      </c>
-      <c r="E19" s="187"/>
-      <c r="F19" s="199"/>
-      <c r="G19" s="223" t="e">
+      <c r="A19" s="174" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" s="174"/>
+      <c r="F19" s="185"/>
+      <c r="G19" s="206" t="e">
         <f>SUM(G18+G15)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F20" s="199"/>
-      <c r="G20" s="221"/>
+      <c r="F20" s="185"/>
+      <c r="G20" s="204"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="187" t="s">
-        <v>59</v>
-      </c>
-      <c r="F21" s="199"/>
-      <c r="G21" s="221"/>
+      <c r="A21" s="174" t="s">
+        <v>58</v>
+      </c>
+      <c r="F21" s="185"/>
+      <c r="G21" s="204"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B22" s="191" t="s">
-        <v>149</v>
-      </c>
-      <c r="F22" s="199"/>
-      <c r="G22" s="221" t="e">
+      <c r="B22" s="178" t="s">
+        <v>143</v>
+      </c>
+      <c r="F22" s="185"/>
+      <c r="G22" s="204" t="e">
         <f>-'P10'!G12</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="187" t="s">
-        <v>60</v>
-      </c>
-      <c r="E23" s="187"/>
-      <c r="F23" s="199"/>
-      <c r="G23" s="223" t="e">
+      <c r="A23" s="174" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="174"/>
+      <c r="F23" s="185"/>
+      <c r="G23" s="206" t="e">
         <f>SUM(G22)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F24" s="199"/>
-      <c r="G24" s="221"/>
+      <c r="F24" s="185"/>
+      <c r="G24" s="204"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="187" t="s">
-        <v>61</v>
-      </c>
-      <c r="F25" s="199"/>
-      <c r="G25" s="221"/>
+      <c r="A25" s="174" t="s">
+        <v>60</v>
+      </c>
+      <c r="F25" s="185"/>
+      <c r="G25" s="204"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B26" s="190" t="s">
-        <v>71</v>
-      </c>
-      <c r="F26" s="199"/>
-      <c r="G26" s="221">
+      <c r="B26" s="177" t="s">
+        <v>70</v>
+      </c>
+      <c r="F26" s="185"/>
+      <c r="G26" s="204">
         <f>+BS!E19</f>
         <v>6000</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="187" t="s">
-        <v>62</v>
-      </c>
-      <c r="F27" s="199"/>
-      <c r="G27" s="223">
+      <c r="A27" s="174" t="s">
+        <v>61</v>
+      </c>
+      <c r="F27" s="185"/>
+      <c r="G27" s="206">
         <f>SUM(G26)</f>
         <v>6000</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="187" t="s">
-        <v>66</v>
-      </c>
-      <c r="F28" s="199"/>
-      <c r="G28" s="221" t="e">
+      <c r="A28" s="174" t="s">
+        <v>65</v>
+      </c>
+      <c r="F28" s="185"/>
+      <c r="G28" s="204" t="e">
         <f>+G19+G23+G27</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B29" s="190" t="s">
-        <v>63</v>
-      </c>
-      <c r="F29" s="199"/>
-      <c r="G29" s="221">
+      <c r="B29" s="177" t="s">
+        <v>62</v>
+      </c>
+      <c r="F29" s="185"/>
+      <c r="G29" s="204">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="190" t="s">
-        <v>64</v>
-      </c>
-      <c r="F30" s="199"/>
-      <c r="G30" s="224" t="e">
+      <c r="B30" s="177" t="s">
+        <v>63</v>
+      </c>
+      <c r="F30" s="185"/>
+      <c r="G30" s="207" t="e">
         <f>SUM(G28:G29)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="F31" s="199"/>
-      <c r="G31" s="221"/>
+      <c r="F31" s="185"/>
+      <c r="G31" s="204"/>
     </row>
-    <row r="32" spans="1:7" s="191" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="188" t="s">
-        <v>151</v>
-      </c>
-      <c r="C32" s="185"/>
-      <c r="F32" s="209"/>
+    <row r="32" spans="1:7" s="178" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="175" t="s">
+        <v>145</v>
+      </c>
+      <c r="C32" s="172"/>
+      <c r="F32" s="195"/>
     </row>
-    <row r="33" spans="1:9" s="191" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="202" t="s">
-        <v>150</v>
-      </c>
-      <c r="G33" s="208">
+    <row r="33" spans="1:9" s="178" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="188" t="s">
+        <v>144</v>
+      </c>
+      <c r="G33" s="194">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" s="191" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G34" s="234">
+    <row r="34" spans="1:9" s="178" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G34" s="216">
         <f>SUM(F33:F33)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" s="191" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="36" spans="1:9" s="191" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="188" t="s">
-        <v>152</v>
-      </c>
-      <c r="G36" s="209"/>
+    <row r="35" spans="1:9" s="178" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="1:9" s="178" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="175" t="s">
+        <v>146</v>
+      </c>
+      <c r="G36" s="195"/>
     </row>
-    <row r="37" spans="1:9" s="191" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="202" t="s">
-        <v>150</v>
-      </c>
-      <c r="D37" s="201"/>
-      <c r="E37" s="201"/>
-      <c r="G37" s="208">
+    <row r="37" spans="1:9" s="178" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="188" t="s">
+        <v>144</v>
+      </c>
+      <c r="D37" s="187"/>
+      <c r="E37" s="187"/>
+      <c r="G37" s="194">
         <f>'P11'!J7</f>
         <v>12560</v>
       </c>
     </row>
-    <row r="38" spans="1:9" s="191" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="188"/>
-      <c r="G38" s="234">
+    <row r="38" spans="1:9" s="178" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="175"/>
+      <c r="G38" s="216">
         <f>SUM(G37:G37)</f>
         <v>12560</v>
       </c>
-      <c r="H38" s="204" t="e">
+      <c r="H38" s="190" t="e">
         <f>G30-G38</f>
         <v>#REF!</v>
       </c>
-      <c r="I38" s="204"/>
+      <c r="I38" s="190"/>
     </row>
     <row r="39" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A41" s="190" t="s">
-        <v>33</v>
+      <c r="A41" s="177" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43" s="191" t="s">
-        <v>34</v>
+      <c r="A43" s="178" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -43921,12 +43647,12 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
-      <c r="D1" s="165" t="s">
-        <v>67</v>
+      <c r="D1" s="160" t="s">
+        <v>66</v>
       </c>
       <c r="E1" s="34"/>
       <c r="F1" s="38"/>
@@ -43934,7 +43660,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="30" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B2" s="35"/>
       <c r="C2" s="35"/>
@@ -43945,7 +43671,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
@@ -43985,7 +43711,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C6" s="3"/>
       <c r="E6" s="1"/>
@@ -43995,10 +43721,10 @@
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D7" s="73">
-        <f>+TB!C27</f>
+        <f>+TB!C18</f>
         <v>2328236</v>
       </c>
       <c r="E7" s="1"/>
@@ -44006,7 +43732,7 @@
       <c r="G7" s="70"/>
     </row>
     <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D8" s="120">
+      <c r="D8" s="116">
         <f>D7</f>
         <v>2328236</v>
       </c>
@@ -44015,7 +43741,7 @@
       <c r="I8" s="73"/>
     </row>
     <row r="9" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="D9" s="125"/>
+      <c r="D9" s="121"/>
       <c r="F9" s="60"/>
       <c r="G9" s="72"/>
       <c r="I9" s="73"/>
@@ -44035,11 +43761,11 @@
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
       <c r="B11" s="2" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="73">
-        <f>TB!B30</f>
+        <f>TB!B20</f>
         <v>1220000</v>
       </c>
       <c r="E11" s="1"/>
@@ -44049,11 +43775,11 @@
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="2" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C12" s="76"/>
-      <c r="D12" s="124" t="e">
-        <f>TB!B29</f>
+      <c r="D12" s="120" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E12" s="1"/>
@@ -44063,12 +43789,12 @@
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
       <c r="B13" s="2" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="C13" s="76"/>
-      <c r="D13" s="124">
-        <f>TB!B34</f>
-        <v>2520</v>
+      <c r="D13" s="120" t="e">
+        <f>TB!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="38"/>
@@ -44077,12 +43803,12 @@
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C14" s="76"/>
-      <c r="D14" s="124">
-        <f>TB!B35</f>
-        <v>630</v>
+      <c r="D14" s="120" t="e">
+        <f>TB!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="38"/>
@@ -44091,11 +43817,11 @@
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C15" s="76"/>
-      <c r="D15" s="124" t="e">
-        <f>+TB!B37</f>
+      <c r="D15" s="120" t="e">
+        <f>+TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E15" s="1"/>
@@ -44105,11 +43831,11 @@
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="C16" s="76"/>
-      <c r="D16" s="124" t="e">
-        <f>+TB!B31+TB!B32</f>
+      <c r="D16" s="120" t="e">
+        <f>+TB!#REF!+TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E16" s="1"/>
@@ -44119,11 +43845,11 @@
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
       <c r="B17" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C17" s="76"/>
-      <c r="D17" s="124" t="e">
-        <f>TB!B39</f>
+      <c r="D17" s="120" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E17" s="1"/>
@@ -44133,11 +43859,11 @@
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
       <c r="B18" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C18" s="76"/>
-      <c r="D18" s="124" t="e">
-        <f>TB!B38</f>
+      <c r="D18" s="120" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E18" s="1"/>
@@ -44147,11 +43873,11 @@
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C19" s="76"/>
-      <c r="D19" s="124" t="e">
-        <f>TB!B33</f>
+      <c r="D19" s="120" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E19" s="1"/>
@@ -44161,11 +43887,11 @@
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C20" s="76"/>
-      <c r="D20" s="124" t="e">
-        <f>TB!B42</f>
+      <c r="D20" s="120" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E20" s="1"/>
@@ -44175,11 +43901,11 @@
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="2" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="C21" s="76"/>
-      <c r="D21" s="124" t="e">
-        <f>TB!B36</f>
+      <c r="D21" s="120" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E21" s="1"/>
@@ -44189,11 +43915,11 @@
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C22" s="76"/>
-      <c r="D22" s="124" t="e">
-        <f>TB!B45</f>
+      <c r="D22" s="120" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E22" s="1"/>
@@ -44203,11 +43929,11 @@
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C23" s="76"/>
-      <c r="D23" s="124" t="e">
-        <f>TB!B44</f>
+      <c r="D23" s="120" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="E23" s="1"/>
@@ -44217,11 +43943,11 @@
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
       <c r="B24" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C24" s="76"/>
-      <c r="D24" s="124">
-        <f>+TB!B47</f>
+      <c r="D24" s="120">
+        <f>+TB!B22</f>
         <v>15000</v>
       </c>
       <c r="E24" s="1"/>
@@ -44231,11 +43957,11 @@
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C25" s="76"/>
-      <c r="D25" s="124">
-        <f>+TB!B48</f>
+      <c r="D25" s="120">
+        <f>+TB!B23</f>
         <v>25000</v>
       </c>
       <c r="E25" s="1"/>
@@ -44243,7 +43969,7 @@
       <c r="G25" s="70"/>
     </row>
     <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D26" s="120" t="e">
+      <c r="D26" s="116" t="e">
         <f>SUM(D11:D25)</f>
         <v>#REF!</v>
       </c>
@@ -44254,7 +43980,7 @@
     <row r="27" spans="1:7" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B27" s="6"/>
       <c r="C27" s="76"/>
-      <c r="D27" s="124"/>
+      <c r="D27" s="120"/>
       <c r="F27" s="38"/>
       <c r="G27" s="66"/>
     </row>
@@ -44263,54 +43989,54 @@
         <v>6</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B29" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C29" s="3"/>
-      <c r="D29" s="125">
-        <f>+TB!B41</f>
-        <v>163480</v>
+      <c r="D29" s="121" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B30" s="1"/>
       <c r="C30" s="3"/>
-      <c r="D30" s="120">
+      <c r="D30" s="116" t="e">
         <f>SUM(D29)</f>
-        <v>163480</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B31" s="1"/>
       <c r="C31" s="3"/>
-      <c r="D31" s="125"/>
+      <c r="D31" s="121"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="9">
         <v>7</v>
       </c>
       <c r="B32" s="30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="65"/>
       <c r="B33" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="D33" s="119">
-        <f>TB!B46</f>
+        <v>103</v>
+      </c>
+      <c r="D33" s="115">
+        <f>TB!B21</f>
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D34" s="121">
+      <c r="D34" s="117">
         <f>+D33</f>
         <v>0</v>
       </c>
@@ -44344,7 +44070,7 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -44354,13 +44080,13 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="165" t="s">
-        <v>68</v>
+      <c r="J1" s="160" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="79" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" s="79"/>
       <c r="C2" s="79"/>
@@ -44374,7 +44100,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="80"/>
-      <c r="B3" s="95"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="80"/>
       <c r="D3" s="80"/>
       <c r="E3" s="80"/>
@@ -44388,21 +44114,21 @@
       <c r="A4" s="36">
         <v>8</v>
       </c>
-      <c r="B4" s="95" t="s">
-        <v>149</v>
+      <c r="B4" s="92" t="s">
+        <v>143</v>
       </c>
       <c r="C4" s="37"/>
       <c r="D4" s="37"/>
     </row>
     <row r="5" spans="1:13" ht="28.8" x14ac:dyDescent="0.35">
       <c r="A5" s="36"/>
-      <c r="B5" s="99" t="s">
-        <v>27</v>
+      <c r="B5" s="96" t="s">
+        <v>26</v>
       </c>
       <c r="C5" s="37"/>
       <c r="D5" s="37"/>
       <c r="E5" s="39" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="F5" s="39"/>
       <c r="G5" s="40" t="s">
@@ -44413,143 +44139,143 @@
       </c>
       <c r="I5" s="42"/>
       <c r="J5" s="43" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="36"/>
       <c r="B6" s="44" t="str">
-        <f>+TB!A9</f>
+        <f>+TB!A8</f>
         <v>Furniture &amp; Fittings</v>
       </c>
       <c r="C6" s="44"/>
       <c r="D6" s="44"/>
-      <c r="E6" s="135">
+      <c r="E6" s="131">
         <v>0</v>
       </c>
-      <c r="F6" s="135"/>
-      <c r="G6" s="135">
-        <f>TB!B9</f>
+      <c r="F6" s="131"/>
+      <c r="G6" s="131">
+        <f>TB!B8</f>
         <v>153700</v>
       </c>
-      <c r="H6" s="122"/>
-      <c r="I6" s="123"/>
-      <c r="J6" s="122">
+      <c r="H6" s="118"/>
+      <c r="I6" s="119"/>
+      <c r="J6" s="118">
         <f>SUM(E6:G6)</f>
         <v>153700</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="36"/>
-      <c r="B7" s="44" t="str">
-        <f>+TB!A10</f>
-        <v>Office Equipment</v>
+      <c r="B7" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C7" s="44"/>
       <c r="D7" s="44"/>
-      <c r="E7" s="135">
+      <c r="E7" s="131">
         <v>0</v>
       </c>
-      <c r="F7" s="135"/>
-      <c r="G7" s="135" t="e">
-        <f>TB!B10</f>
+      <c r="F7" s="131"/>
+      <c r="G7" s="131" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H7" s="122"/>
-      <c r="I7" s="123"/>
-      <c r="J7" s="122" t="e">
+      <c r="H7" s="118"/>
+      <c r="I7" s="119"/>
+      <c r="J7" s="118" t="e">
         <f t="shared" ref="J7:J11" si="0">SUM(E7:G7)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="36"/>
-      <c r="B8" s="44" t="str">
-        <f>+TB!A11</f>
-        <v>Computer &amp; Printers</v>
+      <c r="B8" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="44"/>
-      <c r="E8" s="135">
+      <c r="E8" s="131">
         <v>0</v>
       </c>
-      <c r="F8" s="135"/>
-      <c r="G8" s="135" t="e">
-        <f>TB!B11</f>
+      <c r="F8" s="131"/>
+      <c r="G8" s="131" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H8" s="122"/>
-      <c r="I8" s="123"/>
-      <c r="J8" s="122" t="e">
+      <c r="H8" s="118"/>
+      <c r="I8" s="119"/>
+      <c r="J8" s="118" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="36"/>
-      <c r="B9" s="44" t="str">
-        <f>+TB!A12</f>
-        <v>Furniture &amp; Fittings</v>
+      <c r="B9" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C9" s="44"/>
       <c r="D9" s="44"/>
-      <c r="E9" s="135">
+      <c r="E9" s="131">
         <v>0</v>
       </c>
-      <c r="F9" s="135"/>
-      <c r="G9" s="135" t="e">
-        <f>TB!B12</f>
+      <c r="F9" s="131"/>
+      <c r="G9" s="131" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H9" s="122"/>
-      <c r="I9" s="123"/>
-      <c r="J9" s="122" t="e">
+      <c r="H9" s="118"/>
+      <c r="I9" s="119"/>
+      <c r="J9" s="118" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="36"/>
-      <c r="B10" s="44" t="str">
-        <f>+TB!A13</f>
-        <v>Telephone</v>
+      <c r="B10" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="44"/>
-      <c r="E10" s="135">
+      <c r="E10" s="131">
         <v>0</v>
       </c>
-      <c r="F10" s="135"/>
-      <c r="G10" s="135" t="e">
-        <f>TB!B13</f>
+      <c r="F10" s="131"/>
+      <c r="G10" s="131" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H10" s="122"/>
-      <c r="I10" s="123"/>
-      <c r="J10" s="122" t="e">
+      <c r="H10" s="118"/>
+      <c r="I10" s="119"/>
+      <c r="J10" s="118" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="36"/>
-      <c r="B11" s="44" t="str">
-        <f>+TB!A14</f>
-        <v>CCTV Camera</v>
+      <c r="B11" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="C11" s="44"/>
       <c r="D11" s="44"/>
-      <c r="E11" s="135">
+      <c r="E11" s="131">
         <v>0</v>
       </c>
-      <c r="F11" s="135"/>
-      <c r="G11" s="135" t="e">
-        <f>TB!B14</f>
+      <c r="F11" s="131"/>
+      <c r="G11" s="131" t="e">
+        <f>TB!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H11" s="122"/>
-      <c r="I11" s="123"/>
-      <c r="J11" s="122" t="e">
+      <c r="H11" s="118"/>
+      <c r="I11" s="119"/>
+      <c r="J11" s="118" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
@@ -44559,18 +44285,18 @@
       <c r="B12" s="44"/>
       <c r="C12" s="44"/>
       <c r="D12" s="44"/>
-      <c r="E12" s="136">
+      <c r="E12" s="132">
         <f>SUM(E6:E11)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="135"/>
-      <c r="G12" s="136" t="e">
+      <c r="F12" s="131"/>
+      <c r="G12" s="132" t="e">
         <f>SUM(G6:G11)</f>
         <v>#REF!</v>
       </c>
-      <c r="H12" s="122"/>
-      <c r="I12" s="123"/>
-      <c r="J12" s="136" t="e">
+      <c r="H12" s="118"/>
+      <c r="I12" s="119"/>
+      <c r="J12" s="132" t="e">
         <f>SUM(J6:J11)</f>
         <v>#REF!</v>
       </c>
@@ -44602,12 +44328,12 @@
     <row r="15" spans="1:13" ht="28.8" x14ac:dyDescent="0.35">
       <c r="A15" s="36"/>
       <c r="B15" s="36" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C15" s="37"/>
       <c r="D15" s="37"/>
       <c r="E15" s="39" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="F15" s="39"/>
       <c r="G15" s="39" t="s">
@@ -44618,7 +44344,7 @@
       </c>
       <c r="I15" s="42"/>
       <c r="J15" s="43" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="M15" s="49"/>
     </row>
@@ -44630,132 +44356,132 @@
       </c>
       <c r="C16" s="44"/>
       <c r="D16" s="44"/>
-      <c r="E16" s="135">
+      <c r="E16" s="131">
         <v>0</v>
       </c>
-      <c r="F16" s="135"/>
-      <c r="G16" s="122">
+      <c r="F16" s="131"/>
+      <c r="G16" s="118">
         <f>PPE!G4</f>
         <v>28887.178082191782</v>
       </c>
-      <c r="H16" s="122"/>
-      <c r="I16" s="123"/>
-      <c r="J16" s="149">
+      <c r="H16" s="118"/>
+      <c r="I16" s="119"/>
+      <c r="J16" s="144">
         <f>SUM(E16:G16)</f>
         <v>28887.178082191782</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="50"/>
-      <c r="B17" s="44" t="str">
+      <c r="B17" s="44" t="e">
         <f t="shared" si="1"/>
-        <v>Office Equipment</v>
+        <v>#REF!</v>
       </c>
       <c r="C17" s="44"/>
       <c r="D17" s="44"/>
-      <c r="E17" s="135">
+      <c r="E17" s="131">
         <v>0</v>
       </c>
-      <c r="F17" s="135"/>
-      <c r="G17" s="122" t="e">
+      <c r="F17" s="131"/>
+      <c r="G17" s="118" t="e">
         <f>PPE!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H17" s="122"/>
-      <c r="I17" s="123"/>
-      <c r="J17" s="149" t="e">
+      <c r="H17" s="118"/>
+      <c r="I17" s="119"/>
+      <c r="J17" s="144" t="e">
         <f t="shared" ref="J17:J21" si="2">SUM(E17:G17)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="50"/>
-      <c r="B18" s="44" t="str">
+      <c r="B18" s="44" t="e">
         <f t="shared" si="1"/>
-        <v>Computer &amp; Printers</v>
+        <v>#REF!</v>
       </c>
       <c r="C18" s="44"/>
       <c r="D18" s="44"/>
-      <c r="E18" s="135">
+      <c r="E18" s="131">
         <v>0</v>
       </c>
-      <c r="F18" s="135"/>
-      <c r="G18" s="122" t="e">
+      <c r="F18" s="131"/>
+      <c r="G18" s="118" t="e">
         <f>PPE!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H18" s="122"/>
-      <c r="I18" s="123"/>
-      <c r="J18" s="149" t="e">
+      <c r="H18" s="118"/>
+      <c r="I18" s="119"/>
+      <c r="J18" s="144" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="50"/>
-      <c r="B19" s="44" t="str">
+      <c r="B19" s="44" t="e">
         <f t="shared" si="1"/>
-        <v>Furniture &amp; Fittings</v>
+        <v>#REF!</v>
       </c>
       <c r="C19" s="44"/>
       <c r="D19" s="44"/>
-      <c r="E19" s="135">
+      <c r="E19" s="131">
         <v>0</v>
       </c>
-      <c r="F19" s="135"/>
-      <c r="G19" s="122" t="e">
+      <c r="F19" s="131"/>
+      <c r="G19" s="118" t="e">
         <f>PPE!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H19" s="122"/>
-      <c r="I19" s="123"/>
-      <c r="J19" s="149" t="e">
+      <c r="H19" s="118"/>
+      <c r="I19" s="119"/>
+      <c r="J19" s="144" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="50"/>
-      <c r="B20" s="44" t="str">
+      <c r="B20" s="44" t="e">
         <f t="shared" si="1"/>
-        <v>Telephone</v>
+        <v>#REF!</v>
       </c>
       <c r="C20" s="44"/>
       <c r="D20" s="44"/>
-      <c r="E20" s="135">
+      <c r="E20" s="131">
         <v>0</v>
       </c>
-      <c r="F20" s="135"/>
-      <c r="G20" s="122" t="e">
+      <c r="F20" s="131"/>
+      <c r="G20" s="118" t="e">
         <f>PPE!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H20" s="122"/>
-      <c r="I20" s="123"/>
-      <c r="J20" s="149" t="e">
+      <c r="H20" s="118"/>
+      <c r="I20" s="119"/>
+      <c r="J20" s="144" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="50"/>
-      <c r="B21" s="44" t="str">
+      <c r="B21" s="44" t="e">
         <f t="shared" si="1"/>
-        <v>CCTV Camera</v>
+        <v>#REF!</v>
       </c>
       <c r="C21" s="44"/>
       <c r="D21" s="44"/>
-      <c r="E21" s="135">
+      <c r="E21" s="131">
         <v>0</v>
       </c>
-      <c r="F21" s="135"/>
-      <c r="G21" s="122" t="e">
+      <c r="F21" s="131"/>
+      <c r="G21" s="118" t="e">
         <f>PPE!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="H21" s="122"/>
-      <c r="I21" s="123"/>
-      <c r="J21" s="149" t="e">
+      <c r="H21" s="118"/>
+      <c r="I21" s="119"/>
+      <c r="J21" s="144" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
@@ -44765,18 +44491,18 @@
       <c r="B22" s="44"/>
       <c r="C22" s="44"/>
       <c r="D22" s="44"/>
-      <c r="E22" s="136">
+      <c r="E22" s="132">
         <f>SUM(E16:E21)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="135"/>
-      <c r="G22" s="196" t="e">
+      <c r="F22" s="131"/>
+      <c r="G22" s="182" t="e">
         <f>SUM(G16:G21)</f>
         <v>#REF!</v>
       </c>
-      <c r="H22" s="122"/>
-      <c r="I22" s="123"/>
-      <c r="J22" s="136" t="e">
+      <c r="H22" s="118"/>
+      <c r="I22" s="119"/>
+      <c r="J22" s="132" t="e">
         <f>SUM(J16:J21)</f>
         <v>#REF!</v>
       </c>
@@ -44795,11 +44521,11 @@
     </row>
     <row r="24" spans="1:10" ht="28.8" x14ac:dyDescent="0.35">
       <c r="A24" s="2"/>
-      <c r="B24" s="99" t="s">
-        <v>81</v>
-      </c>
-      <c r="J24" s="93" t="s">
-        <v>140</v>
+      <c r="B24" s="96" t="s">
+        <v>80</v>
+      </c>
+      <c r="J24" s="90" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -44815,9 +44541,9 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
-      <c r="B26" s="44" t="str">
+      <c r="B26" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>Office Equipment</v>
+        <v>#REF!</v>
       </c>
       <c r="J26" s="74" t="e">
         <f t="shared" si="4"/>
@@ -44826,9 +44552,9 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="2"/>
-      <c r="B27" s="44" t="str">
+      <c r="B27" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>Computer &amp; Printers</v>
+        <v>#REF!</v>
       </c>
       <c r="J27" s="74" t="e">
         <f t="shared" si="4"/>
@@ -44837,9 +44563,9 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="2"/>
-      <c r="B28" s="44" t="str">
+      <c r="B28" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>Furniture &amp; Fittings</v>
+        <v>#REF!</v>
       </c>
       <c r="J28" s="74" t="e">
         <f t="shared" si="4"/>
@@ -44848,9 +44574,9 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="2"/>
-      <c r="B29" s="44" t="str">
+      <c r="B29" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>Telephone</v>
+        <v>#REF!</v>
       </c>
       <c r="J29" s="74" t="e">
         <f t="shared" si="4"/>
@@ -44859,9 +44585,9 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="2"/>
-      <c r="B30" s="44" t="str">
+      <c r="B30" s="44" t="e">
         <f t="shared" si="3"/>
-        <v>CCTV Camera</v>
+        <v>#REF!</v>
       </c>
       <c r="J30" s="74" t="e">
         <f t="shared" si="4"/>
@@ -44870,7 +44596,7 @@
     </row>
     <row r="31" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="2"/>
-      <c r="J31" s="150" t="e">
+      <c r="J31" s="145" t="e">
         <f>SUM(J25:J30)</f>
         <v>#REF!</v>
       </c>

</xml_diff>

<commit_message>
feat: implement Trial Balance table and integrate with Financial Reports page
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B53AE7-D416-4887-994D-BE21CF413D5F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4E5BC4-0FC5-4D66-9138-329178E8ABA3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="192">
   <si>
     <t>STATEMENT OF FINANCIAL POSITION</t>
   </si>
@@ -522,9 +522,6 @@
     <t>Commission Income</t>
   </si>
   <si>
-    <t>N K R S Lanka Capuital Pvt Ltd</t>
-  </si>
-  <si>
     <t>N K R S LANKA CAPITAL (PRIVATE) LIMITED</t>
   </si>
   <si>
@@ -646,6 +643,12 @@
   </si>
   <si>
     <t>Expenses</t>
+  </si>
+  <si>
+    <t>Accounts</t>
+  </si>
+  <si>
+    <t>N K R S Lanka Capital Pvt Ltd</t>
   </si>
 </sst>
 </file>
@@ -936,7 +939,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="237">
+  <cellXfs count="236">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1383,12 +1386,6 @@
     </xf>
     <xf numFmtId="43" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="166" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1422,6 +1419,9 @@
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="23">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1943,7 +1943,7 @@
         <v>117</v>
       </c>
       <c r="F3" s="138" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G3" s="138" t="s">
         <v>118</v>
@@ -2020,7 +2020,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2253,7 +2253,7 @@
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="114" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C20" s="58"/>
       <c r="D20" s="58"/>
@@ -2267,7 +2267,7 @@
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="114" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C21" s="58"/>
       <c r="D21" s="58"/>
@@ -2485,7 +2485,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="30"/>
       <c r="F1" s="93"/>
@@ -2508,7 +2508,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="30" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="E17" s="101"/>
       <c r="H17" s="136" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
@@ -3013,12 +3013,12 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="198" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="193" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H46" s="173">
         <v>0</v>
@@ -3026,7 +3026,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="193" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H47" s="217" t="e">
         <f>-H15</f>
@@ -3045,12 +3045,12 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="193" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="193" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H51" s="173">
         <v>0</v>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="193" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H52" s="173">
         <v>0</v>
@@ -3066,7 +3066,7 @@
     </row>
     <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="193" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H53" s="218" t="e">
         <f>SUM(H48:H52)</f>
@@ -3093,7 +3093,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="221" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -3109,13 +3109,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="221" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B4" s="165"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B5" s="170">
         <v>99975</v>
@@ -3132,7 +3132,7 @@
         <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -3143,22 +3143,22 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="221" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B11" s="165"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>156</v>
+      </c>
+      <c r="B12" t="s">
         <v>157</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>158</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>159</v>
-      </c>
-      <c r="D12" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -3221,209 +3221,211 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="222" t="s">
-        <v>149</v>
-      </c>
-      <c r="B1" s="222"/>
-      <c r="C1" s="222"/>
+      <c r="A1" s="235" t="s">
+        <v>191</v>
+      </c>
+      <c r="B1" s="235"/>
+      <c r="C1" s="235"/>
     </row>
     <row r="2" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="222" t="s">
+      <c r="A2" s="235" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="222"/>
-      <c r="C2" s="222"/>
+      <c r="B2" s="235"/>
+      <c r="C2" s="235"/>
     </row>
     <row r="3" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="222" t="s">
+      <c r="A3" s="235" t="s">
         <v>108</v>
       </c>
-      <c r="B3" s="222"/>
-      <c r="C3" s="222"/>
+      <c r="B3" s="235"/>
+      <c r="C3" s="235"/>
     </row>
     <row r="4" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A4" s="223"/>
-      <c r="B4" s="224" t="s">
+      <c r="A4" s="230" t="s">
+        <v>190</v>
+      </c>
+      <c r="B4" s="222" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="225" t="s">
+      <c r="C4" s="223" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A5" s="226" t="s">
+      <c r="A5" s="224" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="227"/>
-      <c r="C5" s="227"/>
+      <c r="B5" s="225"/>
+      <c r="C5" s="225"/>
     </row>
     <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A6" s="228" t="s">
+      <c r="A6" s="226" t="s">
         <v>120</v>
       </c>
-      <c r="B6" s="234">
+      <c r="B6" s="232">
         <v>12560</v>
       </c>
-      <c r="C6" s="227"/>
+      <c r="C6" s="225"/>
     </row>
     <row r="7" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A7" s="226" t="s">
+      <c r="A7" s="224" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="227"/>
-      <c r="C7" s="227"/>
+      <c r="B7" s="225"/>
+      <c r="C7" s="225"/>
       <c r="J7" s="162"/>
     </row>
     <row r="8" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A8" s="228" t="s">
+      <c r="A8" s="226" t="s">
         <v>110</v>
       </c>
-      <c r="B8" s="227">
+      <c r="B8" s="225">
         <f>+PPE!D4</f>
         <v>153700</v>
       </c>
-      <c r="C8" s="227"/>
+      <c r="C8" s="225"/>
       <c r="J8" s="162"/>
     </row>
     <row r="9" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A9" s="228" t="s">
+      <c r="A9" s="226" t="s">
         <v>122</v>
       </c>
-      <c r="B9" s="227"/>
-      <c r="C9" s="227">
+      <c r="B9" s="225"/>
+      <c r="C9" s="225">
         <f>+PPE!G5</f>
         <v>28887.178082191782</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A10" s="226" t="s">
-        <v>188</v>
-      </c>
-      <c r="B10" s="227"/>
-      <c r="C10" s="227"/>
+      <c r="A10" s="224" t="s">
+        <v>187</v>
+      </c>
+      <c r="B10" s="225"/>
+      <c r="C10" s="225"/>
     </row>
     <row r="11" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="228" t="s">
+      <c r="A11" s="226" t="s">
         <v>121</v>
       </c>
-      <c r="B11" s="227"/>
-      <c r="C11" s="227">
+      <c r="B11" s="225"/>
+      <c r="C11" s="225">
         <f>+B22</f>
         <v>15000</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A12" s="228" t="s">
+      <c r="A12" s="226" t="s">
         <v>100</v>
       </c>
-      <c r="B12" s="227"/>
-      <c r="C12" s="227">
+      <c r="B12" s="225"/>
+      <c r="C12" s="225">
         <f>+B23</f>
         <v>25000</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" s="221" t="s">
-        <v>189</v>
-      </c>
-      <c r="B13" s="229"/>
-      <c r="C13" s="230"/>
+        <v>188</v>
+      </c>
+      <c r="B13" s="227"/>
+      <c r="C13" s="228"/>
     </row>
     <row r="14" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A14" s="228" t="s">
+      <c r="A14" s="226" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="227"/>
-      <c r="C14" s="227">
+      <c r="B14" s="225"/>
+      <c r="C14" s="225">
         <f>1000*6</f>
         <v>6000</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A15" s="228" t="s">
-        <v>170</v>
-      </c>
-      <c r="B15" s="227"/>
-      <c r="C15" s="227">
+      <c r="A15" s="226" t="s">
+        <v>169</v>
+      </c>
+      <c r="B15" s="225"/>
+      <c r="C15" s="225">
         <v>1000000</v>
       </c>
     </row>
     <row r="16" spans="1:10" s="213" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A16" s="226" t="s">
-        <v>155</v>
-      </c>
-      <c r="B16" s="227"/>
-      <c r="C16" s="230"/>
+      <c r="A16" s="224" t="s">
+        <v>154</v>
+      </c>
+      <c r="B16" s="225"/>
+      <c r="C16" s="228"/>
     </row>
     <row r="17" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="231" t="s">
-        <v>171</v>
-      </c>
-      <c r="B17" s="235">
+      <c r="A17" s="229" t="s">
+        <v>170</v>
+      </c>
+      <c r="B17" s="233">
         <v>112919.5</v>
       </c>
-      <c r="C17" s="227"/>
+      <c r="C17" s="225"/>
     </row>
     <row r="18" spans="1:3" s="213" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="228" t="s">
+      <c r="A18" s="226" t="s">
         <v>107</v>
       </c>
-      <c r="B18" s="227"/>
-      <c r="C18" s="236">
+      <c r="B18" s="225"/>
+      <c r="C18" s="234">
         <f>+Working!B2</f>
         <v>2328236</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" s="221" t="s">
-        <v>190</v>
-      </c>
-      <c r="B19" s="227"/>
-      <c r="C19" s="227"/>
+        <v>189</v>
+      </c>
+      <c r="B19" s="225"/>
+      <c r="C19" s="225"/>
     </row>
     <row r="20" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A20" s="228" t="s">
-        <v>166</v>
-      </c>
-      <c r="B20" s="227">
+      <c r="A20" s="226" t="s">
+        <v>165</v>
+      </c>
+      <c r="B20" s="225">
         <v>1220000</v>
       </c>
-      <c r="C20" s="227"/>
+      <c r="C20" s="225"/>
     </row>
     <row r="21" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A21" s="228" t="s">
+      <c r="A21" s="226" t="s">
         <v>142</v>
       </c>
-      <c r="B21" s="227"/>
-      <c r="C21" s="227"/>
+      <c r="B21" s="225"/>
+      <c r="C21" s="225"/>
     </row>
     <row r="22" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A22" s="228" t="s">
+      <c r="A22" s="226" t="s">
         <v>121</v>
       </c>
-      <c r="B22" s="227">
+      <c r="B22" s="225">
         <v>15000</v>
       </c>
-      <c r="C22" s="227"/>
+      <c r="C22" s="225"/>
     </row>
     <row r="23" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A23" s="228" t="s">
+      <c r="A23" s="226" t="s">
         <v>100</v>
       </c>
-      <c r="B23" s="227">
+      <c r="B23" s="225">
         <v>25000</v>
       </c>
-      <c r="C23" s="227"/>
+      <c r="C23" s="225"/>
     </row>
     <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="232" t="s">
+      <c r="A24" s="230" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="233">
+      <c r="B24" s="231">
         <f>SUM(B5:B23)</f>
         <v>1539179.5</v>
       </c>
-      <c r="C24" s="233">
+      <c r="C24" s="231">
         <f>SUM(C5:C23)</f>
         <v>3403123.1780821919</v>
       </c>
@@ -3463,7 +3465,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3587,7 +3589,7 @@
     </row>
     <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D16" s="124" t="e">
         <f>SUM(D12:D14)</f>
@@ -3643,7 +3645,7 @@
   <sheetData>
     <row r="1" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4734,7 +4736,7 @@
     </row>
     <row r="12" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A12" s="150" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B12" s="150"/>
       <c r="C12" s="219"/>
@@ -41012,7 +41014,7 @@
     </row>
     <row r="50" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A50" s="28" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B50" s="18"/>
       <c r="C50" s="18"/>
@@ -42019,7 +42021,7 @@
     </row>
     <row r="51" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A51" s="28" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B51" s="18"/>
       <c r="C51" s="18"/>
@@ -43050,7 +43052,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -43175,7 +43177,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E11" s="62">
         <v>0</v>
@@ -43295,7 +43297,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="179" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E1" s="179"/>
       <c r="F1" s="179"/>
@@ -43388,7 +43390,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B12" s="181" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C12" s="181"/>
       <c r="D12" s="181"/>
@@ -43400,7 +43402,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B13" s="181" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C13" s="181"/>
       <c r="D13" s="181"/>
@@ -43647,7 +43649,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
@@ -43671,7 +43673,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
@@ -43761,7 +43763,7 @@
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
       <c r="B11" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="73">
@@ -43789,7 +43791,7 @@
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
       <c r="B13" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C13" s="76"/>
       <c r="D13" s="120" t="e">
@@ -43803,7 +43805,7 @@
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C14" s="76"/>
       <c r="D14" s="120" t="e">
@@ -43831,7 +43833,7 @@
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C16" s="76"/>
       <c r="D16" s="120" t="e">
@@ -43887,7 +43889,7 @@
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C20" s="76"/>
       <c r="D20" s="120" t="e">
@@ -43901,7 +43903,7 @@
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C21" s="76"/>
       <c r="D21" s="120" t="e">
@@ -43996,7 +43998,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B29" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="121" t="e">
@@ -44070,7 +44072,7 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>

</xml_diff>

<commit_message>
feat: enhance PPE worksheet generation with improved styling and formula handling
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4E5BC4-0FC5-4D66-9138-329178E8ABA3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92A19933-8BDD-4631-9DA5-FDA53D42FFED}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPE" sheetId="24" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="192">
   <si>
     <t>STATEMENT OF FINANCIAL POSITION</t>
   </si>
@@ -661,7 +661,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -826,6 +826,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -939,7 +952,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="236">
+  <cellXfs count="240">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1217,27 +1230,6 @@
     <xf numFmtId="166" fontId="12" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="10" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="10" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="10" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
@@ -1284,16 +1276,10 @@
     </xf>
     <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="6" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1421,6 +1407,43 @@
     <xf numFmtId="166" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="17" fontId="26" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="6" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="26" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="26" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="26" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="25" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="23">
@@ -1906,92 +1929,94 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.109375" style="44" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.77734375" style="44" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" style="44" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" style="44" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" style="44" customWidth="1"/>
-    <col min="6" max="6" width="12" style="44" customWidth="1"/>
-    <col min="7" max="7" width="12.5546875" style="44" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="44"/>
-    <col min="9" max="9" width="10.6640625" style="44" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="44"/>
+    <col min="1" max="1" width="19.109375" style="228" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" style="228" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" style="228" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" style="228" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" style="228" customWidth="1"/>
+    <col min="6" max="6" width="12" style="228" customWidth="1"/>
+    <col min="7" max="7" width="12.5546875" style="228" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" style="228"/>
+    <col min="9" max="9" width="10.6640625" style="228" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="228"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="227" t="s">
         <v>114</v>
       </c>
-      <c r="C1" s="37"/>
+      <c r="C1" s="227"/>
     </row>
-    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="137" t="s">
+    <row r="3" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="229" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="138" t="s">
+      <c r="B3" s="230" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="137" t="s">
+      <c r="C3" s="229" t="s">
         <v>119</v>
       </c>
-      <c r="D3" s="139" t="s">
+      <c r="D3" s="231" t="s">
         <v>109</v>
       </c>
-      <c r="E3" s="138" t="s">
+      <c r="E3" s="230" t="s">
         <v>117</v>
       </c>
-      <c r="F3" s="138" t="s">
+      <c r="F3" s="230" t="s">
         <v>162</v>
       </c>
-      <c r="G3" s="138" t="s">
+      <c r="G3" s="230" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="232" t="s">
         <v>110</v>
       </c>
-      <c r="B4" s="140">
+      <c r="B4" s="233">
         <v>45385</v>
       </c>
-      <c r="C4" s="171">
+      <c r="C4" s="234">
         <v>5</v>
       </c>
-      <c r="D4" s="141">
+      <c r="D4" s="235">
         <v>153700</v>
       </c>
-      <c r="E4" s="140">
+      <c r="E4" s="233">
         <v>45728</v>
       </c>
-      <c r="F4" s="141">
+      <c r="F4" s="235">
         <f t="shared" ref="F4" si="0">E4-B4</f>
         <v>343</v>
       </c>
-      <c r="G4" s="142">
+      <c r="G4" s="236">
         <f>(D4/C4)*(F4/365)</f>
         <v>28887.178082191782</v>
       </c>
-      <c r="I4" s="166"/>
+      <c r="I4" s="237"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="139"/>
-      <c r="B5" s="139"/>
-      <c r="C5" s="139"/>
-      <c r="D5" s="143">
+      <c r="A5" s="231" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="238"/>
+      <c r="C5" s="238"/>
+      <c r="D5" s="239">
         <f>SUM(D4:D4)</f>
         <v>153700</v>
       </c>
-      <c r="E5" s="139"/>
-      <c r="F5" s="139"/>
-      <c r="G5" s="143">
+      <c r="E5" s="238"/>
+      <c r="F5" s="238"/>
+      <c r="G5" s="239">
         <f>SUM(G4:G4)</f>
         <v>28887.178082191782</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D7" s="166"/>
+      <c r="D7" s="237"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2030,7 +2055,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="160" t="s">
+      <c r="J1" s="153" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2490,7 +2515,7 @@
       <c r="B1" s="30"/>
       <c r="F1" s="93"/>
       <c r="G1" s="94"/>
-      <c r="H1" s="160" t="s">
+      <c r="H1" s="153" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2564,11 +2589,11 @@
         <v>129</v>
       </c>
       <c r="D11" s="99"/>
-      <c r="F11" s="200" t="e">
+      <c r="F11" s="191" t="e">
         <f>'P10'!G22</f>
         <v>#REF!</v>
       </c>
-      <c r="H11" s="214" t="e">
+      <c r="H11" s="205" t="e">
         <f>+F11</f>
         <v>#REF!</v>
       </c>
@@ -2795,208 +2820,208 @@
         <f>+'P10'!B6</f>
         <v>Furniture &amp; Fittings</v>
       </c>
-      <c r="B35" s="176">
+      <c r="B35" s="167">
         <f>+'P10'!G6</f>
         <v>153700</v>
       </c>
       <c r="C35" s="65">
         <v>5</v>
       </c>
-      <c r="D35" s="147">
+      <c r="D35" s="140">
         <v>0</v>
       </c>
-      <c r="E35" s="146">
+      <c r="E35" s="139">
         <f>B35/C35</f>
         <v>30740</v>
       </c>
-      <c r="F35" s="146">
+      <c r="F35" s="139">
         <f>D35+E35</f>
         <v>30740</v>
       </c>
       <c r="G35" s="111"/>
-      <c r="H35" s="149">
+      <c r="H35" s="142">
         <f>B35-F35</f>
         <v>122960</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" s="201" t="e">
+      <c r="A36" s="192" t="e">
         <f>+'P10'!B7</f>
         <v>#REF!</v>
       </c>
-      <c r="B36" s="176" t="e">
+      <c r="B36" s="167" t="e">
         <f>+'P10'!G7</f>
         <v>#REF!</v>
       </c>
       <c r="C36" s="65">
         <v>5</v>
       </c>
-      <c r="D36" s="210">
+      <c r="D36" s="201">
         <v>0</v>
       </c>
-      <c r="E36" s="208" t="e">
+      <c r="E36" s="199" t="e">
         <f t="shared" ref="E36:E40" si="0">B36/C36</f>
         <v>#REF!</v>
       </c>
-      <c r="F36" s="208" t="e">
+      <c r="F36" s="199" t="e">
         <f t="shared" ref="F36:F40" si="1">D36+E36</f>
         <v>#REF!</v>
       </c>
       <c r="G36" s="111"/>
-      <c r="H36" s="212" t="e">
+      <c r="H36" s="203" t="e">
         <f t="shared" ref="H36:H40" si="2">B36-F36</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" s="201" t="e">
+      <c r="A37" s="192" t="e">
         <f>+'P10'!B8</f>
         <v>#REF!</v>
       </c>
-      <c r="B37" s="176" t="e">
+      <c r="B37" s="167" t="e">
         <f>+'P10'!G8</f>
         <v>#REF!</v>
       </c>
       <c r="C37" s="65">
         <v>5</v>
       </c>
-      <c r="D37" s="210">
+      <c r="D37" s="201">
         <v>0</v>
       </c>
-      <c r="E37" s="208" t="e">
+      <c r="E37" s="199" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F37" s="208" t="e">
+      <c r="F37" s="199" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
       <c r="G37" s="111"/>
-      <c r="H37" s="212" t="e">
+      <c r="H37" s="203" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="191" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="201" t="e">
+    <row r="38" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="192" t="e">
         <f>+'P10'!B9</f>
         <v>#REF!</v>
       </c>
-      <c r="B38" s="176" t="e">
+      <c r="B38" s="167" t="e">
         <f>+'P10'!G9</f>
         <v>#REF!</v>
       </c>
-      <c r="C38" s="197">
+      <c r="C38" s="188">
         <v>5</v>
       </c>
-      <c r="D38" s="210">
+      <c r="D38" s="201">
         <v>0</v>
       </c>
-      <c r="E38" s="208" t="e">
+      <c r="E38" s="199" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F38" s="208" t="e">
+      <c r="F38" s="199" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G38" s="202"/>
-      <c r="H38" s="212" t="e">
+      <c r="G38" s="193"/>
+      <c r="H38" s="203" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="39" spans="1:8" s="191" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="201" t="e">
+    <row r="39" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="192" t="e">
         <f>+'P10'!B10</f>
         <v>#REF!</v>
       </c>
-      <c r="B39" s="176" t="e">
+      <c r="B39" s="167" t="e">
         <f>+'P10'!G10</f>
         <v>#REF!</v>
       </c>
-      <c r="C39" s="197">
+      <c r="C39" s="188">
         <v>5</v>
       </c>
-      <c r="D39" s="210">
+      <c r="D39" s="201">
         <v>0</v>
       </c>
-      <c r="E39" s="208" t="e">
+      <c r="E39" s="199" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F39" s="208" t="e">
+      <c r="F39" s="199" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G39" s="202"/>
-      <c r="H39" s="212" t="e">
+      <c r="G39" s="193"/>
+      <c r="H39" s="203" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="40" spans="1:8" s="191" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="201" t="e">
+    <row r="40" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="192" t="e">
         <f>+'P10'!B11</f>
         <v>#REF!</v>
       </c>
-      <c r="B40" s="176" t="e">
+      <c r="B40" s="167" t="e">
         <f>+'P10'!G11</f>
         <v>#REF!</v>
       </c>
-      <c r="C40" s="197">
+      <c r="C40" s="188">
         <v>5</v>
       </c>
-      <c r="D40" s="210">
+      <c r="D40" s="201">
         <v>0</v>
       </c>
-      <c r="E40" s="208" t="e">
+      <c r="E40" s="199" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F40" s="208" t="e">
+      <c r="F40" s="199" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G40" s="202"/>
-      <c r="H40" s="212" t="e">
+      <c r="G40" s="193"/>
+      <c r="H40" s="203" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="41" spans="1:8" s="191" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="201"/>
-      <c r="B41" s="209"/>
-      <c r="C41" s="197"/>
-      <c r="D41" s="210"/>
-      <c r="E41" s="208"/>
-      <c r="F41" s="208"/>
-      <c r="G41" s="202"/>
-      <c r="H41" s="212"/>
+    <row r="41" spans="1:8" s="182" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="192"/>
+      <c r="B41" s="200"/>
+      <c r="C41" s="188"/>
+      <c r="D41" s="201"/>
+      <c r="E41" s="199"/>
+      <c r="F41" s="199"/>
+      <c r="G41" s="193"/>
+      <c r="H41" s="203"/>
     </row>
     <row r="42" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="B42" s="148" t="e">
+      <c r="B42" s="141" t="e">
         <f>SUM(B35:B40)</f>
         <v>#REF!</v>
       </c>
       <c r="C42" s="113"/>
-      <c r="D42" s="211">
+      <c r="D42" s="202">
         <f>SUM(D35:D40)</f>
         <v>0</v>
       </c>
-      <c r="E42" s="211" t="e">
+      <c r="E42" s="202" t="e">
         <f t="shared" ref="E42:H42" si="3">SUM(E35:E40)</f>
         <v>#REF!</v>
       </c>
-      <c r="F42" s="211" t="e">
+      <c r="F42" s="202" t="e">
         <f t="shared" si="3"/>
         <v>#REF!</v>
       </c>
       <c r="G42" s="113"/>
-      <c r="H42" s="211" t="e">
+      <c r="H42" s="202" t="e">
         <f t="shared" si="3"/>
         <v>#REF!</v>
       </c>
@@ -3012,63 +3037,63 @@
       <c r="H43" s="112"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" s="198" t="s">
+      <c r="A45" s="189" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A46" s="193" t="s">
+      <c r="A46" s="184" t="s">
         <v>175</v>
       </c>
-      <c r="H46" s="173">
+      <c r="H46" s="164">
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A47" s="193" t="s">
+      <c r="A47" s="184" t="s">
         <v>176</v>
       </c>
-      <c r="H47" s="217" t="e">
+      <c r="H47" s="208" t="e">
         <f>-H15</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A48" s="193"/>
-      <c r="H48" s="173" t="e">
+      <c r="A48" s="184"/>
+      <c r="H48" s="164" t="e">
         <f>SUM(H46:H47)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" s="193"/>
+      <c r="A49" s="184"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A50" s="193" t="s">
+      <c r="A50" s="184" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A51" s="193" t="s">
+      <c r="A51" s="184" t="s">
         <v>178</v>
       </c>
-      <c r="H51" s="173">
+      <c r="H51" s="164">
         <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="193" t="s">
+      <c r="A52" s="184" t="s">
         <v>179</v>
       </c>
-      <c r="H52" s="173">
+      <c r="H52" s="164">
         <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A53" s="193" t="s">
+      <c r="A53" s="184" t="s">
         <v>180</v>
       </c>
-      <c r="H53" s="218" t="e">
+      <c r="H53" s="209" t="e">
         <f>SUM(H48:H52)</f>
         <v>#REF!</v>
       </c>
@@ -3092,7 +3117,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="221" t="s">
+      <c r="A1" s="212" t="s">
         <v>154</v>
       </c>
     </row>
@@ -3100,35 +3125,35 @@
       <c r="A2" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="165">
+      <c r="B2" s="158">
         <v>2328236</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="165"/>
+      <c r="B3" s="158"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="221" t="s">
+      <c r="A4" s="212" t="s">
         <v>185</v>
       </c>
-      <c r="B4" s="165"/>
+      <c r="B4" s="158"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>151</v>
       </c>
-      <c r="B5" s="170">
+      <c r="B5" s="162">
         <v>99975</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="165"/>
+      <c r="B6" s="158"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="165"/>
+      <c r="B7" s="158"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="221" t="s">
+      <c r="A8" s="212" t="s">
         <v>19</v>
       </c>
       <c r="C8" t="s">
@@ -3136,16 +3161,16 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B9" s="165"/>
+      <c r="B9" s="158"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="165"/>
+      <c r="B10" s="158"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="221" t="s">
+      <c r="A11" s="212" t="s">
         <v>186</v>
       </c>
-      <c r="B11" s="165"/>
+      <c r="B11" s="158"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -3162,17 +3187,17 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="167">
+      <c r="A13" s="159">
         <v>45597</v>
       </c>
-      <c r="B13" s="165">
+      <c r="B13" s="158">
         <v>4200</v>
       </c>
-      <c r="C13" s="165">
+      <c r="C13" s="158">
         <f>B13*12/20</f>
         <v>2520</v>
       </c>
-      <c r="D13" s="165">
+      <c r="D13" s="158">
         <f>C13*3/12</f>
         <v>630</v>
       </c>
@@ -3181,23 +3206,23 @@
       <c r="A14" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="168">
+      <c r="B14" s="160">
         <f>SUM(B13:B13)</f>
         <v>4200</v>
       </c>
-      <c r="C14" s="169">
+      <c r="C14" s="161">
         <f>SUM(C13:C13)</f>
         <v>2520</v>
       </c>
-      <c r="D14" s="169">
+      <c r="D14" s="161">
         <f>SUM(D13:D13)</f>
         <v>630</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="165"/>
-      <c r="C15" s="165"/>
-      <c r="D15" s="165"/>
+      <c r="B15" s="158"/>
+      <c r="C15" s="158"/>
+      <c r="D15" s="158"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3211,221 +3236,221 @@
   <dimension ref="A1:J25"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25" style="163" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25" style="156" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.109375" style="88" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" style="164" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" style="161" bestFit="1" customWidth="1"/>
-    <col min="5" max="9" width="9.109375" style="161"/>
-    <col min="10" max="10" width="11.5546875" style="161" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="161"/>
+    <col min="3" max="3" width="10" style="157" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" style="154" bestFit="1" customWidth="1"/>
+    <col min="5" max="9" width="9.109375" style="154"/>
+    <col min="10" max="10" width="11.5546875" style="154" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.109375" style="154"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="235" t="s">
+      <c r="A1" s="226" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="235"/>
-      <c r="C1" s="235"/>
+      <c r="B1" s="226"/>
+      <c r="C1" s="226"/>
     </row>
     <row r="2" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="235" t="s">
+      <c r="A2" s="226" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="235"/>
-      <c r="C2" s="235"/>
+      <c r="B2" s="226"/>
+      <c r="C2" s="226"/>
     </row>
     <row r="3" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="235" t="s">
+      <c r="A3" s="226" t="s">
         <v>108</v>
       </c>
-      <c r="B3" s="235"/>
-      <c r="C3" s="235"/>
+      <c r="B3" s="226"/>
+      <c r="C3" s="226"/>
     </row>
     <row r="4" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A4" s="230" t="s">
+      <c r="A4" s="221" t="s">
         <v>190</v>
       </c>
-      <c r="B4" s="222" t="s">
+      <c r="B4" s="213" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="223" t="s">
+      <c r="C4" s="214" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A5" s="224" t="s">
+      <c r="A5" s="215" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="225"/>
-      <c r="C5" s="225"/>
+      <c r="B5" s="216"/>
+      <c r="C5" s="216"/>
     </row>
     <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A6" s="226" t="s">
+      <c r="A6" s="217" t="s">
         <v>120</v>
       </c>
-      <c r="B6" s="232">
+      <c r="B6" s="223">
         <v>12560</v>
       </c>
-      <c r="C6" s="225"/>
+      <c r="C6" s="216"/>
     </row>
     <row r="7" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A7" s="224" t="s">
+      <c r="A7" s="215" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="225"/>
-      <c r="C7" s="225"/>
-      <c r="J7" s="162"/>
+      <c r="B7" s="216"/>
+      <c r="C7" s="216"/>
+      <c r="J7" s="155"/>
     </row>
     <row r="8" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A8" s="226" t="s">
+      <c r="A8" s="217" t="s">
         <v>110</v>
       </c>
-      <c r="B8" s="225">
+      <c r="B8" s="216">
         <f>+PPE!D4</f>
         <v>153700</v>
       </c>
-      <c r="C8" s="225"/>
-      <c r="J8" s="162"/>
+      <c r="C8" s="216"/>
+      <c r="J8" s="155"/>
     </row>
     <row r="9" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A9" s="226" t="s">
+      <c r="A9" s="217" t="s">
         <v>122</v>
       </c>
-      <c r="B9" s="225"/>
-      <c r="C9" s="225">
+      <c r="B9" s="216"/>
+      <c r="C9" s="216">
         <f>+PPE!G5</f>
         <v>28887.178082191782</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A10" s="224" t="s">
+      <c r="A10" s="215" t="s">
         <v>187</v>
       </c>
-      <c r="B10" s="225"/>
-      <c r="C10" s="225"/>
+      <c r="B10" s="216"/>
+      <c r="C10" s="216"/>
     </row>
     <row r="11" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="226" t="s">
+      <c r="A11" s="217" t="s">
         <v>121</v>
       </c>
-      <c r="B11" s="225"/>
-      <c r="C11" s="225">
+      <c r="B11" s="216"/>
+      <c r="C11" s="216">
         <f>+B22</f>
         <v>15000</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A12" s="226" t="s">
+      <c r="A12" s="217" t="s">
         <v>100</v>
       </c>
-      <c r="B12" s="225"/>
-      <c r="C12" s="225">
+      <c r="B12" s="216"/>
+      <c r="C12" s="216">
         <f>+B23</f>
         <v>25000</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="221" t="s">
+      <c r="A13" s="212" t="s">
         <v>188</v>
       </c>
-      <c r="B13" s="227"/>
-      <c r="C13" s="228"/>
+      <c r="B13" s="218"/>
+      <c r="C13" s="219"/>
     </row>
     <row r="14" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A14" s="226" t="s">
+      <c r="A14" s="217" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="225"/>
-      <c r="C14" s="225">
+      <c r="B14" s="216"/>
+      <c r="C14" s="216">
         <f>1000*6</f>
         <v>6000</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A15" s="226" t="s">
+      <c r="A15" s="217" t="s">
         <v>169</v>
       </c>
-      <c r="B15" s="225"/>
-      <c r="C15" s="225">
+      <c r="B15" s="216"/>
+      <c r="C15" s="216">
         <v>1000000</v>
       </c>
     </row>
-    <row r="16" spans="1:10" s="213" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A16" s="224" t="s">
+    <row r="16" spans="1:10" s="204" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="215" t="s">
         <v>154</v>
       </c>
-      <c r="B16" s="225"/>
-      <c r="C16" s="228"/>
+      <c r="B16" s="216"/>
+      <c r="C16" s="219"/>
     </row>
     <row r="17" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="229" t="s">
+      <c r="A17" s="220" t="s">
         <v>170</v>
       </c>
-      <c r="B17" s="233">
+      <c r="B17" s="224">
         <v>112919.5</v>
       </c>
-      <c r="C17" s="225"/>
+      <c r="C17" s="216"/>
     </row>
-    <row r="18" spans="1:3" s="213" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="226" t="s">
+    <row r="18" spans="1:3" s="204" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="217" t="s">
         <v>107</v>
       </c>
-      <c r="B18" s="225"/>
-      <c r="C18" s="234">
+      <c r="B18" s="216"/>
+      <c r="C18" s="225">
         <f>+Working!B2</f>
         <v>2328236</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="221" t="s">
+      <c r="A19" s="212" t="s">
         <v>189</v>
       </c>
-      <c r="B19" s="225"/>
-      <c r="C19" s="225"/>
+      <c r="B19" s="216"/>
+      <c r="C19" s="216"/>
     </row>
     <row r="20" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A20" s="226" t="s">
+      <c r="A20" s="217" t="s">
         <v>165</v>
       </c>
-      <c r="B20" s="225">
+      <c r="B20" s="216">
         <v>1220000</v>
       </c>
-      <c r="C20" s="225"/>
+      <c r="C20" s="216"/>
     </row>
     <row r="21" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A21" s="226" t="s">
+      <c r="A21" s="217" t="s">
         <v>142</v>
       </c>
-      <c r="B21" s="225"/>
-      <c r="C21" s="225"/>
+      <c r="B21" s="216"/>
+      <c r="C21" s="216"/>
     </row>
     <row r="22" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A22" s="226" t="s">
+      <c r="A22" s="217" t="s">
         <v>121</v>
       </c>
-      <c r="B22" s="225">
+      <c r="B22" s="216">
         <v>15000</v>
       </c>
-      <c r="C22" s="225"/>
+      <c r="C22" s="216"/>
     </row>
     <row r="23" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A23" s="226" t="s">
+      <c r="A23" s="217" t="s">
         <v>100</v>
       </c>
-      <c r="B23" s="225">
+      <c r="B23" s="216">
         <v>25000</v>
       </c>
-      <c r="C23" s="225"/>
+      <c r="C23" s="216"/>
     </row>
     <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="230" t="s">
+      <c r="A24" s="221" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="231">
+      <c r="B24" s="222">
         <f>SUM(B5:B23)</f>
         <v>1539179.5</v>
       </c>
-      <c r="C24" s="231">
+      <c r="C24" s="222">
         <f>SUM(C5:C23)</f>
         <v>3403123.1780821919</v>
       </c>
@@ -3469,7 +3494,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="160" t="s">
+      <c r="D1" s="153" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3650,7 +3675,7 @@
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="160" t="s">
+      <c r="E1" s="153" t="s">
         <v>36</v>
       </c>
     </row>
@@ -3694,7 +3719,7 @@
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="152"/>
+      <c r="B6" s="145"/>
     </row>
     <row r="7" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -3702,7 +3727,7 @@
       </c>
       <c r="B7" s="1"/>
       <c r="E7" s="73"/>
-      <c r="F7" s="151"/>
+      <c r="F7" s="144"/>
     </row>
     <row r="8" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A8" s="18" t="s">
@@ -3716,18 +3741,18 @@
         <f>+'P10'!J31</f>
         <v>#REF!</v>
       </c>
-      <c r="F8" s="151"/>
+      <c r="F8" s="144"/>
     </row>
     <row r="9" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="E9" s="126" t="e">
         <f>SUM(E8)</f>
         <v>#REF!</v>
       </c>
-      <c r="F9" s="151"/>
+      <c r="F9" s="144"/>
     </row>
     <row r="10" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="E10" s="121"/>
-      <c r="F10" s="151"/>
+      <c r="F10" s="144"/>
     </row>
     <row r="11" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
@@ -4735,13 +4760,13 @@
       <c r="ALO11" s="13"/>
     </row>
     <row r="12" spans="1:1003" x14ac:dyDescent="0.35">
-      <c r="A12" s="150" t="s">
+      <c r="A12" s="143" t="s">
         <v>170</v>
       </c>
-      <c r="B12" s="150"/>
-      <c r="C12" s="219"/>
-      <c r="D12" s="219"/>
-      <c r="E12" s="220">
+      <c r="B12" s="143"/>
+      <c r="C12" s="210"/>
+      <c r="D12" s="210"/>
+      <c r="E12" s="211">
         <f>TB!B17</f>
         <v>112919.5</v>
       </c>
@@ -8774,7 +8799,7 @@
     </row>
     <row r="16" spans="1:1003" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="E16" s="121"/>
-      <c r="F16" s="151"/>
+      <c r="F16" s="144"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13"/>
       <c r="L16" s="13"/>
@@ -9774,10 +9799,10 @@
       <c r="A17" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="152"/>
+      <c r="B17" s="145"/>
       <c r="E17" s="73"/>
-      <c r="F17" s="151"/>
-      <c r="I17" s="153"/>
+      <c r="F17" s="144"/>
+      <c r="I17" s="146"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13"/>
       <c r="L17" s="13"/>
@@ -10779,7 +10804,7 @@
       </c>
       <c r="B18" s="1"/>
       <c r="E18" s="73"/>
-      <c r="F18" s="151"/>
+      <c r="F18" s="144"/>
       <c r="J18" s="13"/>
       <c r="K18" s="13"/>
       <c r="L18" s="13"/>
@@ -11787,7 +11812,7 @@
         <f>+'P11'!J17</f>
         <v>6000</v>
       </c>
-      <c r="F19" s="151"/>
+      <c r="F19" s="144"/>
       <c r="J19" s="13"/>
       <c r="K19" s="13"/>
       <c r="L19" s="13"/>
@@ -12791,7 +12816,7 @@
         <f>+CE!G13</f>
         <v>#REF!</v>
       </c>
-      <c r="F20" s="151"/>
+      <c r="F20" s="144"/>
       <c r="J20" s="13"/>
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
@@ -13792,7 +13817,7 @@
         <f>SUM(E19:E20)</f>
         <v>#REF!</v>
       </c>
-      <c r="F21" s="151"/>
+      <c r="F21" s="144"/>
       <c r="J21" s="62"/>
       <c r="K21" s="13"/>
       <c r="L21" s="13"/>
@@ -14790,7 +14815,7 @@
     </row>
     <row r="22" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="E22" s="121"/>
-      <c r="F22" s="151"/>
+      <c r="F22" s="144"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
       <c r="L22" s="13"/>
@@ -15793,7 +15818,7 @@
       <c r="E23" s="121">
         <v>0</v>
       </c>
-      <c r="F23" s="151"/>
+      <c r="F23" s="144"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
@@ -16791,7 +16816,7 @@
     </row>
     <row r="24" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="E24" s="73"/>
-      <c r="F24" s="151"/>
+      <c r="F24" s="144"/>
       <c r="J24" s="13"/>
       <c r="K24" s="13"/>
       <c r="L24" s="13"/>
@@ -17793,7 +17818,7 @@
       </c>
       <c r="B25" s="1"/>
       <c r="E25" s="73"/>
-      <c r="F25" s="151"/>
+      <c r="F25" s="144"/>
       <c r="J25" s="13"/>
       <c r="K25" s="13"/>
       <c r="L25" s="13"/>
@@ -18790,7 +18815,7 @@
       <c r="ALO25" s="13"/>
     </row>
     <row r="26" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A26" s="154" t="s">
+      <c r="A26" s="147" t="s">
         <v>105</v>
       </c>
       <c r="C26" s="3">
@@ -18801,7 +18826,7 @@
         <f>+'P11'!J24</f>
         <v>#REF!</v>
       </c>
-      <c r="F26" s="151"/>
+      <c r="F26" s="144"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
       <c r="L26" s="13"/>
@@ -19798,15 +19823,15 @@
       <c r="ALO26" s="13"/>
     </row>
     <row r="27" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A27" s="154" t="s">
+      <c r="A27" s="147" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="155"/>
+      <c r="B27" s="148"/>
       <c r="E27" s="73">
         <f>TB!C15</f>
         <v>1000000</v>
       </c>
-      <c r="F27" s="151"/>
+      <c r="F27" s="144"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
@@ -20803,14 +20828,14 @@
       <c r="ALO27" s="13"/>
     </row>
     <row r="28" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A28" s="156" t="s">
+      <c r="A28" s="149" t="s">
         <v>41</v>
       </c>
       <c r="E28" s="126" t="e">
         <f>SUM(E26:E27)</f>
         <v>#REF!</v>
       </c>
-      <c r="F28" s="151"/>
+      <c r="F28" s="144"/>
       <c r="J28" s="13"/>
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
@@ -21807,14 +21832,14 @@
       <c r="ALO28" s="13"/>
     </row>
     <row r="29" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A29" s="156" t="s">
+      <c r="A29" s="149" t="s">
         <v>42</v>
       </c>
       <c r="E29" s="128" t="e">
         <f>E28+E23</f>
         <v>#REF!</v>
       </c>
-      <c r="F29" s="151"/>
+      <c r="F29" s="144"/>
       <c r="J29" s="13"/>
       <c r="K29" s="13"/>
       <c r="L29" s="13"/>
@@ -22819,7 +22844,7 @@
         <f>+E21+E29</f>
         <v>#REF!</v>
       </c>
-      <c r="F30" s="151"/>
+      <c r="F30" s="144"/>
       <c r="G30" s="77" t="e">
         <f>E15-E30</f>
         <v>#REF!</v>
@@ -28856,16 +28881,16 @@
       <c r="ALX35" s="2"/>
     </row>
     <row r="36" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="157" t="s">
+      <c r="A36" s="150" t="s">
         <v>43</v>
       </c>
-      <c r="B36" s="157"/>
-      <c r="C36" s="157"/>
-      <c r="D36" s="157"/>
+      <c r="B36" s="150"/>
+      <c r="C36" s="150"/>
+      <c r="D36" s="150"/>
       <c r="E36" s="24"/>
-      <c r="F36" s="157"/>
-      <c r="G36" s="157"/>
-      <c r="H36" s="157"/>
+      <c r="F36" s="150"/>
+      <c r="G36" s="150"/>
+      <c r="H36" s="150"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
@@ -29871,14 +29896,14 @@
       <c r="ALX36" s="2"/>
     </row>
     <row r="37" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="157"/>
-      <c r="B37" s="157"/>
-      <c r="C37" s="157"/>
-      <c r="D37" s="157"/>
+      <c r="A37" s="150"/>
+      <c r="B37" s="150"/>
+      <c r="C37" s="150"/>
+      <c r="D37" s="150"/>
       <c r="E37" s="24"/>
-      <c r="F37" s="157"/>
-      <c r="G37" s="157"/>
-      <c r="H37" s="157"/>
+      <c r="F37" s="150"/>
+      <c r="G37" s="150"/>
+      <c r="H37" s="150"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
@@ -30884,14 +30909,14 @@
       <c r="ALX37" s="2"/>
     </row>
     <row r="38" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="158"/>
-      <c r="B38" s="158"/>
-      <c r="C38" s="158"/>
-      <c r="D38" s="158"/>
+      <c r="A38" s="151"/>
+      <c r="B38" s="151"/>
+      <c r="C38" s="151"/>
+      <c r="D38" s="151"/>
       <c r="E38" s="25"/>
-      <c r="F38" s="158"/>
-      <c r="G38" s="158"/>
-      <c r="H38" s="158"/>
+      <c r="F38" s="151"/>
+      <c r="G38" s="151"/>
+      <c r="H38" s="151"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
@@ -34921,16 +34946,16 @@
       <c r="ALX41" s="2"/>
     </row>
     <row r="42" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="157" t="s">
+      <c r="A42" s="150" t="s">
         <v>46</v>
       </c>
-      <c r="B42" s="159"/>
-      <c r="C42" s="159"/>
-      <c r="D42" s="159"/>
+      <c r="B42" s="152"/>
+      <c r="C42" s="152"/>
+      <c r="D42" s="152"/>
       <c r="E42" s="26"/>
-      <c r="F42" s="159"/>
-      <c r="G42" s="159"/>
-      <c r="H42" s="159"/>
+      <c r="F42" s="152"/>
+      <c r="G42" s="152"/>
+      <c r="H42" s="152"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
@@ -35936,16 +35961,16 @@
       <c r="ALX42" s="2"/>
     </row>
     <row r="43" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="157" t="s">
+      <c r="A43" s="150" t="s">
         <v>47</v>
       </c>
-      <c r="B43" s="159"/>
-      <c r="C43" s="159"/>
-      <c r="D43" s="159"/>
+      <c r="B43" s="152"/>
+      <c r="C43" s="152"/>
+      <c r="D43" s="152"/>
       <c r="E43" s="26"/>
-      <c r="F43" s="159"/>
-      <c r="G43" s="159"/>
-      <c r="H43" s="159"/>
+      <c r="F43" s="152"/>
+      <c r="G43" s="152"/>
+      <c r="H43" s="152"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
@@ -36951,14 +36976,14 @@
       <c r="ALX43" s="2"/>
     </row>
     <row r="44" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="157"/>
-      <c r="B44" s="159"/>
-      <c r="C44" s="159"/>
-      <c r="D44" s="159"/>
+      <c r="A44" s="150"/>
+      <c r="B44" s="152"/>
+      <c r="C44" s="152"/>
+      <c r="D44" s="152"/>
       <c r="E44" s="26"/>
-      <c r="F44" s="159"/>
-      <c r="G44" s="159"/>
-      <c r="H44" s="159"/>
+      <c r="F44" s="152"/>
+      <c r="G44" s="152"/>
+      <c r="H44" s="152"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
@@ -37964,14 +37989,14 @@
       <c r="ALX44" s="2"/>
     </row>
     <row r="45" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="157"/>
-      <c r="B45" s="159"/>
-      <c r="C45" s="159"/>
-      <c r="D45" s="159"/>
+      <c r="A45" s="150"/>
+      <c r="B45" s="152"/>
+      <c r="C45" s="152"/>
+      <c r="D45" s="152"/>
       <c r="E45" s="26"/>
-      <c r="F45" s="159"/>
-      <c r="G45" s="159"/>
-      <c r="H45" s="159"/>
+      <c r="F45" s="152"/>
+      <c r="G45" s="152"/>
+      <c r="H45" s="152"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
@@ -43061,7 +43086,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="160" t="s">
+      <c r="I1" s="153" t="s">
         <v>50</v>
       </c>
       <c r="J1" s="1"/>
@@ -43204,17 +43229,17 @@
       <c r="A13" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="E13" s="180">
+      <c r="E13" s="171">
         <f>SUM(E7:E11)</f>
         <v>6000</v>
       </c>
-      <c r="F13" s="196"/>
-      <c r="G13" s="180" t="e">
+      <c r="F13" s="187"/>
+      <c r="G13" s="171" t="e">
         <f>SUM(G7:G11)</f>
         <v>#REF!</v>
       </c>
-      <c r="H13" s="196"/>
-      <c r="I13" s="180" t="e">
+      <c r="H13" s="187"/>
+      <c r="I13" s="171" t="e">
         <f>SUM(I7:I11)</f>
         <v>#REF!</v>
       </c>
@@ -43283,343 +43308,343 @@
   <dimension ref="A1:I43"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.88671875" style="177" customWidth="1"/>
-    <col min="2" max="2" width="30.44140625" style="177" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" style="177" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" style="177" customWidth="1"/>
-    <col min="5" max="5" width="9" style="177" customWidth="1"/>
-    <col min="6" max="6" width="0.6640625" style="177" customWidth="1"/>
-    <col min="7" max="7" width="13.109375" style="177" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="177" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" style="177" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="177"/>
+    <col min="1" max="1" width="2.88671875" style="168" customWidth="1"/>
+    <col min="2" max="2" width="30.44140625" style="168" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" style="168" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" style="168" customWidth="1"/>
+    <col min="5" max="5" width="9" style="168" customWidth="1"/>
+    <col min="6" max="6" width="0.6640625" style="168" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" style="168" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="168" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" style="168" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="168"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="179" t="s">
+      <c r="A1" s="170" t="s">
         <v>149</v>
       </c>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
-      <c r="G1" s="215" t="s">
+      <c r="E1" s="170"/>
+      <c r="F1" s="170"/>
+      <c r="G1" s="206" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="179"/>
+      <c r="H1" s="170"/>
     </row>
-    <row r="2" spans="1:8" s="174" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="179" t="s">
+    <row r="2" spans="1:8" s="165" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="170" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="189"/>
-      <c r="H2" s="179"/>
+      <c r="E2" s="170"/>
+      <c r="F2" s="170"/>
+      <c r="G2" s="180"/>
+      <c r="H2" s="170"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="174" t="str">
+      <c r="A3" s="165" t="str">
         <f>+PL!A3</f>
         <v>FOR THE YEAR PERIOD 31ST MARCH</v>
       </c>
-      <c r="B3" s="179"/>
-      <c r="C3" s="179"/>
-      <c r="D3" s="179"/>
-      <c r="E3" s="179"/>
-      <c r="F3" s="179"/>
-      <c r="G3" s="184">
+      <c r="B3" s="170"/>
+      <c r="C3" s="170"/>
+      <c r="D3" s="170"/>
+      <c r="E3" s="170"/>
+      <c r="F3" s="170"/>
+      <c r="G3" s="175">
         <v>2025</v>
       </c>
-      <c r="H3" s="179"/>
+      <c r="H3" s="170"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="G4" s="192" t="s">
+      <c r="G4" s="183" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F5" s="183"/>
+      <c r="F5" s="174"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="174" t="s">
+      <c r="A6" s="165" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="183"/>
-      <c r="G6" s="186"/>
+      <c r="F6" s="174"/>
+      <c r="G6" s="177"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="178" t="s">
+      <c r="A7" s="169" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="199"/>
-      <c r="G7" s="203" t="e">
+      <c r="F7" s="190"/>
+      <c r="G7" s="194" t="e">
         <f>+PL!D12</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="177" t="s">
+      <c r="A8" s="168" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="185"/>
-      <c r="G8" s="204"/>
+      <c r="F8" s="176"/>
+      <c r="G8" s="195"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B9" s="181" t="s">
+      <c r="B9" s="172" t="s">
         <v>129</v>
       </c>
-      <c r="C9" s="181"/>
-      <c r="D9" s="181"/>
-      <c r="F9" s="185"/>
-      <c r="G9" s="204" t="e">
+      <c r="C9" s="172"/>
+      <c r="D9" s="172"/>
+      <c r="F9" s="176"/>
+      <c r="G9" s="195" t="e">
         <f>'P09'!D22</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="174" t="s">
+      <c r="A10" s="165" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="185"/>
-      <c r="G10" s="205" t="e">
+      <c r="F10" s="176"/>
+      <c r="G10" s="196" t="e">
         <f>SUM(G7:G9)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F11" s="185"/>
-      <c r="G11" s="204"/>
+      <c r="F11" s="176"/>
+      <c r="G11" s="195"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B12" s="181" t="s">
+      <c r="B12" s="172" t="s">
         <v>172</v>
       </c>
-      <c r="C12" s="181"/>
-      <c r="D12" s="181"/>
-      <c r="F12" s="185"/>
-      <c r="G12" s="204">
+      <c r="C12" s="172"/>
+      <c r="D12" s="172"/>
+      <c r="F12" s="176"/>
+      <c r="G12" s="195">
         <f>-BS!E12</f>
         <v>-112919.5</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="181" t="s">
+      <c r="B13" s="172" t="s">
         <v>182</v>
       </c>
-      <c r="C13" s="181"/>
-      <c r="D13" s="181"/>
-      <c r="F13" s="185"/>
-      <c r="G13" s="204" t="e">
+      <c r="C13" s="172"/>
+      <c r="D13" s="172"/>
+      <c r="F13" s="176"/>
+      <c r="G13" s="195" t="e">
         <f>BS!E26</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B14" s="181" t="s">
+      <c r="B14" s="172" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="181"/>
-      <c r="D14" s="181"/>
-      <c r="F14" s="185"/>
-      <c r="G14" s="204">
+      <c r="C14" s="172"/>
+      <c r="D14" s="172"/>
+      <c r="F14" s="176"/>
+      <c r="G14" s="195">
         <f>BS!E27</f>
         <v>1000000</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="174" t="s">
+      <c r="A15" s="165" t="s">
         <v>56</v>
       </c>
-      <c r="F15" s="185"/>
-      <c r="G15" s="205" t="e">
+      <c r="F15" s="176"/>
+      <c r="G15" s="196" t="e">
         <f>SUM(G10:G14)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F16" s="185"/>
-      <c r="G16" s="204"/>
+      <c r="F16" s="176"/>
+      <c r="G16" s="195"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B17" s="177" t="s">
+      <c r="B17" s="168" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="185"/>
-      <c r="G17" s="204">
+      <c r="F17" s="176"/>
+      <c r="G17" s="195">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F18" s="185"/>
-      <c r="G18" s="206">
+      <c r="F18" s="176"/>
+      <c r="G18" s="197">
         <f>SUM(G17:G17)</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="174" t="s">
+      <c r="A19" s="165" t="s">
         <v>57</v>
       </c>
-      <c r="E19" s="174"/>
-      <c r="F19" s="185"/>
-      <c r="G19" s="206" t="e">
+      <c r="E19" s="165"/>
+      <c r="F19" s="176"/>
+      <c r="G19" s="197" t="e">
         <f>SUM(G18+G15)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F20" s="185"/>
-      <c r="G20" s="204"/>
+      <c r="F20" s="176"/>
+      <c r="G20" s="195"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="174" t="s">
+      <c r="A21" s="165" t="s">
         <v>58</v>
       </c>
-      <c r="F21" s="185"/>
-      <c r="G21" s="204"/>
+      <c r="F21" s="176"/>
+      <c r="G21" s="195"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B22" s="178" t="s">
+      <c r="B22" s="169" t="s">
         <v>143</v>
       </c>
-      <c r="F22" s="185"/>
-      <c r="G22" s="204" t="e">
+      <c r="F22" s="176"/>
+      <c r="G22" s="195" t="e">
         <f>-'P10'!G12</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="174" t="s">
+      <c r="A23" s="165" t="s">
         <v>59</v>
       </c>
-      <c r="E23" s="174"/>
-      <c r="F23" s="185"/>
-      <c r="G23" s="206" t="e">
+      <c r="E23" s="165"/>
+      <c r="F23" s="176"/>
+      <c r="G23" s="197" t="e">
         <f>SUM(G22)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F24" s="185"/>
-      <c r="G24" s="204"/>
+      <c r="F24" s="176"/>
+      <c r="G24" s="195"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="174" t="s">
+      <c r="A25" s="165" t="s">
         <v>60</v>
       </c>
-      <c r="F25" s="185"/>
-      <c r="G25" s="204"/>
+      <c r="F25" s="176"/>
+      <c r="G25" s="195"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B26" s="177" t="s">
+      <c r="B26" s="168" t="s">
         <v>70</v>
       </c>
-      <c r="F26" s="185"/>
-      <c r="G26" s="204">
+      <c r="F26" s="176"/>
+      <c r="G26" s="195">
         <f>+BS!E19</f>
         <v>6000</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="174" t="s">
+      <c r="A27" s="165" t="s">
         <v>61</v>
       </c>
-      <c r="F27" s="185"/>
-      <c r="G27" s="206">
+      <c r="F27" s="176"/>
+      <c r="G27" s="197">
         <f>SUM(G26)</f>
         <v>6000</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="174" t="s">
+      <c r="A28" s="165" t="s">
         <v>65</v>
       </c>
-      <c r="F28" s="185"/>
-      <c r="G28" s="204" t="e">
+      <c r="F28" s="176"/>
+      <c r="G28" s="195" t="e">
         <f>+G19+G23+G27</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B29" s="177" t="s">
+      <c r="B29" s="168" t="s">
         <v>62</v>
       </c>
-      <c r="F29" s="185"/>
-      <c r="G29" s="204">
+      <c r="F29" s="176"/>
+      <c r="G29" s="195">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="177" t="s">
+      <c r="B30" s="168" t="s">
         <v>63</v>
       </c>
-      <c r="F30" s="185"/>
-      <c r="G30" s="207" t="e">
+      <c r="F30" s="176"/>
+      <c r="G30" s="198" t="e">
         <f>SUM(G28:G29)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="F31" s="185"/>
-      <c r="G31" s="204"/>
+      <c r="F31" s="176"/>
+      <c r="G31" s="195"/>
     </row>
-    <row r="32" spans="1:7" s="178" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="175" t="s">
+    <row r="32" spans="1:7" s="169" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="166" t="s">
         <v>145</v>
       </c>
-      <c r="C32" s="172"/>
-      <c r="F32" s="195"/>
+      <c r="C32" s="163"/>
+      <c r="F32" s="186"/>
     </row>
-    <row r="33" spans="1:9" s="178" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="188" t="s">
+    <row r="33" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="179" t="s">
         <v>144</v>
       </c>
-      <c r="G33" s="194">
+      <c r="G33" s="185">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" s="178" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G34" s="216">
+    <row r="34" spans="1:9" s="169" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G34" s="207">
         <f>SUM(F33:F33)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" s="178" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="36" spans="1:9" s="178" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="175" t="s">
+    <row r="35" spans="1:9" s="169" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="166" t="s">
         <v>146</v>
       </c>
-      <c r="G36" s="195"/>
+      <c r="G36" s="186"/>
     </row>
-    <row r="37" spans="1:9" s="178" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="188" t="s">
+    <row r="37" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="179" t="s">
         <v>144</v>
       </c>
-      <c r="D37" s="187"/>
-      <c r="E37" s="187"/>
-      <c r="G37" s="194">
+      <c r="D37" s="178"/>
+      <c r="E37" s="178"/>
+      <c r="G37" s="185">
         <f>'P11'!J7</f>
         <v>12560</v>
       </c>
     </row>
-    <row r="38" spans="1:9" s="178" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="175"/>
-      <c r="G38" s="216">
+    <row r="38" spans="1:9" s="169" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="166"/>
+      <c r="G38" s="207">
         <f>SUM(G37:G37)</f>
         <v>12560</v>
       </c>
-      <c r="H38" s="190" t="e">
+      <c r="H38" s="181" t="e">
         <f>G30-G38</f>
         <v>#REF!</v>
       </c>
-      <c r="I38" s="190"/>
+      <c r="I38" s="181"/>
     </row>
     <row r="39" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A41" s="177" t="s">
+      <c r="A41" s="168" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43" s="178" t="s">
+      <c r="A43" s="169" t="s">
         <v>33</v>
       </c>
     </row>
@@ -43653,7 +43678,7 @@
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
-      <c r="D1" s="160" t="s">
+      <c r="D1" s="153" t="s">
         <v>66</v>
       </c>
       <c r="E1" s="34"/>
@@ -44082,7 +44107,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="160" t="s">
+      <c r="J1" s="153" t="s">
         <v>67</v>
       </c>
     </row>
@@ -44368,7 +44393,7 @@
       </c>
       <c r="H16" s="118"/>
       <c r="I16" s="119"/>
-      <c r="J16" s="144">
+      <c r="J16" s="137">
         <f>SUM(E16:G16)</f>
         <v>28887.178082191782</v>
       </c>
@@ -44391,7 +44416,7 @@
       </c>
       <c r="H17" s="118"/>
       <c r="I17" s="119"/>
-      <c r="J17" s="144" t="e">
+      <c r="J17" s="137" t="e">
         <f t="shared" ref="J17:J21" si="2">SUM(E17:G17)</f>
         <v>#REF!</v>
       </c>
@@ -44414,7 +44439,7 @@
       </c>
       <c r="H18" s="118"/>
       <c r="I18" s="119"/>
-      <c r="J18" s="144" t="e">
+      <c r="J18" s="137" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
@@ -44437,7 +44462,7 @@
       </c>
       <c r="H19" s="118"/>
       <c r="I19" s="119"/>
-      <c r="J19" s="144" t="e">
+      <c r="J19" s="137" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
@@ -44460,7 +44485,7 @@
       </c>
       <c r="H20" s="118"/>
       <c r="I20" s="119"/>
-      <c r="J20" s="144" t="e">
+      <c r="J20" s="137" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
@@ -44483,7 +44508,7 @@
       </c>
       <c r="H21" s="118"/>
       <c r="I21" s="119"/>
-      <c r="J21" s="144" t="e">
+      <c r="J21" s="137" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
@@ -44498,7 +44523,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="131"/>
-      <c r="G22" s="182" t="e">
+      <c r="G22" s="173" t="e">
         <f>SUM(G16:G21)</f>
         <v>#REF!</v>
       </c>
@@ -44598,7 +44623,7 @@
     </row>
     <row r="31" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="2"/>
-      <c r="J31" s="145" t="e">
+      <c r="J31" s="138" t="e">
         <f>SUM(J25:J30)</f>
         <v>#REF!</v>
       </c>

</xml_diff>

<commit_message>
feat: implement changes in equity reporting by adding CE DTO and integrating it into financial reports
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92A19933-8BDD-4631-9DA5-FDA53D42FFED}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE78BF2-CBD4-4FF0-84F0-C6AD79DAF653}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPE" sheetId="24" r:id="rId1"/>
     <sheet name="Working" sheetId="25" r:id="rId2"/>
     <sheet name="TB" sheetId="7" r:id="rId3"/>
-    <sheet name="PL" sheetId="2" r:id="rId4"/>
-    <sheet name="BS" sheetId="1" r:id="rId5"/>
-    <sheet name="CE" sheetId="8" r:id="rId6"/>
+    <sheet name="CE" sheetId="8" r:id="rId4"/>
+    <sheet name="PL" sheetId="2" r:id="rId5"/>
+    <sheet name="BS" sheetId="1" r:id="rId6"/>
     <sheet name="CF" sheetId="15" r:id="rId7"/>
     <sheet name="P09" sheetId="6" r:id="rId8"/>
     <sheet name="P10" sheetId="5" r:id="rId9"/>
@@ -840,7 +840,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -850,6 +850,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -952,7 +958,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="240">
+  <cellXfs count="243">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1405,9 +1411,6 @@
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1444,6 +1447,16 @@
     </xf>
     <xf numFmtId="43" fontId="25" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="12" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="12" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="11" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="23">
@@ -1931,92 +1944,92 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.109375" style="228" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.77734375" style="228" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" style="228" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" style="228" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" style="228" customWidth="1"/>
-    <col min="6" max="6" width="12" style="228" customWidth="1"/>
-    <col min="7" max="7" width="12.5546875" style="228" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="228"/>
-    <col min="9" max="9" width="10.6640625" style="228" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="228"/>
+    <col min="1" max="1" width="19.109375" style="227" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" style="227" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" style="227" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" style="227" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" style="227" customWidth="1"/>
+    <col min="6" max="6" width="12" style="227" customWidth="1"/>
+    <col min="7" max="7" width="12.5546875" style="227" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" style="227"/>
+    <col min="9" max="9" width="10.6640625" style="227" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="227"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="227" t="s">
+      <c r="A1" s="226" t="s">
         <v>114</v>
       </c>
-      <c r="C1" s="227"/>
+      <c r="C1" s="226"/>
     </row>
     <row r="3" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="229" t="s">
+      <c r="A3" s="228" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="230" t="s">
+      <c r="B3" s="229" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="229" t="s">
+      <c r="C3" s="228" t="s">
         <v>119</v>
       </c>
-      <c r="D3" s="231" t="s">
+      <c r="D3" s="230" t="s">
         <v>109</v>
       </c>
-      <c r="E3" s="230" t="s">
+      <c r="E3" s="229" t="s">
         <v>117</v>
       </c>
-      <c r="F3" s="230" t="s">
+      <c r="F3" s="229" t="s">
         <v>162</v>
       </c>
-      <c r="G3" s="230" t="s">
+      <c r="G3" s="229" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="232" t="s">
+      <c r="A4" s="231" t="s">
         <v>110</v>
       </c>
-      <c r="B4" s="233">
+      <c r="B4" s="232">
         <v>45385</v>
       </c>
-      <c r="C4" s="234">
+      <c r="C4" s="233">
         <v>5</v>
       </c>
-      <c r="D4" s="235">
+      <c r="D4" s="234">
         <v>153700</v>
       </c>
-      <c r="E4" s="233">
+      <c r="E4" s="232">
         <v>45728</v>
       </c>
-      <c r="F4" s="235">
+      <c r="F4" s="234">
         <f t="shared" ref="F4" si="0">E4-B4</f>
         <v>343</v>
       </c>
-      <c r="G4" s="236">
+      <c r="G4" s="235">
         <f>(D4/C4)*(F4/365)</f>
         <v>28887.178082191782</v>
       </c>
-      <c r="I4" s="237"/>
+      <c r="I4" s="236"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="231" t="s">
+      <c r="A5" s="230" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="238"/>
-      <c r="C5" s="238"/>
-      <c r="D5" s="239">
+      <c r="B5" s="237"/>
+      <c r="C5" s="237"/>
+      <c r="D5" s="238">
         <f>SUM(D4:D4)</f>
         <v>153700</v>
       </c>
-      <c r="E5" s="238"/>
-      <c r="F5" s="238"/>
-      <c r="G5" s="239">
+      <c r="E5" s="237"/>
+      <c r="F5" s="237"/>
+      <c r="G5" s="238">
         <f>SUM(G4:G4)</f>
         <v>28887.178082191782</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D7" s="237"/>
+      <c r="D7" s="236"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3246,25 +3259,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="226" t="s">
+      <c r="A1" s="239" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="226"/>
-      <c r="C1" s="226"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="239"/>
     </row>
     <row r="2" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="226" t="s">
+      <c r="A2" s="239" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="226"/>
-      <c r="C2" s="226"/>
+      <c r="B2" s="239"/>
+      <c r="C2" s="239"/>
     </row>
     <row r="3" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="226" t="s">
+      <c r="A3" s="239" t="s">
         <v>108</v>
       </c>
-      <c r="B3" s="226"/>
-      <c r="C3" s="226"/>
+      <c r="B3" s="239"/>
+      <c r="C3" s="239"/>
     </row>
     <row r="4" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A4" s="221" t="s">
@@ -3474,6 +3487,251 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr codeName="Sheet6"/>
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" style="13" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" style="13" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" style="13" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" style="13" customWidth="1"/>
+    <col min="6" max="6" width="0.5546875" style="13" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" style="13" customWidth="1"/>
+    <col min="8" max="8" width="0.5546875" style="13" customWidth="1"/>
+    <col min="9" max="9" width="12.21875" style="13" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="153" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" spans="1:10" s="30" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.35">
+      <c r="E4" s="90" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="31"/>
+      <c r="G4" s="90" t="s">
+        <v>76</v>
+      </c>
+      <c r="H4" s="31"/>
+      <c r="I4" s="90" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E5" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="242">
+        <v>0</v>
+      </c>
+      <c r="F7" s="84"/>
+      <c r="G7" s="242">
+        <v>0</v>
+      </c>
+      <c r="H7" s="84"/>
+      <c r="I7" s="84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E8" s="84"/>
+      <c r="F8" s="84"/>
+      <c r="G8" s="84"/>
+      <c r="H8" s="84"/>
+      <c r="I8" s="84"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" s="129">
+        <f>+TB!C14</f>
+        <v>6000</v>
+      </c>
+      <c r="F9" s="129"/>
+      <c r="G9" s="241">
+        <v>0</v>
+      </c>
+      <c r="H9" s="129"/>
+      <c r="I9" s="62">
+        <f>+E9</f>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E10" s="129"/>
+      <c r="F10" s="129"/>
+      <c r="G10" s="129"/>
+      <c r="H10" s="129"/>
+      <c r="I10" s="62"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="E11" s="240">
+        <v>0</v>
+      </c>
+      <c r="F11" s="62"/>
+      <c r="G11" s="62" t="e">
+        <f>+PL!D16</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H11" s="62"/>
+      <c r="I11" s="62" t="e">
+        <f>G11</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+      <c r="I12" s="62"/>
+    </row>
+    <row r="13" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E13" s="171">
+        <f>SUM(E7:E11)</f>
+        <v>6000</v>
+      </c>
+      <c r="F13" s="187"/>
+      <c r="G13" s="171" t="e">
+        <f>SUM(G7:G11)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H13" s="187"/>
+      <c r="I13" s="171" t="e">
+        <f>SUM(I7:I11)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="E14" s="130"/>
+      <c r="F14" s="130"/>
+      <c r="G14" s="130"/>
+      <c r="H14" s="130"/>
+      <c r="I14" s="130"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" s="13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.85" right="0.5" top="0.75" bottom="0.17" header="0.17" footer="0.17"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:G24"/>
@@ -3648,7 +3906,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:ALX51"/>
@@ -43057,251 +43315,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" style="13" customWidth="1"/>
-    <col min="3" max="3" width="8.33203125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" style="13" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" style="13" customWidth="1"/>
-    <col min="6" max="6" width="0.5546875" style="13" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" style="13" customWidth="1"/>
-    <col min="8" max="8" width="0.5546875" style="13" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" style="13" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="153" t="s">
-        <v>50</v>
-      </c>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.35">
-      <c r="E4" s="90" t="s">
-        <v>75</v>
-      </c>
-      <c r="F4" s="31"/>
-      <c r="G4" s="90" t="s">
-        <v>76</v>
-      </c>
-      <c r="H4" s="31"/>
-      <c r="I4" s="90" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E5" s="31" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="E7" s="84">
-        <v>0</v>
-      </c>
-      <c r="F7" s="84"/>
-      <c r="G7" s="84">
-        <v>0</v>
-      </c>
-      <c r="H7" s="84"/>
-      <c r="I7" s="84">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E8" s="84"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="84"/>
-      <c r="H8" s="84"/>
-      <c r="I8" s="84"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="E9" s="129">
-        <f>+TB!C14</f>
-        <v>6000</v>
-      </c>
-      <c r="F9" s="129"/>
-      <c r="G9" s="129">
-        <v>0</v>
-      </c>
-      <c r="H9" s="129"/>
-      <c r="I9" s="62">
-        <f>+E9</f>
-        <v>6000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E10" s="129"/>
-      <c r="F10" s="129"/>
-      <c r="G10" s="129"/>
-      <c r="H10" s="129"/>
-      <c r="I10" s="62"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="E11" s="62">
-        <v>0</v>
-      </c>
-      <c r="F11" s="62"/>
-      <c r="G11" s="62" t="e">
-        <f>+PL!D16</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H11" s="62"/>
-      <c r="I11" s="62" t="e">
-        <f>G11</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="62"/>
-      <c r="I12" s="62"/>
-    </row>
-    <row r="13" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="E13" s="171">
-        <f>SUM(E7:E11)</f>
-        <v>6000</v>
-      </c>
-      <c r="F13" s="187"/>
-      <c r="G13" s="171" t="e">
-        <f>SUM(G7:G11)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H13" s="187"/>
-      <c r="I13" s="171" t="e">
-        <f>SUM(I7:I11)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="E14" s="130"/>
-      <c r="F14" s="130"/>
-      <c r="G14" s="130"/>
-      <c r="H14" s="130"/>
-      <c r="I14" s="130"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="33"/>
-      <c r="I15" s="33"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="33"/>
-      <c r="I16" s="33"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
-      <c r="I17" s="33"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="E18" s="33"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="33"/>
-      <c r="I18" s="33"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="33"/>
-      <c r="I19" s="33"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23" s="18" t="s">
-        <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.85" right="0.5" top="0.75" bottom="0.17" header="0.17" footer="0.17"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet7"/>

</xml_diff>

<commit_message>
feat: add P09 worksheet generation with trial balance integration
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B722E2E5-E1CB-4466-8B59-8EE3BCA66BDE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626D41D6-5090-429E-AA7A-AD7E9D920402}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPE" sheetId="24" r:id="rId1"/>
     <sheet name="Working" sheetId="25" r:id="rId2"/>
     <sheet name="TB" sheetId="7" r:id="rId3"/>
-    <sheet name="CE" sheetId="8" r:id="rId4"/>
-    <sheet name="CF" sheetId="15" r:id="rId5"/>
-    <sheet name="PL" sheetId="2" r:id="rId6"/>
-    <sheet name="BS" sheetId="1" r:id="rId7"/>
-    <sheet name="P09" sheetId="6" r:id="rId8"/>
-    <sheet name="P10" sheetId="5" r:id="rId9"/>
-    <sheet name="P11" sheetId="19" r:id="rId10"/>
+    <sheet name="P11" sheetId="19" r:id="rId4"/>
+    <sheet name="CE" sheetId="8" r:id="rId5"/>
+    <sheet name="CF" sheetId="15" r:id="rId6"/>
+    <sheet name="PL" sheetId="2" r:id="rId7"/>
+    <sheet name="BS" sheetId="1" r:id="rId8"/>
+    <sheet name="P09" sheetId="6" r:id="rId9"/>
+    <sheet name="P10" sheetId="5" r:id="rId10"/>
     <sheet name="Income Tax" sheetId="20" r:id="rId11"/>
   </sheets>
   <externalReferences>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="180">
   <si>
     <t>STATEMENT OF FINANCIAL POSITION</t>
   </si>
@@ -371,9 +371,6 @@
     <t>WDV</t>
   </si>
   <si>
-    <t>Printing &amp; Stationery</t>
-  </si>
-  <si>
     <t>Audit Fee</t>
   </si>
   <si>
@@ -390,9 +387,6 @@
   </si>
   <si>
     <t>Trade Creditors &amp; Other Payable</t>
-  </si>
-  <si>
-    <t>Telephone &amp; Internet</t>
   </si>
   <si>
     <t>Interest Income</t>
@@ -480,18 +474,6 @@
  31.03.2025</t>
   </si>
   <si>
-    <t>Salaries &amp; Wages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electricity </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Office Rent </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Depreciation </t>
-  </si>
-  <si>
     <t>Accountancy Fee</t>
   </si>
   <si>
@@ -516,9 +498,6 @@
     <t>At the End</t>
   </si>
   <si>
-    <t>Incorporation Fee</t>
-  </si>
-  <si>
     <t>Commission Income</t>
   </si>
   <si>
@@ -532,9 +511,6 @@
   </si>
   <si>
     <t>Bad Debts</t>
-  </si>
-  <si>
-    <t>Insurance</t>
   </si>
   <si>
     <t>Income</t>
@@ -564,22 +540,10 @@
     <t>Date</t>
   </si>
   <si>
-    <t xml:space="preserve">Business Promotion &amp; Marketing Expneses </t>
-  </si>
-  <si>
-    <t xml:space="preserve">EPF </t>
-  </si>
-  <si>
     <t>Dirtectors remuniration</t>
   </si>
   <si>
     <t>FOR THE PERIOD ENDED 31ST MARCH</t>
-  </si>
-  <si>
-    <t>Director Remuniration</t>
-  </si>
-  <si>
-    <t>Office Repair &amp; Maintance</t>
   </si>
   <si>
     <t>Director C/A - Invetment</t>
@@ -1455,10 +1419,10 @@
     <xf numFmtId="43" fontId="11" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="43" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="43" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="23">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1959,36 +1923,36 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="226" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C1" s="226"/>
     </row>
     <row r="3" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A3" s="228" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="229" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="228" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" s="230" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="229" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="229" t="s">
+      <c r="F3" s="229" t="s">
+        <v>154</v>
+      </c>
+      <c r="G3" s="229" t="s">
         <v>116</v>
-      </c>
-      <c r="C3" s="228" t="s">
-        <v>119</v>
-      </c>
-      <c r="D3" s="230" t="s">
-        <v>109</v>
-      </c>
-      <c r="E3" s="229" t="s">
-        <v>117</v>
-      </c>
-      <c r="F3" s="229" t="s">
-        <v>162</v>
-      </c>
-      <c r="G3" s="229" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="231" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B4" s="232">
         <v>45385</v>
@@ -2038,6 +2002,1614 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <sheetPr codeName="Sheet9"/>
+  <dimension ref="A1:AMD52"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="5" style="15" customWidth="1"/>
+    <col min="2" max="2" width="25" style="2" customWidth="1"/>
+    <col min="3" max="3" width="6.33203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" style="38" customWidth="1"/>
+    <col min="6" max="6" width="0.6640625" style="17" customWidth="1"/>
+    <col min="7" max="7" width="13" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" style="2" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="0.6640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="13.33203125" style="2" customWidth="1"/>
+    <col min="11" max="1018" width="9.109375" style="2"/>
+    <col min="1019" max="16384" width="9.109375" style="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="153" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" s="79" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" s="80"/>
+      <c r="B3" s="92"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" s="36">
+        <v>8</v>
+      </c>
+      <c r="B4" s="92" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+    </row>
+    <row r="5" spans="1:13" ht="28.8" x14ac:dyDescent="0.35">
+      <c r="A5" s="36"/>
+      <c r="B5" s="96" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="F5" s="39"/>
+      <c r="G5" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="41" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="42"/>
+      <c r="J5" s="43" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" s="36"/>
+      <c r="B6" s="44" t="str">
+        <f>+TB!A8</f>
+        <v>Furniture &amp; Fittings</v>
+      </c>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="131">
+        <v>0</v>
+      </c>
+      <c r="F6" s="131"/>
+      <c r="G6" s="131">
+        <f>TB!B8</f>
+        <v>153700</v>
+      </c>
+      <c r="H6" s="118"/>
+      <c r="I6" s="119"/>
+      <c r="J6" s="118">
+        <f>SUM(E6:G6)</f>
+        <v>153700</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" s="36"/>
+      <c r="B7" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="131">
+        <v>0</v>
+      </c>
+      <c r="F7" s="131"/>
+      <c r="G7" s="131" t="e">
+        <f>TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H7" s="118"/>
+      <c r="I7" s="119"/>
+      <c r="J7" s="118" t="e">
+        <f t="shared" ref="J7:J11" si="0">SUM(E7:G7)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" s="36"/>
+      <c r="B8" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="131">
+        <v>0</v>
+      </c>
+      <c r="F8" s="131"/>
+      <c r="G8" s="131" t="e">
+        <f>TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H8" s="118"/>
+      <c r="I8" s="119"/>
+      <c r="J8" s="118" t="e">
+        <f t="shared" si="0"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" s="36"/>
+      <c r="B9" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
+      <c r="E9" s="131">
+        <v>0</v>
+      </c>
+      <c r="F9" s="131"/>
+      <c r="G9" s="131" t="e">
+        <f>TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H9" s="118"/>
+      <c r="I9" s="119"/>
+      <c r="J9" s="118" t="e">
+        <f t="shared" si="0"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" s="36"/>
+      <c r="B10" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C10" s="44"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="131">
+        <v>0</v>
+      </c>
+      <c r="F10" s="131"/>
+      <c r="G10" s="131" t="e">
+        <f>TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H10" s="118"/>
+      <c r="I10" s="119"/>
+      <c r="J10" s="118" t="e">
+        <f t="shared" si="0"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A11" s="36"/>
+      <c r="B11" s="44" t="e">
+        <f>+TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="131">
+        <v>0</v>
+      </c>
+      <c r="F11" s="131"/>
+      <c r="G11" s="131" t="e">
+        <f>TB!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H11" s="118"/>
+      <c r="I11" s="119"/>
+      <c r="J11" s="118" t="e">
+        <f t="shared" si="0"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="36"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="132">
+        <f>SUM(E6:E11)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="131"/>
+      <c r="G12" s="132" t="e">
+        <f>SUM(G6:G11)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H12" s="118"/>
+      <c r="I12" s="119"/>
+      <c r="J12" s="132" t="e">
+        <f>SUM(J6:J11)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="36"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="47"/>
+      <c r="F13" s="47"/>
+      <c r="G13" s="47"/>
+      <c r="H13" s="47"/>
+      <c r="I13" s="47"/>
+      <c r="J13" s="46"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A14" s="36"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+    </row>
+    <row r="15" spans="1:13" ht="28.8" x14ac:dyDescent="0.35">
+      <c r="A15" s="36"/>
+      <c r="B15" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="41" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="42"/>
+      <c r="J15" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="M15" s="49"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A16" s="50"/>
+      <c r="B16" s="44" t="str">
+        <f t="shared" ref="B16:B21" si="1">B6</f>
+        <v>Furniture &amp; Fittings</v>
+      </c>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="131">
+        <v>0</v>
+      </c>
+      <c r="F16" s="131"/>
+      <c r="G16" s="118">
+        <f>PPE!G4</f>
+        <v>28887.178082191782</v>
+      </c>
+      <c r="H16" s="118"/>
+      <c r="I16" s="119"/>
+      <c r="J16" s="137">
+        <f>SUM(E16:G16)</f>
+        <v>28887.178082191782</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="50"/>
+      <c r="B17" s="44" t="e">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="131">
+        <v>0</v>
+      </c>
+      <c r="F17" s="131"/>
+      <c r="G17" s="118" t="e">
+        <f>PPE!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H17" s="118"/>
+      <c r="I17" s="119"/>
+      <c r="J17" s="137" t="e">
+        <f t="shared" ref="J17:J21" si="2">SUM(E17:G17)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="50"/>
+      <c r="B18" s="44" t="e">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="131">
+        <v>0</v>
+      </c>
+      <c r="F18" s="131"/>
+      <c r="G18" s="118" t="e">
+        <f>PPE!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H18" s="118"/>
+      <c r="I18" s="119"/>
+      <c r="J18" s="137" t="e">
+        <f t="shared" si="2"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="50"/>
+      <c r="B19" s="44" t="e">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="131">
+        <v>0</v>
+      </c>
+      <c r="F19" s="131"/>
+      <c r="G19" s="118" t="e">
+        <f>PPE!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H19" s="118"/>
+      <c r="I19" s="119"/>
+      <c r="J19" s="137" t="e">
+        <f t="shared" si="2"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" s="50"/>
+      <c r="B20" s="44" t="e">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="131">
+        <v>0</v>
+      </c>
+      <c r="F20" s="131"/>
+      <c r="G20" s="118" t="e">
+        <f>PPE!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H20" s="118"/>
+      <c r="I20" s="119"/>
+      <c r="J20" s="137" t="e">
+        <f t="shared" si="2"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21" s="50"/>
+      <c r="B21" s="44" t="e">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="C21" s="44"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="131">
+        <v>0</v>
+      </c>
+      <c r="F21" s="131"/>
+      <c r="G21" s="118" t="e">
+        <f>PPE!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H21" s="118"/>
+      <c r="I21" s="119"/>
+      <c r="J21" s="137" t="e">
+        <f t="shared" si="2"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="50"/>
+      <c r="B22" s="44"/>
+      <c r="C22" s="44"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="132">
+        <f>SUM(E16:E21)</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="131"/>
+      <c r="G22" s="173" t="e">
+        <f>SUM(G16:G21)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H22" s="118"/>
+      <c r="I22" s="119"/>
+      <c r="J22" s="132" t="e">
+        <f>SUM(J16:J21)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="36"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="48"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="38"/>
+    </row>
+    <row r="24" spans="1:10" ht="28.8" x14ac:dyDescent="0.35">
+      <c r="A24" s="2"/>
+      <c r="B24" s="96" t="s">
+        <v>80</v>
+      </c>
+      <c r="J24" s="90" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="2"/>
+      <c r="B25" s="44" t="str">
+        <f t="shared" ref="B25:B30" si="3">B16</f>
+        <v>Furniture &amp; Fittings</v>
+      </c>
+      <c r="J25" s="74">
+        <f t="shared" ref="J25:J30" si="4">J6-J16</f>
+        <v>124812.82191780822</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="2"/>
+      <c r="B26" s="44" t="e">
+        <f t="shared" si="3"/>
+        <v>#REF!</v>
+      </c>
+      <c r="J26" s="74" t="e">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="2"/>
+      <c r="B27" s="44" t="e">
+        <f t="shared" si="3"/>
+        <v>#REF!</v>
+      </c>
+      <c r="J27" s="74" t="e">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="2"/>
+      <c r="B28" s="44" t="e">
+        <f t="shared" si="3"/>
+        <v>#REF!</v>
+      </c>
+      <c r="J28" s="74" t="e">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" s="2"/>
+      <c r="B29" s="44" t="e">
+        <f t="shared" si="3"/>
+        <v>#REF!</v>
+      </c>
+      <c r="J29" s="74" t="e">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="2"/>
+      <c r="B30" s="44" t="e">
+        <f t="shared" si="3"/>
+        <v>#REF!</v>
+      </c>
+      <c r="J30" s="74" t="e">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="2"/>
+      <c r="J31" s="138" t="e">
+        <f>SUM(J25:J30)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="2"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" s="2"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36" s="2"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" s="2"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40" s="2"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A41" s="2"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42" s="2"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43" s="2"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44" s="2"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45" s="2"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46" s="2"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A47" s="2"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A48" s="2"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49" s="2"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A50" s="2"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A51" s="2"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A52" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.85" right="0.5" top="0.75" bottom="0.17" header="0.17" footer="0.17"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <sheetPr codeName="Sheet11"/>
+  <dimension ref="A1:K54"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.109375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.88671875" style="13" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" style="13" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" style="13" customWidth="1"/>
+    <col min="7" max="7" width="0.6640625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="13" customWidth="1"/>
+    <col min="9" max="10" width="9.109375" style="13"/>
+    <col min="11" max="11" width="10.6640625" style="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="153" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="30"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="30" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="30"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="30" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="95"/>
+      <c r="B5" s="95"/>
+      <c r="D5" s="96"/>
+      <c r="E5" s="96"/>
+      <c r="H5" s="96" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="63" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="21"/>
+      <c r="H6" s="21" t="e">
+        <f>+PL!D12</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="97"/>
+      <c r="E7" s="21"/>
+      <c r="H7" s="21"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="64" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" s="21"/>
+      <c r="H8" s="98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E9" s="21"/>
+      <c r="H9" s="21" t="e">
+        <f>SUM(H6:H8)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="30"/>
+      <c r="E10" s="21"/>
+      <c r="H10" s="21"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="D11" s="99"/>
+      <c r="F11" s="191" t="e">
+        <f>'P10'!G22</f>
+        <v>#REF!</v>
+      </c>
+      <c r="H11" s="205" t="e">
+        <f>+F11</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E12" s="21"/>
+      <c r="H12" s="21" t="e">
+        <f>SUM(H9:H11)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="30" t="s">
+        <v>128</v>
+      </c>
+      <c r="B13" s="30"/>
+      <c r="E13" s="21"/>
+      <c r="H13" s="21"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" s="65" t="s">
+        <v>134</v>
+      </c>
+      <c r="H14" s="98" t="e">
+        <f>-E42</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="E15" s="21"/>
+      <c r="H15" s="100" t="e">
+        <f>SUM(H12:H14)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E16" s="101"/>
+      <c r="H16" s="101"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="E17" s="101"/>
+      <c r="H17" s="136" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="E18" s="101"/>
+      <c r="H18" s="101"/>
+    </row>
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="102" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="103" t="s">
+        <v>90</v>
+      </c>
+      <c r="F19" s="32" t="str">
+        <f>+H17</f>
+        <v>Loss</v>
+      </c>
+      <c r="H19" s="101" t="e">
+        <f>F19*0.3</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E20" s="101"/>
+      <c r="H20" s="101"/>
+    </row>
+    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="104" t="s">
+        <v>91</v>
+      </c>
+      <c r="E21" s="101"/>
+      <c r="H21" s="101"/>
+    </row>
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="E22" s="65">
+        <v>24252</v>
+      </c>
+      <c r="F22" s="106">
+        <v>0</v>
+      </c>
+      <c r="G22" s="105"/>
+      <c r="H22" s="106">
+        <f>-SUM(F22:F22)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="3.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D23" s="65"/>
+      <c r="E23" s="101"/>
+      <c r="F23" s="101"/>
+      <c r="G23" s="105"/>
+      <c r="H23" s="101"/>
+    </row>
+    <row r="24" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="E24" s="101"/>
+      <c r="H24" s="107" t="e">
+        <f>SUM(H19:H22)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K24" s="29"/>
+    </row>
+    <row r="25" spans="1:11" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="E25" s="101"/>
+      <c r="H25" s="101"/>
+    </row>
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E26" s="101"/>
+      <c r="H26" s="101"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A27" s="63" t="s">
+        <v>93</v>
+      </c>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="101"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+    </row>
+    <row r="28" spans="1:11" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E28" s="101"/>
+      <c r="H28" s="101"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29" s="87" t="s">
+        <v>94</v>
+      </c>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18"/>
+    </row>
+    <row r="30" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="18"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+    </row>
+    <row r="31" spans="1:11" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="108" t="s">
+        <v>95</v>
+      </c>
+      <c r="B31" s="109" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="96" t="s">
+        <v>96</v>
+      </c>
+      <c r="D31" s="110" t="s">
+        <v>129</v>
+      </c>
+      <c r="E31" s="90" t="s">
+        <v>97</v>
+      </c>
+      <c r="F31" s="90" t="s">
+        <v>130</v>
+      </c>
+      <c r="G31" s="90"/>
+      <c r="H31" s="96" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="108"/>
+      <c r="B32" s="109"/>
+      <c r="C32" s="65"/>
+      <c r="D32" s="111"/>
+      <c r="E32" s="111"/>
+      <c r="F32" s="111"/>
+      <c r="G32" s="111"/>
+      <c r="H32" s="65"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33" s="108" t="s">
+        <v>131</v>
+      </c>
+      <c r="B33" s="109"/>
+      <c r="C33" s="65"/>
+      <c r="D33" s="111"/>
+      <c r="E33" s="111"/>
+      <c r="F33" s="111"/>
+      <c r="G33" s="111"/>
+      <c r="H33" s="65"/>
+    </row>
+    <row r="34" spans="1:8" ht="5.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="108"/>
+      <c r="B34" s="109"/>
+      <c r="C34" s="65"/>
+      <c r="D34" s="111"/>
+      <c r="E34" s="111"/>
+      <c r="F34" s="111"/>
+      <c r="G34" s="111"/>
+      <c r="H34" s="65"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A35" s="108" t="str">
+        <f>+'P10'!B6</f>
+        <v>Furniture &amp; Fittings</v>
+      </c>
+      <c r="B35" s="167">
+        <f>+'P10'!G6</f>
+        <v>153700</v>
+      </c>
+      <c r="C35" s="65">
+        <v>5</v>
+      </c>
+      <c r="D35" s="140">
+        <v>0</v>
+      </c>
+      <c r="E35" s="139">
+        <f>B35/C35</f>
+        <v>30740</v>
+      </c>
+      <c r="F35" s="139">
+        <f>D35+E35</f>
+        <v>30740</v>
+      </c>
+      <c r="G35" s="111"/>
+      <c r="H35" s="142">
+        <f>B35-F35</f>
+        <v>122960</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A36" s="192" t="e">
+        <f>+'P10'!B7</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B36" s="167" t="e">
+        <f>+'P10'!G7</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C36" s="65">
+        <v>5</v>
+      </c>
+      <c r="D36" s="201">
+        <v>0</v>
+      </c>
+      <c r="E36" s="199" t="e">
+        <f t="shared" ref="E36:E40" si="0">B36/C36</f>
+        <v>#REF!</v>
+      </c>
+      <c r="F36" s="199" t="e">
+        <f t="shared" ref="F36:F40" si="1">D36+E36</f>
+        <v>#REF!</v>
+      </c>
+      <c r="G36" s="111"/>
+      <c r="H36" s="203" t="e">
+        <f t="shared" ref="H36:H40" si="2">B36-F36</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A37" s="192" t="e">
+        <f>+'P10'!B8</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B37" s="167" t="e">
+        <f>+'P10'!G8</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C37" s="65">
+        <v>5</v>
+      </c>
+      <c r="D37" s="201">
+        <v>0</v>
+      </c>
+      <c r="E37" s="199" t="e">
+        <f t="shared" si="0"/>
+        <v>#REF!</v>
+      </c>
+      <c r="F37" s="199" t="e">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="G37" s="111"/>
+      <c r="H37" s="203" t="e">
+        <f t="shared" si="2"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="192" t="e">
+        <f>+'P10'!B9</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B38" s="167" t="e">
+        <f>+'P10'!G9</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C38" s="188">
+        <v>5</v>
+      </c>
+      <c r="D38" s="201">
+        <v>0</v>
+      </c>
+      <c r="E38" s="199" t="e">
+        <f t="shared" si="0"/>
+        <v>#REF!</v>
+      </c>
+      <c r="F38" s="199" t="e">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="G38" s="193"/>
+      <c r="H38" s="203" t="e">
+        <f t="shared" si="2"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="192" t="e">
+        <f>+'P10'!B10</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B39" s="167" t="e">
+        <f>+'P10'!G10</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C39" s="188">
+        <v>5</v>
+      </c>
+      <c r="D39" s="201">
+        <v>0</v>
+      </c>
+      <c r="E39" s="199" t="e">
+        <f t="shared" si="0"/>
+        <v>#REF!</v>
+      </c>
+      <c r="F39" s="199" t="e">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="G39" s="193"/>
+      <c r="H39" s="203" t="e">
+        <f t="shared" si="2"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="192" t="e">
+        <f>+'P10'!B11</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B40" s="167" t="e">
+        <f>+'P10'!G11</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C40" s="188">
+        <v>5</v>
+      </c>
+      <c r="D40" s="201">
+        <v>0</v>
+      </c>
+      <c r="E40" s="199" t="e">
+        <f t="shared" si="0"/>
+        <v>#REF!</v>
+      </c>
+      <c r="F40" s="199" t="e">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="G40" s="193"/>
+      <c r="H40" s="203" t="e">
+        <f t="shared" si="2"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" s="182" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="192"/>
+      <c r="B41" s="200"/>
+      <c r="C41" s="188"/>
+      <c r="D41" s="201"/>
+      <c r="E41" s="199"/>
+      <c r="F41" s="199"/>
+      <c r="G41" s="193"/>
+      <c r="H41" s="203"/>
+    </row>
+    <row r="42" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A42" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="B42" s="141" t="e">
+        <f>SUM(B35:B40)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C42" s="113"/>
+      <c r="D42" s="202">
+        <f>SUM(D35:D40)</f>
+        <v>0</v>
+      </c>
+      <c r="E42" s="202" t="e">
+        <f t="shared" ref="E42:H42" si="3">SUM(E35:E40)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="F42" s="202" t="e">
+        <f t="shared" si="3"/>
+        <v>#REF!</v>
+      </c>
+      <c r="G42" s="113"/>
+      <c r="H42" s="202" t="e">
+        <f t="shared" si="3"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="18"/>
+      <c r="B43" s="112"/>
+      <c r="C43" s="112"/>
+      <c r="D43" s="112"/>
+      <c r="E43" s="112"/>
+      <c r="F43" s="112"/>
+      <c r="G43" s="112"/>
+      <c r="H43" s="112"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A45" s="189" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A46" s="184" t="s">
+        <v>163</v>
+      </c>
+      <c r="H46" s="164">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A47" s="184" t="s">
+        <v>164</v>
+      </c>
+      <c r="H47" s="208" t="e">
+        <f>-H15</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A48" s="184"/>
+      <c r="H48" s="164" t="e">
+        <f>SUM(H46:H47)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A49" s="184"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A50" s="184" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A51" s="184" t="s">
+        <v>166</v>
+      </c>
+      <c r="H51" s="164">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A52" s="184" t="s">
+        <v>167</v>
+      </c>
+      <c r="H52" s="164">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A53" s="184" t="s">
+        <v>168</v>
+      </c>
+      <c r="H53" s="209" t="e">
+        <f>SUM(H48:H52)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+  </sheetData>
+  <pageMargins left="0.85" right="0.5" top="0.75" bottom="0.17" header="0.17" footer="0.17"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2A291A8-AC8E-4BB6-A21B-06A29BC55837}">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="212" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="158">
+        <v>2328236</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B3" s="158"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="212" t="s">
+        <v>173</v>
+      </c>
+      <c r="B4" s="158"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B5" s="162">
+        <v>99975</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="158"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="158"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="212" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B9" s="158"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B10" s="158"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="212" t="s">
+        <v>174</v>
+      </c>
+      <c r="B11" s="158"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>148</v>
+      </c>
+      <c r="B12" t="s">
+        <v>149</v>
+      </c>
+      <c r="C12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="159">
+        <v>45597</v>
+      </c>
+      <c r="B13" s="158">
+        <v>4200</v>
+      </c>
+      <c r="C13" s="158">
+        <f>B13*12/20</f>
+        <v>2520</v>
+      </c>
+      <c r="D13" s="158">
+        <f>C13*3/12</f>
+        <v>630</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="160">
+        <f>SUM(B13:B13)</f>
+        <v>4200</v>
+      </c>
+      <c r="C14" s="161">
+        <f>SUM(C13:C13)</f>
+        <v>2520</v>
+      </c>
+      <c r="D14" s="161">
+        <f>SUM(D13:D13)</f>
+        <v>630</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="158"/>
+      <c r="C15" s="158"/>
+      <c r="D15" s="158"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr codeName="Sheet3"/>
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25" style="156" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" style="88" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="157" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" style="154" bestFit="1" customWidth="1"/>
+    <col min="5" max="9" width="9.109375" style="154"/>
+    <col min="10" max="10" width="11.5546875" style="154" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.109375" style="154"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A1" s="243" t="s">
+        <v>179</v>
+      </c>
+      <c r="B1" s="243"/>
+      <c r="C1" s="243"/>
+    </row>
+    <row r="2" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A2" s="243" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="243"/>
+      <c r="C2" s="243"/>
+    </row>
+    <row r="3" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A3" s="243" t="s">
+        <v>106</v>
+      </c>
+      <c r="B3" s="243"/>
+      <c r="C3" s="243"/>
+    </row>
+    <row r="4" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A4" s="221" t="s">
+        <v>178</v>
+      </c>
+      <c r="B4" s="213" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="214" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A5" s="215" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="216"/>
+      <c r="C5" s="216"/>
+    </row>
+    <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A6" s="217" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" s="223">
+        <v>12560</v>
+      </c>
+      <c r="C6" s="216"/>
+    </row>
+    <row r="7" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A7" s="215" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="216"/>
+      <c r="C7" s="216"/>
+      <c r="J7" s="155"/>
+    </row>
+    <row r="8" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A8" s="217" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="216">
+        <f>+PPE!D4</f>
+        <v>153700</v>
+      </c>
+      <c r="C8" s="216"/>
+      <c r="J8" s="155"/>
+    </row>
+    <row r="9" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A9" s="217" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="216"/>
+      <c r="C9" s="216">
+        <f>+PPE!G5</f>
+        <v>28887.178082191782</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A10" s="215" t="s">
+        <v>175</v>
+      </c>
+      <c r="B10" s="216"/>
+      <c r="C10" s="216"/>
+    </row>
+    <row r="11" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A11" s="217" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="216"/>
+      <c r="C11" s="216">
+        <f>+B22</f>
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A12" s="217" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="216"/>
+      <c r="C12" s="216">
+        <f>+B23</f>
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="212" t="s">
+        <v>176</v>
+      </c>
+      <c r="B13" s="218"/>
+      <c r="C13" s="219"/>
+    </row>
+    <row r="14" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A14" s="217" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="216"/>
+      <c r="C14" s="216">
+        <f>1000*6</f>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A15" s="217" t="s">
+        <v>157</v>
+      </c>
+      <c r="B15" s="216"/>
+      <c r="C15" s="216">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" s="204" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="215" t="s">
+        <v>146</v>
+      </c>
+      <c r="B16" s="216"/>
+      <c r="C16" s="219"/>
+    </row>
+    <row r="17" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A17" s="220" t="s">
+        <v>158</v>
+      </c>
+      <c r="B17" s="224">
+        <v>112919.5</v>
+      </c>
+      <c r="C17" s="216"/>
+    </row>
+    <row r="18" spans="1:3" s="204" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="217" t="s">
+        <v>105</v>
+      </c>
+      <c r="B18" s="216"/>
+      <c r="C18" s="225">
+        <f>+Working!B2</f>
+        <v>2328236</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="212" t="s">
+        <v>177</v>
+      </c>
+      <c r="B19" s="216"/>
+      <c r="C19" s="216"/>
+    </row>
+    <row r="20" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="217" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20" s="216">
+        <v>1220000</v>
+      </c>
+      <c r="C20" s="216"/>
+    </row>
+    <row r="21" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A21" s="217" t="s">
+        <v>136</v>
+      </c>
+      <c r="B21" s="216">
+        <v>1000</v>
+      </c>
+      <c r="C21" s="216"/>
+    </row>
+    <row r="22" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A22" s="217" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" s="216">
+        <v>15000</v>
+      </c>
+      <c r="C22" s="216"/>
+    </row>
+    <row r="23" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A23" s="217" t="s">
+        <v>99</v>
+      </c>
+      <c r="B23" s="216">
+        <v>25000</v>
+      </c>
+      <c r="C23" s="216"/>
+    </row>
+    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="222">
+        <f>SUM(B5:B23)</f>
+        <v>1540179.5</v>
+      </c>
+      <c r="C24" s="222">
+        <f>SUM(C5:C23)</f>
+        <v>3403123.1780821919</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="14.4" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="88">
+        <f>B24-C24</f>
+        <v>-1862943.6780821919</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:AMD67"/>
@@ -2059,7 +3631,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2070,7 +3642,7 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="153" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -2140,7 +3712,7 @@
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="56" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C7" s="56"/>
       <c r="D7" s="56"/>
@@ -2281,7 +3853,7 @@
         <v>11</v>
       </c>
       <c r="B19" s="58" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C19" s="58"/>
       <c r="D19" s="58"/>
@@ -2292,7 +3864,7 @@
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="114" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C20" s="58"/>
       <c r="D20" s="58"/>
@@ -2306,7 +3878,7 @@
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="114" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C21" s="58"/>
       <c r="D21" s="58"/>
@@ -2320,7 +3892,7 @@
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="114" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C22" s="58"/>
       <c r="D22" s="58"/>
@@ -2334,7 +3906,7 @@
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="114" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C23" s="58"/>
       <c r="D23" s="58"/>
@@ -2503,993 +4075,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <sheetPr codeName="Sheet11"/>
-  <dimension ref="A1:K54"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="20.109375" style="13" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" style="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.88671875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" style="13" customWidth="1"/>
-    <col min="5" max="5" width="11.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" style="13" customWidth="1"/>
-    <col min="7" max="7" width="0.6640625" style="13" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" style="13" customWidth="1"/>
-    <col min="9" max="10" width="9.109375" style="13"/>
-    <col min="11" max="11" width="10.6640625" style="13" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.109375" style="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="153" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="B2" s="30"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="B3" s="30"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="30" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="95"/>
-      <c r="B5" s="95"/>
-      <c r="D5" s="96"/>
-      <c r="E5" s="96"/>
-      <c r="H5" s="96" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="63" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" s="21"/>
-      <c r="H6" s="21" t="e">
-        <f>+PL!D12</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="97"/>
-      <c r="E7" s="21"/>
-      <c r="H7" s="21"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="64" t="s">
-        <v>84</v>
-      </c>
-      <c r="E8" s="21"/>
-      <c r="H8" s="98">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="E9" s="21"/>
-      <c r="H9" s="21" t="e">
-        <f>SUM(H6:H8)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="B10" s="30"/>
-      <c r="E10" s="21"/>
-      <c r="H10" s="21"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="D11" s="99"/>
-      <c r="F11" s="191" t="e">
-        <f>'P10'!G22</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H11" s="205" t="e">
-        <f>+F11</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="E12" s="21"/>
-      <c r="H12" s="21" t="e">
-        <f>SUM(H9:H11)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="30" t="s">
-        <v>130</v>
-      </c>
-      <c r="B13" s="30"/>
-      <c r="E13" s="21"/>
-      <c r="H13" s="21"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F14" s="65" t="s">
-        <v>140</v>
-      </c>
-      <c r="H14" s="98" t="e">
-        <f>-E42</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="E15" s="21"/>
-      <c r="H15" s="100" t="e">
-        <f>SUM(H12:H14)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="E16" s="101"/>
-      <c r="H16" s="101"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A17" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="E17" s="101"/>
-      <c r="H17" s="136" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="E18" s="101"/>
-      <c r="H18" s="101"/>
-    </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="102" t="s">
-        <v>89</v>
-      </c>
-      <c r="E19" s="103" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" s="32" t="str">
-        <f>+H17</f>
-        <v>Loss</v>
-      </c>
-      <c r="H19" s="101" t="e">
-        <f>F19*0.3</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
-      <c r="E20" s="101"/>
-      <c r="H20" s="101"/>
-    </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="104" t="s">
-        <v>91</v>
-      </c>
-      <c r="E21" s="101"/>
-      <c r="H21" s="101"/>
-    </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="E22" s="65">
-        <v>24252</v>
-      </c>
-      <c r="F22" s="106">
-        <v>0</v>
-      </c>
-      <c r="G22" s="105"/>
-      <c r="H22" s="106">
-        <f>-SUM(F22:F22)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="3.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D23" s="65"/>
-      <c r="E23" s="101"/>
-      <c r="F23" s="101"/>
-      <c r="G23" s="105"/>
-      <c r="H23" s="101"/>
-    </row>
-    <row r="24" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="E24" s="101"/>
-      <c r="H24" s="107" t="e">
-        <f>SUM(H19:H22)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K24" s="29"/>
-    </row>
-    <row r="25" spans="1:11" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="E25" s="101"/>
-      <c r="H25" s="101"/>
-    </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
-      <c r="E26" s="101"/>
-      <c r="H26" s="101"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A27" s="63" t="s">
-        <v>93</v>
-      </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="101"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="18"/>
-      <c r="H27" s="18"/>
-    </row>
-    <row r="28" spans="1:11" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E28" s="101"/>
-      <c r="H28" s="101"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A29" s="87" t="s">
-        <v>94</v>
-      </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="18"/>
-      <c r="H29" s="18"/>
-    </row>
-    <row r="30" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="18"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="18"/>
-      <c r="H30" s="18"/>
-    </row>
-    <row r="31" spans="1:11" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="108" t="s">
-        <v>95</v>
-      </c>
-      <c r="B31" s="109" t="s">
-        <v>26</v>
-      </c>
-      <c r="C31" s="96" t="s">
-        <v>96</v>
-      </c>
-      <c r="D31" s="110" t="s">
-        <v>131</v>
-      </c>
-      <c r="E31" s="90" t="s">
-        <v>97</v>
-      </c>
-      <c r="F31" s="90" t="s">
-        <v>132</v>
-      </c>
-      <c r="G31" s="90"/>
-      <c r="H31" s="96" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="108"/>
-      <c r="B32" s="109"/>
-      <c r="C32" s="65"/>
-      <c r="D32" s="111"/>
-      <c r="E32" s="111"/>
-      <c r="F32" s="111"/>
-      <c r="G32" s="111"/>
-      <c r="H32" s="65"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A33" s="108" t="s">
-        <v>133</v>
-      </c>
-      <c r="B33" s="109"/>
-      <c r="C33" s="65"/>
-      <c r="D33" s="111"/>
-      <c r="E33" s="111"/>
-      <c r="F33" s="111"/>
-      <c r="G33" s="111"/>
-      <c r="H33" s="65"/>
-    </row>
-    <row r="34" spans="1:8" ht="5.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="108"/>
-      <c r="B34" s="109"/>
-      <c r="C34" s="65"/>
-      <c r="D34" s="111"/>
-      <c r="E34" s="111"/>
-      <c r="F34" s="111"/>
-      <c r="G34" s="111"/>
-      <c r="H34" s="65"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" s="108" t="str">
-        <f>+'P10'!B6</f>
-        <v>Furniture &amp; Fittings</v>
-      </c>
-      <c r="B35" s="167">
-        <f>+'P10'!G6</f>
-        <v>153700</v>
-      </c>
-      <c r="C35" s="65">
-        <v>5</v>
-      </c>
-      <c r="D35" s="140">
-        <v>0</v>
-      </c>
-      <c r="E35" s="139">
-        <f>B35/C35</f>
-        <v>30740</v>
-      </c>
-      <c r="F35" s="139">
-        <f>D35+E35</f>
-        <v>30740</v>
-      </c>
-      <c r="G35" s="111"/>
-      <c r="H35" s="142">
-        <f>B35-F35</f>
-        <v>122960</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" s="192" t="e">
-        <f>+'P10'!B7</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B36" s="167" t="e">
-        <f>+'P10'!G7</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C36" s="65">
-        <v>5</v>
-      </c>
-      <c r="D36" s="201">
-        <v>0</v>
-      </c>
-      <c r="E36" s="199" t="e">
-        <f t="shared" ref="E36:E40" si="0">B36/C36</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F36" s="199" t="e">
-        <f t="shared" ref="F36:F40" si="1">D36+E36</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G36" s="111"/>
-      <c r="H36" s="203" t="e">
-        <f t="shared" ref="H36:H40" si="2">B36-F36</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" s="192" t="e">
-        <f>+'P10'!B8</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B37" s="167" t="e">
-        <f>+'P10'!G8</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C37" s="65">
-        <v>5</v>
-      </c>
-      <c r="D37" s="201">
-        <v>0</v>
-      </c>
-      <c r="E37" s="199" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="F37" s="199" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G37" s="111"/>
-      <c r="H37" s="203" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="192" t="e">
-        <f>+'P10'!B9</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B38" s="167" t="e">
-        <f>+'P10'!G9</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C38" s="188">
-        <v>5</v>
-      </c>
-      <c r="D38" s="201">
-        <v>0</v>
-      </c>
-      <c r="E38" s="199" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="F38" s="199" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G38" s="193"/>
-      <c r="H38" s="203" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="192" t="e">
-        <f>+'P10'!B10</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B39" s="167" t="e">
-        <f>+'P10'!G10</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C39" s="188">
-        <v>5</v>
-      </c>
-      <c r="D39" s="201">
-        <v>0</v>
-      </c>
-      <c r="E39" s="199" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="F39" s="199" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G39" s="193"/>
-      <c r="H39" s="203" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="192" t="e">
-        <f>+'P10'!B11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B40" s="167" t="e">
-        <f>+'P10'!G11</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C40" s="188">
-        <v>5</v>
-      </c>
-      <c r="D40" s="201">
-        <v>0</v>
-      </c>
-      <c r="E40" s="199" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="F40" s="199" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G40" s="193"/>
-      <c r="H40" s="203" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" s="182" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="192"/>
-      <c r="B41" s="200"/>
-      <c r="C41" s="188"/>
-      <c r="D41" s="201"/>
-      <c r="E41" s="199"/>
-      <c r="F41" s="199"/>
-      <c r="G41" s="193"/>
-      <c r="H41" s="203"/>
-    </row>
-    <row r="42" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="B42" s="141" t="e">
-        <f>SUM(B35:B40)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C42" s="113"/>
-      <c r="D42" s="202">
-        <f>SUM(D35:D40)</f>
-        <v>0</v>
-      </c>
-      <c r="E42" s="202" t="e">
-        <f t="shared" ref="E42:H42" si="3">SUM(E35:E40)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F42" s="202" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G42" s="113"/>
-      <c r="H42" s="202" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="18"/>
-      <c r="B43" s="112"/>
-      <c r="C43" s="112"/>
-      <c r="D43" s="112"/>
-      <c r="E43" s="112"/>
-      <c r="F43" s="112"/>
-      <c r="G43" s="112"/>
-      <c r="H43" s="112"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" s="189" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A46" s="184" t="s">
-        <v>175</v>
-      </c>
-      <c r="H46" s="164">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A47" s="184" t="s">
-        <v>176</v>
-      </c>
-      <c r="H47" s="208" t="e">
-        <f>-H15</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A48" s="184"/>
-      <c r="H48" s="164" t="e">
-        <f>SUM(H46:H47)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" s="184"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A50" s="184" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A51" s="184" t="s">
-        <v>178</v>
-      </c>
-      <c r="H51" s="164">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="184" t="s">
-        <v>179</v>
-      </c>
-      <c r="H52" s="164">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A53" s="184" t="s">
-        <v>180</v>
-      </c>
-      <c r="H53" s="209" t="e">
-        <f>SUM(H48:H52)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-  </sheetData>
-  <pageMargins left="0.85" right="0.5" top="0.75" bottom="0.17" header="0.17" footer="0.17"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2A291A8-AC8E-4BB6-A21B-06A29BC55837}">
-  <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="212" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B2" s="158">
-        <v>2328236</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="158"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="212" t="s">
-        <v>185</v>
-      </c>
-      <c r="B4" s="158"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B5" s="162">
-        <v>99975</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="158"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="158"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="212" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B9" s="158"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="158"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="212" t="s">
-        <v>186</v>
-      </c>
-      <c r="B11" s="158"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>156</v>
-      </c>
-      <c r="B12" t="s">
-        <v>157</v>
-      </c>
-      <c r="C12" t="s">
-        <v>158</v>
-      </c>
-      <c r="D12" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="159">
-        <v>45597</v>
-      </c>
-      <c r="B13" s="158">
-        <v>4200</v>
-      </c>
-      <c r="C13" s="158">
-        <f>B13*12/20</f>
-        <v>2520</v>
-      </c>
-      <c r="D13" s="158">
-        <f>C13*3/12</f>
-        <v>630</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="160">
-        <f>SUM(B13:B13)</f>
-        <v>4200</v>
-      </c>
-      <c r="C14" s="161">
-        <f>SUM(C13:C13)</f>
-        <v>2520</v>
-      </c>
-      <c r="D14" s="161">
-        <f>SUM(D13:D13)</f>
-        <v>630</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="158"/>
-      <c r="C15" s="158"/>
-      <c r="D15" s="158"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="25" style="156" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" style="88" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" style="157" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" style="154" bestFit="1" customWidth="1"/>
-    <col min="5" max="9" width="9.109375" style="154"/>
-    <col min="10" max="10" width="11.5546875" style="154" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="154"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="242" t="s">
-        <v>191</v>
-      </c>
-      <c r="B1" s="242"/>
-      <c r="C1" s="242"/>
-    </row>
-    <row r="2" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="242" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="242"/>
-      <c r="C2" s="242"/>
-    </row>
-    <row r="3" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="242" t="s">
-        <v>108</v>
-      </c>
-      <c r="B3" s="242"/>
-      <c r="C3" s="242"/>
-    </row>
-    <row r="4" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A4" s="221" t="s">
-        <v>190</v>
-      </c>
-      <c r="B4" s="213" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="214" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A5" s="215" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="216"/>
-      <c r="C5" s="216"/>
-    </row>
-    <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A6" s="217" t="s">
-        <v>120</v>
-      </c>
-      <c r="B6" s="223">
-        <v>12560</v>
-      </c>
-      <c r="C6" s="216"/>
-    </row>
-    <row r="7" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A7" s="215" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="216"/>
-      <c r="C7" s="216"/>
-      <c r="J7" s="155"/>
-    </row>
-    <row r="8" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A8" s="217" t="s">
-        <v>110</v>
-      </c>
-      <c r="B8" s="216">
-        <f>+PPE!D4</f>
-        <v>153700</v>
-      </c>
-      <c r="C8" s="216"/>
-      <c r="J8" s="155"/>
-    </row>
-    <row r="9" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A9" s="217" t="s">
-        <v>122</v>
-      </c>
-      <c r="B9" s="216"/>
-      <c r="C9" s="216">
-        <f>+PPE!G5</f>
-        <v>28887.178082191782</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A10" s="215" t="s">
-        <v>187</v>
-      </c>
-      <c r="B10" s="216"/>
-      <c r="C10" s="216"/>
-    </row>
-    <row r="11" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="217" t="s">
-        <v>121</v>
-      </c>
-      <c r="B11" s="216"/>
-      <c r="C11" s="216">
-        <f>+B22</f>
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A12" s="217" t="s">
-        <v>100</v>
-      </c>
-      <c r="B12" s="216"/>
-      <c r="C12" s="216">
-        <f>+B23</f>
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="212" t="s">
-        <v>188</v>
-      </c>
-      <c r="B13" s="218"/>
-      <c r="C13" s="219"/>
-    </row>
-    <row r="14" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A14" s="217" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="216"/>
-      <c r="C14" s="216">
-        <f>1000*6</f>
-        <v>6000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A15" s="217" t="s">
-        <v>169</v>
-      </c>
-      <c r="B15" s="216"/>
-      <c r="C15" s="216">
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" s="204" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A16" s="215" t="s">
-        <v>154</v>
-      </c>
-      <c r="B16" s="216"/>
-      <c r="C16" s="219"/>
-    </row>
-    <row r="17" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="220" t="s">
-        <v>170</v>
-      </c>
-      <c r="B17" s="224">
-        <v>112919.5</v>
-      </c>
-      <c r="C17" s="216"/>
-    </row>
-    <row r="18" spans="1:3" s="204" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="217" t="s">
-        <v>107</v>
-      </c>
-      <c r="B18" s="216"/>
-      <c r="C18" s="225">
-        <f>+Working!B2</f>
-        <v>2328236</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="212" t="s">
-        <v>189</v>
-      </c>
-      <c r="B19" s="216"/>
-      <c r="C19" s="216"/>
-    </row>
-    <row r="20" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A20" s="217" t="s">
-        <v>165</v>
-      </c>
-      <c r="B20" s="216">
-        <v>1220000</v>
-      </c>
-      <c r="C20" s="216"/>
-    </row>
-    <row r="21" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A21" s="217" t="s">
-        <v>142</v>
-      </c>
-      <c r="B21" s="216">
-        <v>1000</v>
-      </c>
-      <c r="C21" s="216"/>
-    </row>
-    <row r="22" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A22" s="217" t="s">
-        <v>121</v>
-      </c>
-      <c r="B22" s="216">
-        <v>15000</v>
-      </c>
-      <c r="C22" s="216"/>
-    </row>
-    <row r="23" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A23" s="217" t="s">
-        <v>100</v>
-      </c>
-      <c r="B23" s="216">
-        <v>25000</v>
-      </c>
-      <c r="C23" s="216"/>
-    </row>
-    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="221" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" s="222">
-        <f>SUM(B5:B23)</f>
-        <v>1540179.5</v>
-      </c>
-      <c r="C24" s="222">
-        <f>SUM(C5:C23)</f>
-        <v>3403123.1780821919</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="14.4" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="88">
-        <f>B24-C24</f>
-        <v>-1862943.6780821919</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:J23"/>
@@ -3509,7 +4095,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3539,7 +4125,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -3586,7 +4172,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E7" s="241">
         <v>0</v>
@@ -3634,7 +4220,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="E11" s="239">
         <v>0</v>
@@ -3659,7 +4245,7 @@
     </row>
     <row r="13" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E13" s="171">
         <f>SUM(E7:E11)</f>
@@ -3734,7 +4320,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:I43"/>
@@ -3754,7 +4340,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="170" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="E1" s="170"/>
       <c r="F1" s="170"/>
@@ -3821,13 +4407,13 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B9" s="172" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C9" s="172"/>
       <c r="D9" s="172"/>
       <c r="F9" s="176"/>
       <c r="G9" s="195" t="e">
-        <f>'P09'!D22</f>
+        <f>'P09'!#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
@@ -3847,7 +4433,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B12" s="172" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="C12" s="172"/>
       <c r="D12" s="172"/>
@@ -3859,7 +4445,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B13" s="172" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="C13" s="172"/>
       <c r="D13" s="172"/>
@@ -3871,7 +4457,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B14" s="172" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C14" s="172"/>
       <c r="D14" s="172"/>
@@ -3936,7 +4522,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B22" s="169" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F22" s="176"/>
       <c r="G22" s="195" t="e">
@@ -4021,16 +4607,16 @@
     </row>
     <row r="32" spans="1:7" s="169" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="166" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C32" s="163"/>
       <c r="F32" s="186"/>
     </row>
     <row r="33" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B33" s="179" t="s">
-        <v>144</v>
-      </c>
-      <c r="G33" s="243">
+        <v>138</v>
+      </c>
+      <c r="G33" s="242">
         <v>0</v>
       </c>
     </row>
@@ -4043,13 +4629,13 @@
     <row r="35" spans="1:9" s="169" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
     <row r="36" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="166" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="G36" s="186"/>
     </row>
     <row r="37" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B37" s="179" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D37" s="178"/>
       <c r="E37" s="178"/>
@@ -4087,7 +4673,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:G24"/>
@@ -4104,7 +4690,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4122,7 +4708,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -4170,9 +4756,9 @@
         <v>5</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="121" t="e">
-        <f>-'P09'!D26</f>
-        <v>#REF!</v>
+      <c r="D8" s="121">
+        <f>-'P09'!D13</f>
+        <v>-40000</v>
       </c>
       <c r="G8" s="5"/>
     </row>
@@ -4191,7 +4777,7 @@
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="123" t="e">
-        <f>-'P09'!D30</f>
+        <f>-'P09'!D17</f>
         <v>#REF!</v>
       </c>
     </row>
@@ -4219,7 +4805,7 @@
         <v>7</v>
       </c>
       <c r="D14" s="123">
-        <f>-'P09'!D34</f>
+        <f>-'P09'!D21</f>
         <v>-1000</v>
       </c>
     </row>
@@ -4228,7 +4814,7 @@
     </row>
     <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="12" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="D16" s="124" t="e">
         <f>SUM(D12:D14)</f>
@@ -4262,7 +4848,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:ALX51"/>
@@ -4284,7 +4870,7 @@
   <sheetData>
     <row r="1" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4304,7 +4890,7 @@
     </row>
     <row r="3" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -4345,7 +4931,7 @@
     </row>
     <row r="8" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A8" s="18" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C8" s="3">
         <v>8</v>
@@ -5375,7 +5961,7 @@
     </row>
     <row r="12" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A12" s="143" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="B12" s="143"/>
       <c r="C12" s="210"/>
@@ -19430,7 +20016,7 @@
     </row>
     <row r="26" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="A26" s="147" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C26" s="3">
         <v>11</v>
@@ -41653,7 +42239,7 @@
     </row>
     <row r="50" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A50" s="28" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="B50" s="18"/>
       <c r="C50" s="18"/>
@@ -42660,7 +43246,7 @@
     </row>
     <row r="51" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A51" s="28" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="B51" s="18"/>
       <c r="C51" s="18"/>
@@ -43671,10 +44257,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet8"/>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" style="2" customWidth="1"/>
@@ -43691,7 +44277,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
@@ -43715,7 +44301,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
@@ -43765,7 +44351,7 @@
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="2" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D7" s="73">
         <f>+TB!C18</f>
@@ -43805,909 +44391,105 @@
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
       <c r="B11" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="73">
-        <f>TB!B20</f>
-        <v>1220000</v>
+        <v>133</v>
+      </c>
+      <c r="C11" s="76"/>
+      <c r="D11" s="120">
+        <f>+TB!B22</f>
+        <v>15000</v>
       </c>
       <c r="E11" s="1"/>
-      <c r="F11" s="51"/>
+      <c r="F11" s="38"/>
       <c r="G11" s="70"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="2" t="s">
-        <v>135</v>
+        <v>99</v>
       </c>
       <c r="C12" s="76"/>
-      <c r="D12" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
+      <c r="D12" s="120">
+        <f>+TB!B23</f>
+        <v>25000</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="38"/>
       <c r="G12" s="70"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" s="3"/>
-      <c r="B13" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C13" s="76"/>
-      <c r="D13" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="70"/>
+    <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D13" s="116">
+        <f>SUM(D11:D12)</f>
+        <v>40000</v>
+      </c>
+      <c r="E13" s="46"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="75"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="3"/>
-      <c r="B14" s="2" t="s">
-        <v>161</v>
-      </c>
+    <row r="14" spans="1:9" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="6"/>
       <c r="C14" s="76"/>
-      <c r="D14" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E14" s="1"/>
+      <c r="D14" s="120"/>
       <c r="F14" s="38"/>
-      <c r="G14" s="70"/>
+      <c r="G14" s="66"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="3"/>
-      <c r="B15" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C15" s="76"/>
-      <c r="D15" s="120" t="e">
+      <c r="A15" s="3">
+        <v>6</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B16" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="121" t="e">
         <f>+TB!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="E15" s="1"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="70"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="3"/>
-      <c r="B16" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C16" s="76"/>
-      <c r="D16" s="120" t="e">
-        <f>+TB!#REF!+TB!#REF!</f>
+    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B17" s="1"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="116" t="e">
+        <f>SUM(D16)</f>
         <v>#REF!</v>
       </c>
-      <c r="E16" s="1"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="70"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="3"/>
-      <c r="B17" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C17" s="76"/>
-      <c r="D17" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="38"/>
-      <c r="G17" s="70"/>
+    <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="1"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="121"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="3"/>
-      <c r="B18" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C18" s="76"/>
-      <c r="D18" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E18" s="1"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="70"/>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="9">
+        <v>7</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="3"/>
-      <c r="B19" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C19" s="76"/>
-      <c r="D19" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E19" s="1"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="70"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="3"/>
-      <c r="B20" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C20" s="76"/>
-      <c r="D20" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="70"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="3"/>
-      <c r="B21" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C21" s="76"/>
-      <c r="D21" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="70"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="3"/>
-      <c r="B22" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C22" s="76"/>
-      <c r="D22" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="70"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="3"/>
-      <c r="B23" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C23" s="76"/>
-      <c r="D23" s="120" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="38"/>
-      <c r="G23" s="70"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="3"/>
-      <c r="B24" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C24" s="76"/>
-      <c r="D24" s="120">
-        <f>+TB!B22</f>
-        <v>15000</v>
-      </c>
-      <c r="E24" s="1"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="70"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="3"/>
-      <c r="B25" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C25" s="76"/>
-      <c r="D25" s="120">
-        <f>+TB!B23</f>
-        <v>25000</v>
-      </c>
-      <c r="E25" s="1"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="70"/>
-    </row>
-    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D26" s="116" t="e">
-        <f>SUM(D11:D25)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E26" s="46"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="75"/>
-    </row>
-    <row r="27" spans="1:7" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="6"/>
-      <c r="C27" s="76"/>
-      <c r="D27" s="120"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="66"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="3">
-        <v>6</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C28" s="3"/>
-      <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B29" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C29" s="3"/>
-      <c r="D29" s="121" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="1"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="116" t="e">
-        <f>SUM(D29)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="1"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="121"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="9">
-        <v>7</v>
-      </c>
-      <c r="B32" s="30" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" s="65"/>
-      <c r="B33" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="D33" s="115">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="65"/>
+      <c r="B20" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D20" s="115">
         <f>TB!B21</f>
         <v>1000</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D34" s="117">
-        <f>+D33</f>
+    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D21" s="117">
+        <f>+D20</f>
         <v>1000</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-  </sheetData>
-  <pageMargins left="0.85" right="0.5" top="0.75" bottom="0.17" header="0.17" footer="0.17"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <sheetPr codeName="Sheet9"/>
-  <dimension ref="A1:AMD52"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="5" style="15" customWidth="1"/>
-    <col min="2" max="2" width="25" style="2" customWidth="1"/>
-    <col min="3" max="3" width="6.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.109375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.5546875" style="38" customWidth="1"/>
-    <col min="6" max="6" width="0.6640625" style="17" customWidth="1"/>
-    <col min="7" max="7" width="13" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" style="2" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="0.6640625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="13.33203125" style="2" customWidth="1"/>
-    <col min="11" max="1018" width="9.109375" style="2"/>
-    <col min="1019" max="16384" width="9.109375" style="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="153" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" s="79" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="80"/>
-      <c r="B3" s="92"/>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" s="36">
-        <v>8</v>
-      </c>
-      <c r="B4" s="92" t="s">
-        <v>143</v>
-      </c>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-    </row>
-    <row r="5" spans="1:13" ht="28.8" x14ac:dyDescent="0.35">
-      <c r="A5" s="36"/>
-      <c r="B5" s="96" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="39" t="s">
-        <v>111</v>
-      </c>
-      <c r="F5" s="39"/>
-      <c r="G5" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="41" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="42"/>
-      <c r="J5" s="43" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="36"/>
-      <c r="B6" s="44" t="str">
-        <f>+TB!A8</f>
-        <v>Furniture &amp; Fittings</v>
-      </c>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="131">
-        <v>0</v>
-      </c>
-      <c r="F6" s="131"/>
-      <c r="G6" s="131">
-        <f>TB!B8</f>
-        <v>153700</v>
-      </c>
-      <c r="H6" s="118"/>
-      <c r="I6" s="119"/>
-      <c r="J6" s="118">
-        <f>SUM(E6:G6)</f>
-        <v>153700</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" s="36"/>
-      <c r="B7" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="131">
-        <v>0</v>
-      </c>
-      <c r="F7" s="131"/>
-      <c r="G7" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H7" s="118"/>
-      <c r="I7" s="119"/>
-      <c r="J7" s="118" t="e">
-        <f t="shared" ref="J7:J11" si="0">SUM(E7:G7)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" s="36"/>
-      <c r="B8" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="131">
-        <v>0</v>
-      </c>
-      <c r="F8" s="131"/>
-      <c r="G8" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H8" s="118"/>
-      <c r="I8" s="119"/>
-      <c r="J8" s="118" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" s="36"/>
-      <c r="B9" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="131">
-        <v>0</v>
-      </c>
-      <c r="F9" s="131"/>
-      <c r="G9" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H9" s="118"/>
-      <c r="I9" s="119"/>
-      <c r="J9" s="118" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="36"/>
-      <c r="B10" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="131">
-        <v>0</v>
-      </c>
-      <c r="F10" s="131"/>
-      <c r="G10" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H10" s="118"/>
-      <c r="I10" s="119"/>
-      <c r="J10" s="118" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" s="36"/>
-      <c r="B11" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="131">
-        <v>0</v>
-      </c>
-      <c r="F11" s="131"/>
-      <c r="G11" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H11" s="118"/>
-      <c r="I11" s="119"/>
-      <c r="J11" s="118" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="36"/>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="132">
-        <f>SUM(E6:E11)</f>
-        <v>0</v>
-      </c>
-      <c r="F12" s="131"/>
-      <c r="G12" s="132" t="e">
-        <f>SUM(G6:G11)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H12" s="118"/>
-      <c r="I12" s="119"/>
-      <c r="J12" s="132" t="e">
-        <f>SUM(J6:J11)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="36"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="47"/>
-      <c r="G13" s="47"/>
-      <c r="H13" s="47"/>
-      <c r="I13" s="47"/>
-      <c r="J13" s="46"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" s="36"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-    </row>
-    <row r="15" spans="1:13" ht="28.8" x14ac:dyDescent="0.35">
-      <c r="A15" s="36"/>
-      <c r="B15" s="36" t="s">
-        <v>113</v>
-      </c>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="39" t="s">
-        <v>111</v>
-      </c>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" s="41" t="s">
-        <v>14</v>
-      </c>
-      <c r="I15" s="42"/>
-      <c r="J15" s="43" t="s">
-        <v>112</v>
-      </c>
-      <c r="M15" s="49"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A16" s="50"/>
-      <c r="B16" s="44" t="str">
-        <f t="shared" ref="B16:B21" si="1">B6</f>
-        <v>Furniture &amp; Fittings</v>
-      </c>
-      <c r="C16" s="44"/>
-      <c r="D16" s="44"/>
-      <c r="E16" s="131">
-        <v>0</v>
-      </c>
-      <c r="F16" s="131"/>
-      <c r="G16" s="118">
-        <f>PPE!G4</f>
-        <v>28887.178082191782</v>
-      </c>
-      <c r="H16" s="118"/>
-      <c r="I16" s="119"/>
-      <c r="J16" s="137">
-        <f>SUM(E16:G16)</f>
-        <v>28887.178082191782</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="50"/>
-      <c r="B17" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="131">
-        <v>0</v>
-      </c>
-      <c r="F17" s="131"/>
-      <c r="G17" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H17" s="118"/>
-      <c r="I17" s="119"/>
-      <c r="J17" s="137" t="e">
-        <f t="shared" ref="J17:J21" si="2">SUM(E17:G17)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="50"/>
-      <c r="B18" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C18" s="44"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="131">
-        <v>0</v>
-      </c>
-      <c r="F18" s="131"/>
-      <c r="G18" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H18" s="118"/>
-      <c r="I18" s="119"/>
-      <c r="J18" s="137" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="50"/>
-      <c r="B19" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="131">
-        <v>0</v>
-      </c>
-      <c r="F19" s="131"/>
-      <c r="G19" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H19" s="118"/>
-      <c r="I19" s="119"/>
-      <c r="J19" s="137" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="50"/>
-      <c r="B20" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="131">
-        <v>0</v>
-      </c>
-      <c r="F20" s="131"/>
-      <c r="G20" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H20" s="118"/>
-      <c r="I20" s="119"/>
-      <c r="J20" s="137" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="50"/>
-      <c r="B21" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="131">
-        <v>0</v>
-      </c>
-      <c r="F21" s="131"/>
-      <c r="G21" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H21" s="118"/>
-      <c r="I21" s="119"/>
-      <c r="J21" s="137" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="50"/>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="132">
-        <f>SUM(E16:E21)</f>
-        <v>0</v>
-      </c>
-      <c r="F22" s="131"/>
-      <c r="G22" s="173" t="e">
-        <f>SUM(G16:G21)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H22" s="118"/>
-      <c r="I22" s="119"/>
-      <c r="J22" s="132" t="e">
-        <f>SUM(J16:J21)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="36"/>
-      <c r="B23" s="44"/>
-      <c r="C23" s="44"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="38"/>
-    </row>
-    <row r="24" spans="1:10" ht="28.8" x14ac:dyDescent="0.35">
-      <c r="A24" s="2"/>
-      <c r="B24" s="96" t="s">
-        <v>80</v>
-      </c>
-      <c r="J24" s="90" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="2"/>
-      <c r="B25" s="44" t="str">
-        <f t="shared" ref="B25:B30" si="3">B16</f>
-        <v>Furniture &amp; Fittings</v>
-      </c>
-      <c r="J25" s="74">
-        <f t="shared" ref="J25:J30" si="4">J6-J16</f>
-        <v>124812.82191780822</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="2"/>
-      <c r="B26" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J26" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="2"/>
-      <c r="B27" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J27" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="2"/>
-      <c r="B28" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J28" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="2"/>
-      <c r="B29" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J29" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="2"/>
-      <c r="B30" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J30" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="2"/>
-      <c r="J31" s="138" t="e">
-        <f>SUM(J25:J30)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="2"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" s="2"/>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" s="2"/>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" s="2"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" s="2"/>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" s="2"/>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" s="2"/>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" s="2"/>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" s="2"/>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" s="2"/>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" s="2"/>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" s="2"/>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" s="2"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" s="2"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" s="2"/>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" s="2"/>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" s="2"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" s="2"/>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" s="2"/>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" s="2"/>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" s="2"/>
-    </row>
+    <row r="22" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.85" right="0.5" top="0.75" bottom="0.17" header="0.17" footer="0.17"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: enhance report data handling in FinancialReportsPage component
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626D41D6-5090-429E-AA7A-AD7E9D920402}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E1B289-3DA5-4DF2-BB49-8FD4B9871809}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPE" sheetId="24" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="180">
   <si>
     <t>STATEMENT OF FINANCIAL POSITION</t>
   </si>
@@ -625,7 +625,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -802,6 +802,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1214,7 +1220,6 @@
     <xf numFmtId="43" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1249,7 +1254,6 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1337,10 +1341,6 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1423,6 +1423,14 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="23">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1909,92 +1917,92 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.109375" style="227" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.77734375" style="227" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" style="227" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" style="227" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" style="227" customWidth="1"/>
-    <col min="6" max="6" width="12" style="227" customWidth="1"/>
-    <col min="7" max="7" width="12.5546875" style="227" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="227"/>
-    <col min="9" max="9" width="10.6640625" style="227" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="227"/>
+    <col min="1" max="1" width="19.109375" style="223" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" style="223" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" style="223" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" style="223" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" style="223" customWidth="1"/>
+    <col min="6" max="6" width="12" style="223" customWidth="1"/>
+    <col min="7" max="7" width="12.5546875" style="223" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" style="223"/>
+    <col min="9" max="9" width="10.6640625" style="223" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="223"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="226" t="s">
+      <c r="A1" s="222" t="s">
         <v>112</v>
       </c>
-      <c r="C1" s="226"/>
+      <c r="C1" s="222"/>
     </row>
     <row r="3" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="228" t="s">
+      <c r="A3" s="224" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="229" t="s">
+      <c r="B3" s="225" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="228" t="s">
+      <c r="C3" s="224" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="230" t="s">
+      <c r="D3" s="226" t="s">
         <v>107</v>
       </c>
-      <c r="E3" s="229" t="s">
+      <c r="E3" s="225" t="s">
         <v>115</v>
       </c>
-      <c r="F3" s="229" t="s">
+      <c r="F3" s="225" t="s">
         <v>154</v>
       </c>
-      <c r="G3" s="229" t="s">
+      <c r="G3" s="225" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="231" t="s">
+      <c r="A4" s="227" t="s">
         <v>108</v>
       </c>
-      <c r="B4" s="232">
+      <c r="B4" s="228">
         <v>45385</v>
       </c>
-      <c r="C4" s="233">
+      <c r="C4" s="229">
         <v>5</v>
       </c>
-      <c r="D4" s="234">
+      <c r="D4" s="230">
         <v>153700</v>
       </c>
-      <c r="E4" s="232">
+      <c r="E4" s="228">
         <v>45728</v>
       </c>
-      <c r="F4" s="234">
+      <c r="F4" s="230">
         <f t="shared" ref="F4" si="0">E4-B4</f>
         <v>343</v>
       </c>
-      <c r="G4" s="235">
+      <c r="G4" s="231">
         <f>(D4/C4)*(F4/365)</f>
         <v>28887.178082191782</v>
       </c>
-      <c r="I4" s="236"/>
+      <c r="I4" s="232"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="230" t="s">
+      <c r="A5" s="226" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="237"/>
-      <c r="C5" s="237"/>
-      <c r="D5" s="238">
+      <c r="B5" s="233"/>
+      <c r="C5" s="233"/>
+      <c r="D5" s="234">
         <f>SUM(D4:D4)</f>
         <v>153700</v>
       </c>
-      <c r="E5" s="237"/>
-      <c r="F5" s="237"/>
-      <c r="G5" s="238">
+      <c r="E5" s="233"/>
+      <c r="F5" s="233"/>
+      <c r="G5" s="234">
         <f>SUM(G4:G4)</f>
         <v>28887.178082191782</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D7" s="236"/>
+      <c r="D7" s="232"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2004,7 +2012,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet9"/>
-  <dimension ref="A1:AMD52"/>
+  <dimension ref="A1:AMD37"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" style="15" customWidth="1"/>
@@ -2033,7 +2041,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="153" t="s">
+      <c r="J1" s="152" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2118,103 +2126,79 @@
         <v>153700</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="36"/>
-      <c r="B7" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="B7" s="44"/>
       <c r="C7" s="44"/>
       <c r="D7" s="44"/>
-      <c r="E7" s="131">
+      <c r="E7" s="132">
+        <f>SUM(E6:E6)</f>
         <v>0</v>
       </c>
       <c r="F7" s="131"/>
-      <c r="G7" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
+      <c r="G7" s="132">
+        <f>SUM(G6:G6)</f>
+        <v>153700</v>
       </c>
       <c r="H7" s="118"/>
       <c r="I7" s="119"/>
-      <c r="J7" s="118" t="e">
-        <f t="shared" ref="J7:J11" si="0">SUM(E7:G7)</f>
-        <v>#REF!</v>
+      <c r="J7" s="132">
+        <f>SUM(J6:J6)</f>
+        <v>153700</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A8" s="36"/>
-      <c r="B8" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="131">
-        <v>0</v>
-      </c>
-      <c r="F8" s="131"/>
-      <c r="G8" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H8" s="118"/>
-      <c r="I8" s="119"/>
-      <c r="J8" s="118" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="47"/>
+      <c r="G8" s="47"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="47"/>
+      <c r="J8" s="46"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="36"/>
-      <c r="B9" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="131">
-        <v>0</v>
-      </c>
-      <c r="F9" s="131"/>
-      <c r="G9" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H9" s="118"/>
-      <c r="I9" s="119"/>
-      <c r="J9" s="118" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="47"/>
+      <c r="F9" s="47"/>
+      <c r="G9" s="47"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" ht="28.8" x14ac:dyDescent="0.35">
       <c r="A10" s="36"/>
-      <c r="B10" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="131">
-        <v>0</v>
-      </c>
-      <c r="F10" s="131"/>
-      <c r="G10" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H10" s="118"/>
-      <c r="I10" s="119"/>
-      <c r="J10" s="118" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
+      <c r="B10" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="F10" s="39"/>
+      <c r="G10" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="41" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="42"/>
+      <c r="J10" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="M10" s="49"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" s="36"/>
-      <c r="B11" s="44" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
+      <c r="A11" s="50"/>
+      <c r="B11" s="44" t="str">
+        <f>B6</f>
+        <v>Furniture &amp; Fittings</v>
       </c>
       <c r="C11" s="44"/>
       <c r="D11" s="44"/>
@@ -2222,339 +2206,123 @@
         <v>0</v>
       </c>
       <c r="F11" s="131"/>
-      <c r="G11" s="131" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
+      <c r="G11" s="118">
+        <f>PPE!G4</f>
+        <v>28887.178082191782</v>
       </c>
       <c r="H11" s="118"/>
       <c r="I11" s="119"/>
-      <c r="J11" s="118" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
+      <c r="J11" s="137">
+        <f>SUM(E11:G11)</f>
+        <v>28887.178082191782</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="36"/>
+      <c r="A12" s="50"/>
       <c r="B12" s="44"/>
       <c r="C12" s="44"/>
       <c r="D12" s="44"/>
       <c r="E12" s="132">
-        <f>SUM(E6:E11)</f>
+        <f>SUM(E11:E11)</f>
         <v>0</v>
       </c>
       <c r="F12" s="131"/>
-      <c r="G12" s="132" t="e">
-        <f>SUM(G6:G11)</f>
-        <v>#REF!</v>
+      <c r="G12" s="171">
+        <f>SUM(G11:G11)</f>
+        <v>28887.178082191782</v>
       </c>
       <c r="H12" s="118"/>
       <c r="I12" s="119"/>
-      <c r="J12" s="132" t="e">
-        <f>SUM(J6:J11)</f>
-        <v>#REF!</v>
+      <c r="J12" s="132">
+        <f>SUM(J11:J11)</f>
+        <v>28887.178082191782</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A13" s="36"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="47"/>
-      <c r="G13" s="47"/>
-      <c r="H13" s="47"/>
-      <c r="I13" s="47"/>
-      <c r="J13" s="46"/>
+      <c r="B13" s="44"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="51"/>
+      <c r="H13" s="48"/>
+      <c r="I13" s="46"/>
+      <c r="J13" s="38"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" s="36"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
+    <row r="14" spans="1:13" ht="28.8" x14ac:dyDescent="0.35">
+      <c r="A14" s="2"/>
+      <c r="B14" s="96" t="s">
+        <v>80</v>
+      </c>
+      <c r="J14" s="90" t="s">
+        <v>132</v>
+      </c>
     </row>
-    <row r="15" spans="1:13" ht="28.8" x14ac:dyDescent="0.35">
-      <c r="A15" s="36"/>
-      <c r="B15" s="36" t="s">
-        <v>111</v>
-      </c>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="39" t="s">
-        <v>109</v>
-      </c>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" s="41" t="s">
-        <v>14</v>
-      </c>
-      <c r="I15" s="42"/>
-      <c r="J15" s="43" t="s">
-        <v>110</v>
-      </c>
-      <c r="M15" s="49"/>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A15" s="2"/>
+      <c r="B15" s="44" t="str">
+        <f>B11</f>
+        <v>Furniture &amp; Fittings</v>
+      </c>
+      <c r="J15" s="74">
+        <f>J6-J11</f>
+        <v>124812.82191780822</v>
+      </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A16" s="50"/>
-      <c r="B16" s="44" t="str">
-        <f t="shared" ref="B16:B21" si="1">B6</f>
-        <v>Furniture &amp; Fittings</v>
-      </c>
-      <c r="C16" s="44"/>
-      <c r="D16" s="44"/>
-      <c r="E16" s="131">
-        <v>0</v>
-      </c>
-      <c r="F16" s="131"/>
-      <c r="G16" s="118">
-        <f>PPE!G4</f>
-        <v>28887.178082191782</v>
-      </c>
-      <c r="H16" s="118"/>
-      <c r="I16" s="119"/>
-      <c r="J16" s="137">
-        <f>SUM(E16:G16)</f>
-        <v>28887.178082191782</v>
+    <row r="16" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="2"/>
+      <c r="J16" s="138">
+        <f>SUM(J15:J15)</f>
+        <v>124812.82191780822</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="50"/>
-      <c r="B17" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="131">
-        <v>0</v>
-      </c>
-      <c r="F17" s="131"/>
-      <c r="G17" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H17" s="118"/>
-      <c r="I17" s="119"/>
-      <c r="J17" s="137" t="e">
-        <f t="shared" ref="J17:J21" si="2">SUM(E17:G17)</f>
-        <v>#REF!</v>
-      </c>
+    <row r="17" spans="1:1" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="2"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="50"/>
-      <c r="B18" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C18" s="44"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="131">
-        <v>0</v>
-      </c>
-      <c r="F18" s="131"/>
-      <c r="G18" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H18" s="118"/>
-      <c r="I18" s="119"/>
-      <c r="J18" s="137" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="2"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="50"/>
-      <c r="B19" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="131">
-        <v>0</v>
-      </c>
-      <c r="F19" s="131"/>
-      <c r="G19" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H19" s="118"/>
-      <c r="I19" s="119"/>
-      <c r="J19" s="137" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="2"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="50"/>
-      <c r="B20" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="131">
-        <v>0</v>
-      </c>
-      <c r="F20" s="131"/>
-      <c r="G20" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H20" s="118"/>
-      <c r="I20" s="119"/>
-      <c r="J20" s="137" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="2"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="50"/>
-      <c r="B21" s="44" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="131">
-        <v>0</v>
-      </c>
-      <c r="F21" s="131"/>
-      <c r="G21" s="118" t="e">
-        <f>PPE!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H21" s="118"/>
-      <c r="I21" s="119"/>
-      <c r="J21" s="137" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2"/>
     </row>
-    <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="50"/>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="132">
-        <f>SUM(E16:E21)</f>
-        <v>0</v>
-      </c>
-      <c r="F22" s="131"/>
-      <c r="G22" s="173" t="e">
-        <f>SUM(G16:G21)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H22" s="118"/>
-      <c r="I22" s="119"/>
-      <c r="J22" s="132" t="e">
-        <f>SUM(J16:J21)</f>
-        <v>#REF!</v>
-      </c>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="2"/>
     </row>
-    <row r="23" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="36"/>
-      <c r="B23" s="44"/>
-      <c r="C23" s="44"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="38"/>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="2"/>
     </row>
-    <row r="24" spans="1:10" ht="28.8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" s="2"/>
-      <c r="B24" s="96" t="s">
-        <v>80</v>
-      </c>
-      <c r="J24" s="90" t="s">
-        <v>132</v>
-      </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
-      <c r="B25" s="44" t="str">
-        <f t="shared" ref="B25:B30" si="3">B16</f>
-        <v>Furniture &amp; Fittings</v>
-      </c>
-      <c r="J25" s="74">
-        <f t="shared" ref="J25:J30" si="4">J6-J16</f>
-        <v>124812.82191780822</v>
-      </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
-      <c r="B26" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J26" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" s="2"/>
-      <c r="B27" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J27" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" s="2"/>
-      <c r="B28" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J28" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" s="2"/>
-      <c r="B29" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J29" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" s="2"/>
-      <c r="B30" s="44" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="J30" s="74" t="e">
-        <f t="shared" si="4"/>
-        <v>#REF!</v>
-      </c>
     </row>
-    <row r="31" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" s="2"/>
-      <c r="J31" s="138" t="e">
-        <f>SUM(J25:J30)</f>
-        <v>#REF!</v>
-      </c>
     </row>
-    <row r="32" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" s="2"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
@@ -2571,51 +2339,6 @@
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" s="2"/>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" s="2"/>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" s="2"/>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" s="2"/>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" s="2"/>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" s="2"/>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" s="2"/>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" s="2"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" s="2"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" s="2"/>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" s="2"/>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" s="2"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" s="2"/>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" s="2"/>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" s="2"/>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.85" right="0.5" top="0.75" bottom="0.17" header="0.17" footer="0.17"/>
@@ -2649,7 +2372,7 @@
       <c r="B1" s="30"/>
       <c r="F1" s="93"/>
       <c r="G1" s="94"/>
-      <c r="H1" s="153" t="s">
+      <c r="H1" s="152" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2684,9 +2407,9 @@
         <v>83</v>
       </c>
       <c r="E6" s="21"/>
-      <c r="H6" s="21" t="e">
+      <c r="H6" s="21">
         <f>+PL!D12</f>
-        <v>#REF!</v>
+        <v>2124756</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -2705,9 +2428,9 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="E9" s="21"/>
-      <c r="H9" s="21" t="e">
+      <c r="H9" s="21">
         <f>SUM(H6:H8)</f>
-        <v>#REF!</v>
+        <v>2124756</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -2723,20 +2446,20 @@
         <v>127</v>
       </c>
       <c r="D11" s="99"/>
-      <c r="F11" s="191" t="e">
-        <f>'P10'!G22</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H11" s="205" t="e">
+      <c r="F11" s="189">
+        <f>'P10'!G12</f>
+        <v>28887.178082191782</v>
+      </c>
+      <c r="H11" s="203">
         <f>+F11</f>
-        <v>#REF!</v>
+        <v>28887.178082191782</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="E12" s="21"/>
-      <c r="H12" s="21" t="e">
+      <c r="H12" s="21">
         <f>SUM(H9:H11)</f>
-        <v>#REF!</v>
+        <v>2153643.1780821919</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -2954,7 +2677,7 @@
         <f>+'P10'!B6</f>
         <v>Furniture &amp; Fittings</v>
       </c>
-      <c r="B35" s="167">
+      <c r="B35" s="165">
         <f>+'P10'!G6</f>
         <v>153700</v>
       </c>
@@ -2979,159 +2702,159 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" s="192" t="e">
-        <f>+'P10'!B7</f>
+      <c r="A36" s="190" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B36" s="167" t="e">
-        <f>+'P10'!G7</f>
+      <c r="B36" s="165" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="C36" s="65">
         <v>5</v>
       </c>
-      <c r="D36" s="201">
+      <c r="D36" s="199">
         <v>0</v>
       </c>
-      <c r="E36" s="199" t="e">
+      <c r="E36" s="197" t="e">
         <f t="shared" ref="E36:E40" si="0">B36/C36</f>
         <v>#REF!</v>
       </c>
-      <c r="F36" s="199" t="e">
+      <c r="F36" s="197" t="e">
         <f t="shared" ref="F36:F40" si="1">D36+E36</f>
         <v>#REF!</v>
       </c>
       <c r="G36" s="111"/>
-      <c r="H36" s="203" t="e">
+      <c r="H36" s="201" t="e">
         <f t="shared" ref="H36:H40" si="2">B36-F36</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" s="192" t="e">
-        <f>+'P10'!B8</f>
+      <c r="A37" s="190" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B37" s="167" t="e">
-        <f>+'P10'!G8</f>
+      <c r="B37" s="165" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="C37" s="65">
         <v>5</v>
       </c>
-      <c r="D37" s="201">
+      <c r="D37" s="199">
         <v>0</v>
       </c>
-      <c r="E37" s="199" t="e">
+      <c r="E37" s="197" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F37" s="199" t="e">
+      <c r="F37" s="197" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
       <c r="G37" s="111"/>
-      <c r="H37" s="203" t="e">
+      <c r="H37" s="201" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="192" t="e">
-        <f>+'P10'!B9</f>
+    <row r="38" spans="1:8" s="180" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="190" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B38" s="167" t="e">
-        <f>+'P10'!G9</f>
+      <c r="B38" s="165" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="C38" s="188">
+      <c r="C38" s="186">
         <v>5</v>
       </c>
-      <c r="D38" s="201">
+      <c r="D38" s="199">
         <v>0</v>
       </c>
-      <c r="E38" s="199" t="e">
+      <c r="E38" s="197" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F38" s="199" t="e">
+      <c r="F38" s="197" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G38" s="193"/>
-      <c r="H38" s="203" t="e">
+      <c r="G38" s="191"/>
+      <c r="H38" s="201" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="39" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="192" t="e">
-        <f>+'P10'!B10</f>
+    <row r="39" spans="1:8" s="180" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="190" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B39" s="167" t="e">
-        <f>+'P10'!G10</f>
+      <c r="B39" s="165" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="C39" s="188">
+      <c r="C39" s="186">
         <v>5</v>
       </c>
-      <c r="D39" s="201">
+      <c r="D39" s="199">
         <v>0</v>
       </c>
-      <c r="E39" s="199" t="e">
+      <c r="E39" s="197" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F39" s="199" t="e">
+      <c r="F39" s="197" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G39" s="193"/>
-      <c r="H39" s="203" t="e">
+      <c r="G39" s="191"/>
+      <c r="H39" s="201" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="40" spans="1:8" s="182" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="192" t="e">
-        <f>+'P10'!B11</f>
+    <row r="40" spans="1:8" s="180" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="190" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B40" s="167" t="e">
-        <f>+'P10'!G11</f>
+      <c r="B40" s="165" t="e">
+        <f>+'P10'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="C40" s="188">
+      <c r="C40" s="186">
         <v>5</v>
       </c>
-      <c r="D40" s="201">
+      <c r="D40" s="199">
         <v>0</v>
       </c>
-      <c r="E40" s="199" t="e">
+      <c r="E40" s="197" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="F40" s="199" t="e">
+      <c r="F40" s="197" t="e">
         <f t="shared" si="1"/>
         <v>#REF!</v>
       </c>
-      <c r="G40" s="193"/>
-      <c r="H40" s="203" t="e">
+      <c r="G40" s="191"/>
+      <c r="H40" s="201" t="e">
         <f t="shared" si="2"/>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="41" spans="1:8" s="182" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="192"/>
-      <c r="B41" s="200"/>
-      <c r="C41" s="188"/>
-      <c r="D41" s="201"/>
-      <c r="E41" s="199"/>
-      <c r="F41" s="199"/>
-      <c r="G41" s="193"/>
-      <c r="H41" s="203"/>
+    <row r="41" spans="1:8" s="180" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="190"/>
+      <c r="B41" s="198"/>
+      <c r="C41" s="186"/>
+      <c r="D41" s="199"/>
+      <c r="E41" s="197"/>
+      <c r="F41" s="197"/>
+      <c r="G41" s="191"/>
+      <c r="H41" s="201"/>
     </row>
     <row r="42" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="63" t="s">
@@ -3142,20 +2865,20 @@
         <v>#REF!</v>
       </c>
       <c r="C42" s="113"/>
-      <c r="D42" s="202">
+      <c r="D42" s="200">
         <f>SUM(D35:D40)</f>
         <v>0</v>
       </c>
-      <c r="E42" s="202" t="e">
+      <c r="E42" s="200" t="e">
         <f t="shared" ref="E42:H42" si="3">SUM(E35:E40)</f>
         <v>#REF!</v>
       </c>
-      <c r="F42" s="202" t="e">
+      <c r="F42" s="200" t="e">
         <f t="shared" si="3"/>
         <v>#REF!</v>
       </c>
       <c r="G42" s="113"/>
-      <c r="H42" s="202" t="e">
+      <c r="H42" s="200" t="e">
         <f t="shared" si="3"/>
         <v>#REF!</v>
       </c>
@@ -3171,63 +2894,63 @@
       <c r="H43" s="112"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" s="189" t="s">
+      <c r="A45" s="187" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A46" s="184" t="s">
+      <c r="A46" s="182" t="s">
         <v>163</v>
       </c>
-      <c r="H46" s="164">
+      <c r="H46" s="162">
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A47" s="184" t="s">
+      <c r="A47" s="182" t="s">
         <v>164</v>
       </c>
-      <c r="H47" s="208" t="e">
+      <c r="H47" s="206" t="e">
         <f>-H15</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A48" s="184"/>
-      <c r="H48" s="164" t="e">
+      <c r="A48" s="182"/>
+      <c r="H48" s="162" t="e">
         <f>SUM(H46:H47)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" s="184"/>
+      <c r="A49" s="182"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A50" s="184" t="s">
+      <c r="A50" s="182" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A51" s="184" t="s">
+      <c r="A51" s="182" t="s">
         <v>166</v>
       </c>
-      <c r="H51" s="164">
+      <c r="H51" s="162">
         <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="184" t="s">
+      <c r="A52" s="182" t="s">
         <v>167</v>
       </c>
-      <c r="H52" s="164">
+      <c r="H52" s="162">
         <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A53" s="184" t="s">
+      <c r="A53" s="182" t="s">
         <v>168</v>
       </c>
-      <c r="H53" s="209" t="e">
+      <c r="H53" s="207" t="e">
         <f>SUM(H48:H52)</f>
         <v>#REF!</v>
       </c>
@@ -3251,7 +2974,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="212" t="s">
+      <c r="A1" s="208" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3259,35 +2982,40 @@
       <c r="A2" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="158">
+      <c r="B2" s="157">
         <v>2328236</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="158"/>
+      <c r="B3" s="157"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="212" t="s">
+      <c r="A4" s="208" t="s">
         <v>173</v>
       </c>
-      <c r="B4" s="158"/>
+      <c r="B4" s="157"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="162">
+      <c r="B5" s="220">
         <v>99975</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="158"/>
+      <c r="A6" s="242" t="s">
+        <v>145</v>
+      </c>
+      <c r="B6" s="243">
+        <v>163480</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="158"/>
+      <c r="B7" s="157"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="212" t="s">
+      <c r="A8" s="208" t="s">
         <v>19</v>
       </c>
       <c r="C8" t="s">
@@ -3295,16 +3023,16 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B9" s="158"/>
+      <c r="B9" s="157"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="158"/>
+      <c r="B10" s="157"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="212" t="s">
+      <c r="A11" s="208" t="s">
         <v>174</v>
       </c>
-      <c r="B11" s="158"/>
+      <c r="B11" s="157"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -3321,17 +3049,17 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="159">
+      <c r="A13" s="158">
         <v>45597</v>
       </c>
-      <c r="B13" s="158">
+      <c r="B13" s="157">
         <v>4200</v>
       </c>
-      <c r="C13" s="158">
+      <c r="C13" s="157">
         <f>B13*12/20</f>
         <v>2520</v>
       </c>
-      <c r="D13" s="158">
+      <c r="D13" s="157">
         <f>C13*3/12</f>
         <v>630</v>
       </c>
@@ -3340,23 +3068,23 @@
       <c r="A14" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="160">
+      <c r="B14" s="159">
         <f>SUM(B13:B13)</f>
         <v>4200</v>
       </c>
-      <c r="C14" s="161">
+      <c r="C14" s="160">
         <f>SUM(C13:C13)</f>
         <v>2520</v>
       </c>
-      <c r="D14" s="161">
+      <c r="D14" s="160">
         <f>SUM(D13:D13)</f>
         <v>630</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="158"/>
-      <c r="C15" s="158"/>
-      <c r="D15" s="158"/>
+      <c r="B15" s="157"/>
+      <c r="C15" s="157"/>
+      <c r="D15" s="157"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3367,234 +3095,262 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25" style="156" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25" style="155" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.109375" style="88" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" style="157" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" style="154" bestFit="1" customWidth="1"/>
-    <col min="5" max="9" width="9.109375" style="154"/>
-    <col min="10" max="10" width="11.5546875" style="154" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="154"/>
+    <col min="3" max="3" width="10" style="156" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" style="153" bestFit="1" customWidth="1"/>
+    <col min="5" max="9" width="9.109375" style="153"/>
+    <col min="10" max="10" width="11.5546875" style="153" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.109375" style="153"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="239" t="s">
         <v>179</v>
       </c>
-      <c r="B1" s="243"/>
-      <c r="C1" s="243"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="239"/>
     </row>
     <row r="2" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="243" t="s">
+      <c r="A2" s="239" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="243"/>
-      <c r="C2" s="243"/>
+      <c r="B2" s="239"/>
+      <c r="C2" s="239"/>
     </row>
     <row r="3" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="243" t="s">
+      <c r="A3" s="239" t="s">
         <v>106</v>
       </c>
-      <c r="B3" s="243"/>
-      <c r="C3" s="243"/>
+      <c r="B3" s="239"/>
+      <c r="C3" s="239"/>
     </row>
     <row r="4" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A4" s="221" t="s">
+      <c r="A4" s="217" t="s">
         <v>178</v>
       </c>
-      <c r="B4" s="213" t="s">
+      <c r="B4" s="209" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="214" t="s">
+      <c r="C4" s="210" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A5" s="215" t="s">
+      <c r="A5" s="211" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="216"/>
-      <c r="C5" s="216"/>
+      <c r="B5" s="212"/>
+      <c r="C5" s="212"/>
     </row>
     <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A6" s="217" t="s">
+      <c r="A6" s="213" t="s">
         <v>118</v>
       </c>
-      <c r="B6" s="223">
+      <c r="B6" s="219">
         <v>12560</v>
       </c>
-      <c r="C6" s="216"/>
+      <c r="C6" s="212"/>
     </row>
     <row r="7" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A7" s="215" t="s">
+      <c r="A7" s="211" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="216"/>
-      <c r="C7" s="216"/>
-      <c r="J7" s="155"/>
+      <c r="B7" s="212"/>
+      <c r="C7" s="212"/>
+      <c r="J7" s="154"/>
     </row>
     <row r="8" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A8" s="217" t="s">
+      <c r="A8" s="213" t="s">
         <v>108</v>
       </c>
-      <c r="B8" s="216">
+      <c r="B8" s="212">
         <f>+PPE!D4</f>
         <v>153700</v>
       </c>
-      <c r="C8" s="216"/>
-      <c r="J8" s="155"/>
+      <c r="C8" s="212"/>
+      <c r="J8" s="154"/>
     </row>
     <row r="9" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A9" s="217" t="s">
+      <c r="A9" s="213" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="216"/>
-      <c r="C9" s="216">
+      <c r="B9" s="212"/>
+      <c r="C9" s="212">
         <f>+PPE!G5</f>
         <v>28887.178082191782</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A10" s="215" t="s">
+      <c r="A10" s="211" t="s">
         <v>175</v>
       </c>
-      <c r="B10" s="216"/>
-      <c r="C10" s="216"/>
+      <c r="B10" s="212"/>
+      <c r="C10" s="212"/>
     </row>
     <row r="11" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="217" t="s">
+      <c r="A11" s="213" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="216"/>
-      <c r="C11" s="216">
-        <f>+B22</f>
+      <c r="B11" s="212"/>
+      <c r="C11" s="212">
+        <f>+B24</f>
         <v>15000</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A12" s="217" t="s">
+      <c r="A12" s="213" t="s">
         <v>99</v>
       </c>
-      <c r="B12" s="216"/>
-      <c r="C12" s="216">
-        <f>+B23</f>
+      <c r="B12" s="212"/>
+      <c r="C12" s="212">
+        <f>+B26</f>
         <v>25000</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="212" t="s">
+      <c r="A13" s="208" t="s">
         <v>176</v>
       </c>
-      <c r="B13" s="218"/>
-      <c r="C13" s="219"/>
+      <c r="B13" s="214"/>
+      <c r="C13" s="215"/>
     </row>
     <row r="14" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A14" s="217" t="s">
+      <c r="A14" s="213" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="216"/>
-      <c r="C14" s="216">
+      <c r="B14" s="212"/>
+      <c r="C14" s="212">
         <f>1000*6</f>
         <v>6000</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A15" s="217" t="s">
+      <c r="A15" s="213" t="s">
         <v>157</v>
       </c>
-      <c r="B15" s="216"/>
-      <c r="C15" s="216">
+      <c r="B15" s="212"/>
+      <c r="C15" s="212">
         <v>1000000</v>
       </c>
     </row>
-    <row r="16" spans="1:10" s="204" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A16" s="215" t="s">
+    <row r="16" spans="1:10" s="202" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="211" t="s">
         <v>146</v>
       </c>
-      <c r="B16" s="216"/>
-      <c r="C16" s="219"/>
+      <c r="B16" s="212"/>
+      <c r="C16" s="215"/>
     </row>
     <row r="17" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="220" t="s">
+      <c r="A17" s="216" t="s">
         <v>158</v>
       </c>
-      <c r="B17" s="224">
+      <c r="B17" s="220">
         <v>112919.5</v>
       </c>
-      <c r="C17" s="216"/>
+      <c r="C17" s="212"/>
     </row>
-    <row r="18" spans="1:3" s="204" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="217" t="s">
+    <row r="18" spans="1:3" s="202" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="213" t="s">
         <v>105</v>
       </c>
-      <c r="B18" s="216"/>
-      <c r="C18" s="225">
+      <c r="B18" s="212"/>
+      <c r="C18" s="221">
         <f>+Working!B2</f>
         <v>2328236</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="212" t="s">
+      <c r="A19" s="208" t="s">
         <v>177</v>
       </c>
-      <c r="B19" s="216"/>
-      <c r="C19" s="216"/>
+      <c r="B19" s="212"/>
+      <c r="C19" s="212"/>
     </row>
-    <row r="20" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A20" s="217" t="s">
-        <v>155</v>
-      </c>
-      <c r="B20" s="216">
-        <v>1220000</v>
-      </c>
-      <c r="C20" s="216"/>
+    <row r="20" spans="1:3" s="202" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="241" t="s">
+        <v>152</v>
+      </c>
+      <c r="B20" s="212">
+        <v>12600</v>
+      </c>
+      <c r="C20" s="212"/>
     </row>
-    <row r="21" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A21" s="217" t="s">
-        <v>136</v>
-      </c>
-      <c r="B21" s="216">
-        <v>1000</v>
-      </c>
-      <c r="C21" s="216"/>
+    <row r="21" spans="1:3" s="202" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A21" s="241" t="s">
+        <v>153</v>
+      </c>
+      <c r="B21" s="212">
+        <v>3150</v>
+      </c>
+      <c r="C21" s="212"/>
     </row>
     <row r="22" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A22" s="217" t="s">
-        <v>119</v>
-      </c>
-      <c r="B22" s="216">
-        <v>15000</v>
-      </c>
-      <c r="C22" s="216"/>
+      <c r="A22" s="213" t="s">
+        <v>155</v>
+      </c>
+      <c r="B22" s="212">
+        <v>1220000</v>
+      </c>
+      <c r="C22" s="212"/>
     </row>
     <row r="23" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A23" s="217" t="s">
+      <c r="A23" s="213" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" s="212">
+        <v>1000</v>
+      </c>
+      <c r="C23" s="212"/>
+    </row>
+    <row r="24" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A24" s="213" t="s">
+        <v>119</v>
+      </c>
+      <c r="B24" s="212">
+        <v>15000</v>
+      </c>
+      <c r="C24" s="212"/>
+    </row>
+    <row r="25" spans="1:3" s="202" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A25" s="241" t="s">
+        <v>145</v>
+      </c>
+      <c r="B25" s="212">
+        <f>+Working!B6</f>
+        <v>163480</v>
+      </c>
+      <c r="C25" s="212"/>
+    </row>
+    <row r="26" spans="1:3" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A26" s="213" t="s">
         <v>99</v>
       </c>
-      <c r="B23" s="216">
+      <c r="B26" s="212">
         <v>25000</v>
       </c>
-      <c r="C23" s="216"/>
+      <c r="C26" s="212"/>
     </row>
-    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="221" t="s">
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="217" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="222">
-        <f>SUM(B5:B23)</f>
-        <v>1540179.5</v>
-      </c>
-      <c r="C24" s="222">
-        <f>SUM(C5:C23)</f>
+      <c r="B27" s="218">
+        <f>SUM(B5:B26)</f>
+        <v>1719409.5</v>
+      </c>
+      <c r="C27" s="218">
+        <f>SUM(C5:C26)</f>
         <v>3403123.1780821919</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="14.4" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="88">
-        <f>B24-C24</f>
-        <v>-1862943.6780821919</v>
+    <row r="28" spans="1:3" ht="14.4" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="88">
+        <f>B27-C27</f>
+        <v>-1683713.6780821919</v>
       </c>
     </row>
   </sheetData>
@@ -3641,7 +3397,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="153" t="s">
+      <c r="J1" s="152" t="s">
         <v>103</v>
       </c>
     </row>
@@ -3870,9 +3626,9 @@
       <c r="D20" s="58"/>
       <c r="H20" s="38"/>
       <c r="I20" s="17"/>
-      <c r="J20" s="135" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
+      <c r="J20" s="135">
+        <f>TB!B20</f>
+        <v>12600</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
@@ -3884,9 +3640,9 @@
       <c r="D21" s="58"/>
       <c r="H21" s="38"/>
       <c r="I21" s="17"/>
-      <c r="J21" s="135" t="e">
-        <f>TB!#REF!</f>
-        <v>#REF!</v>
+      <c r="J21" s="135">
+        <f>TB!B21</f>
+        <v>3150</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -3921,9 +3677,9 @@
       <c r="A24" s="57"/>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
-      <c r="J24" s="133" t="e">
+      <c r="J24" s="133">
         <f>SUM(J20:J23)</f>
-        <v>#REF!</v>
+        <v>55750</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -4104,7 +3860,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="153" t="s">
+      <c r="I1" s="152" t="s">
         <v>50</v>
       </c>
       <c r="J1" s="1"/>
@@ -4174,11 +3930,11 @@
       <c r="A7" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="E7" s="241">
+      <c r="E7" s="237">
         <v>0</v>
       </c>
       <c r="F7" s="84"/>
-      <c r="G7" s="241">
+      <c r="G7" s="237">
         <v>0</v>
       </c>
       <c r="H7" s="84"/>
@@ -4202,7 +3958,7 @@
         <v>6000</v>
       </c>
       <c r="F9" s="129"/>
-      <c r="G9" s="240">
+      <c r="G9" s="236">
         <v>0</v>
       </c>
       <c r="H9" s="129"/>
@@ -4222,18 +3978,18 @@
       <c r="A11" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="E11" s="239">
+      <c r="E11" s="235">
         <v>0</v>
       </c>
       <c r="F11" s="62"/>
-      <c r="G11" s="62" t="e">
+      <c r="G11" s="62">
         <f>+PL!D16</f>
-        <v>#REF!</v>
+        <v>2123756</v>
       </c>
       <c r="H11" s="62"/>
-      <c r="I11" s="62" t="e">
+      <c r="I11" s="62">
         <f>G11</f>
-        <v>#REF!</v>
+        <v>2123756</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -4247,19 +4003,19 @@
       <c r="A13" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="E13" s="171">
+      <c r="E13" s="169">
         <f>SUM(E7:E11)</f>
         <v>6000</v>
       </c>
-      <c r="F13" s="187"/>
-      <c r="G13" s="171" t="e">
+      <c r="F13" s="185"/>
+      <c r="G13" s="169">
         <f>SUM(G7:G11)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H13" s="187"/>
-      <c r="I13" s="171" t="e">
+        <v>2123756</v>
+      </c>
+      <c r="H13" s="185"/>
+      <c r="I13" s="169">
         <f>SUM(I7:I11)</f>
-        <v>#REF!</v>
+        <v>2129756</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -4326,344 +4082,344 @@
   <dimension ref="A1:I43"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.88671875" style="168" customWidth="1"/>
-    <col min="2" max="2" width="30.44140625" style="168" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" style="168" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" style="168" customWidth="1"/>
-    <col min="5" max="5" width="9" style="168" customWidth="1"/>
-    <col min="6" max="6" width="0.6640625" style="168" customWidth="1"/>
-    <col min="7" max="7" width="13.109375" style="168" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="168" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" style="168" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="168"/>
+    <col min="1" max="1" width="2.88671875" style="166" customWidth="1"/>
+    <col min="2" max="2" width="30.44140625" style="166" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" style="166" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" style="166" customWidth="1"/>
+    <col min="5" max="5" width="9" style="166" customWidth="1"/>
+    <col min="6" max="6" width="0.6640625" style="166" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" style="166" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="166" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" style="166" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="166"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="170" t="s">
+      <c r="A1" s="168" t="s">
         <v>142</v>
       </c>
-      <c r="E1" s="170"/>
-      <c r="F1" s="170"/>
-      <c r="G1" s="206" t="s">
+      <c r="E1" s="168"/>
+      <c r="F1" s="168"/>
+      <c r="G1" s="204" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="170"/>
+      <c r="H1" s="168"/>
     </row>
-    <row r="2" spans="1:8" s="165" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="170" t="s">
+    <row r="2" spans="1:8" s="163" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="168" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="170"/>
-      <c r="F2" s="170"/>
-      <c r="G2" s="180"/>
-      <c r="H2" s="170"/>
+      <c r="E2" s="168"/>
+      <c r="F2" s="168"/>
+      <c r="G2" s="178"/>
+      <c r="H2" s="168"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="165" t="str">
+      <c r="A3" s="163" t="str">
         <f>+PL!A3</f>
         <v>FOR THE YEAR PERIOD 31ST MARCH</v>
       </c>
-      <c r="B3" s="170"/>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="175">
+      <c r="B3" s="168"/>
+      <c r="C3" s="168"/>
+      <c r="D3" s="168"/>
+      <c r="E3" s="168"/>
+      <c r="F3" s="168"/>
+      <c r="G3" s="173">
         <v>2025</v>
       </c>
-      <c r="H3" s="170"/>
+      <c r="H3" s="168"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="G4" s="183" t="s">
+      <c r="G4" s="181" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F5" s="174"/>
+      <c r="F5" s="172"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="165" t="s">
+      <c r="A6" s="163" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="174"/>
-      <c r="G6" s="177"/>
+      <c r="F6" s="172"/>
+      <c r="G6" s="175"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="169" t="s">
+      <c r="A7" s="167" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="190"/>
-      <c r="G7" s="194" t="e">
+      <c r="F7" s="188"/>
+      <c r="G7" s="192">
         <f>+PL!D12</f>
-        <v>#REF!</v>
+        <v>2124756</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="168" t="s">
+      <c r="A8" s="166" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="176"/>
-      <c r="G8" s="195"/>
+      <c r="F8" s="174"/>
+      <c r="G8" s="193"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B9" s="172" t="s">
+      <c r="B9" s="170" t="s">
         <v>127</v>
       </c>
-      <c r="C9" s="172"/>
-      <c r="D9" s="172"/>
-      <c r="F9" s="176"/>
-      <c r="G9" s="195" t="e">
+      <c r="C9" s="170"/>
+      <c r="D9" s="170"/>
+      <c r="F9" s="174"/>
+      <c r="G9" s="193" t="e">
         <f>'P09'!#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="165" t="s">
+      <c r="A10" s="163" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="176"/>
-      <c r="G10" s="196" t="e">
+      <c r="F10" s="174"/>
+      <c r="G10" s="194" t="e">
         <f>SUM(G7:G9)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F11" s="176"/>
-      <c r="G11" s="195"/>
+      <c r="F11" s="174"/>
+      <c r="G11" s="193"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B12" s="172" t="s">
+      <c r="B12" s="170" t="s">
         <v>160</v>
       </c>
-      <c r="C12" s="172"/>
-      <c r="D12" s="172"/>
-      <c r="F12" s="176"/>
-      <c r="G12" s="195">
+      <c r="C12" s="170"/>
+      <c r="D12" s="170"/>
+      <c r="F12" s="174"/>
+      <c r="G12" s="193">
         <f>-BS!E12</f>
         <v>-112919.5</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="172" t="s">
+      <c r="B13" s="170" t="s">
         <v>170</v>
       </c>
-      <c r="C13" s="172"/>
-      <c r="D13" s="172"/>
-      <c r="F13" s="176"/>
-      <c r="G13" s="195" t="e">
+      <c r="C13" s="170"/>
+      <c r="D13" s="170"/>
+      <c r="F13" s="174"/>
+      <c r="G13" s="193">
         <f>BS!E26</f>
-        <v>#REF!</v>
+        <v>55750</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B14" s="172" t="s">
+      <c r="B14" s="170" t="s">
         <v>101</v>
       </c>
-      <c r="C14" s="172"/>
-      <c r="D14" s="172"/>
-      <c r="F14" s="176"/>
-      <c r="G14" s="195">
+      <c r="C14" s="170"/>
+      <c r="D14" s="170"/>
+      <c r="F14" s="174"/>
+      <c r="G14" s="193">
         <f>BS!E27</f>
         <v>1000000</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="165" t="s">
+      <c r="A15" s="163" t="s">
         <v>56</v>
       </c>
-      <c r="F15" s="176"/>
-      <c r="G15" s="196" t="e">
+      <c r="F15" s="174"/>
+      <c r="G15" s="194" t="e">
         <f>SUM(G10:G14)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="F16" s="176"/>
-      <c r="G16" s="195"/>
+      <c r="F16" s="174"/>
+      <c r="G16" s="193"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B17" s="168" t="s">
+      <c r="B17" s="166" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="176"/>
-      <c r="G17" s="195">
-        <f>TB!B21</f>
+      <c r="F17" s="174"/>
+      <c r="G17" s="193">
+        <f>TB!B23</f>
         <v>1000</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F18" s="176"/>
-      <c r="G18" s="197">
+      <c r="F18" s="174"/>
+      <c r="G18" s="195">
         <f>SUM(G17:G17)</f>
         <v>1000</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="165" t="s">
+      <c r="A19" s="163" t="s">
         <v>57</v>
       </c>
-      <c r="E19" s="165"/>
-      <c r="F19" s="176"/>
-      <c r="G19" s="197" t="e">
+      <c r="E19" s="163"/>
+      <c r="F19" s="174"/>
+      <c r="G19" s="195" t="e">
         <f>SUM(G18+G15)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F20" s="176"/>
-      <c r="G20" s="195"/>
+      <c r="F20" s="174"/>
+      <c r="G20" s="193"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="165" t="s">
+      <c r="A21" s="163" t="s">
         <v>58</v>
       </c>
-      <c r="F21" s="176"/>
-      <c r="G21" s="195"/>
+      <c r="F21" s="174"/>
+      <c r="G21" s="193"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B22" s="169" t="s">
+      <c r="B22" s="167" t="s">
         <v>137</v>
       </c>
-      <c r="F22" s="176"/>
-      <c r="G22" s="195" t="e">
-        <f>-'P10'!G12</f>
-        <v>#REF!</v>
+      <c r="F22" s="174"/>
+      <c r="G22" s="193">
+        <f>-'P10'!G7</f>
+        <v>-153700</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="165" t="s">
+      <c r="A23" s="163" t="s">
         <v>59</v>
       </c>
-      <c r="E23" s="165"/>
-      <c r="F23" s="176"/>
-      <c r="G23" s="197" t="e">
+      <c r="E23" s="163"/>
+      <c r="F23" s="174"/>
+      <c r="G23" s="195">
         <f>SUM(G22)</f>
-        <v>#REF!</v>
+        <v>-153700</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="F24" s="176"/>
-      <c r="G24" s="195"/>
+      <c r="F24" s="174"/>
+      <c r="G24" s="193"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="165" t="s">
+      <c r="A25" s="163" t="s">
         <v>60</v>
       </c>
-      <c r="F25" s="176"/>
-      <c r="G25" s="195"/>
+      <c r="F25" s="174"/>
+      <c r="G25" s="193"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B26" s="168" t="s">
+      <c r="B26" s="166" t="s">
         <v>70</v>
       </c>
-      <c r="F26" s="176"/>
-      <c r="G26" s="195">
+      <c r="F26" s="174"/>
+      <c r="G26" s="193">
         <f>+BS!E19</f>
         <v>6000</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="165" t="s">
+      <c r="A27" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F27" s="176"/>
-      <c r="G27" s="197">
+      <c r="F27" s="174"/>
+      <c r="G27" s="195">
         <f>SUM(G26)</f>
         <v>6000</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="165" t="s">
+      <c r="A28" s="163" t="s">
         <v>65</v>
       </c>
-      <c r="F28" s="176"/>
-      <c r="G28" s="195" t="e">
+      <c r="F28" s="174"/>
+      <c r="G28" s="193" t="e">
         <f>+G19+G23+G27</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B29" s="168" t="s">
+      <c r="B29" s="166" t="s">
         <v>62</v>
       </c>
-      <c r="F29" s="176"/>
-      <c r="G29" s="239">
+      <c r="F29" s="174"/>
+      <c r="G29" s="235">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="168" t="s">
+      <c r="B30" s="166" t="s">
         <v>63</v>
       </c>
-      <c r="F30" s="176"/>
-      <c r="G30" s="198" t="e">
+      <c r="F30" s="174"/>
+      <c r="G30" s="196" t="e">
         <f>SUM(G28:G29)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="F31" s="176"/>
-      <c r="G31" s="195"/>
+      <c r="F31" s="174"/>
+      <c r="G31" s="193"/>
     </row>
-    <row r="32" spans="1:7" s="169" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="166" t="s">
+    <row r="32" spans="1:7" s="167" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="164" t="s">
         <v>139</v>
       </c>
-      <c r="C32" s="163"/>
-      <c r="F32" s="186"/>
+      <c r="C32" s="161"/>
+      <c r="F32" s="184"/>
     </row>
-    <row r="33" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="179" t="s">
+    <row r="33" spans="1:9" s="167" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="177" t="s">
         <v>138</v>
       </c>
-      <c r="G33" s="242">
+      <c r="G33" s="238">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" s="169" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G34" s="207">
+    <row r="34" spans="1:9" s="167" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G34" s="205">
         <f>SUM(F33:F33)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" s="169" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="36" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="166" t="s">
+    <row r="35" spans="1:9" s="167" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="1:9" s="167" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="164" t="s">
         <v>140</v>
       </c>
-      <c r="G36" s="186"/>
+      <c r="G36" s="184"/>
     </row>
-    <row r="37" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="179" t="s">
+    <row r="37" spans="1:9" s="167" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="177" t="s">
         <v>138</v>
       </c>
-      <c r="D37" s="178"/>
-      <c r="E37" s="178"/>
-      <c r="G37" s="185">
+      <c r="D37" s="176"/>
+      <c r="E37" s="176"/>
+      <c r="G37" s="183">
         <f>'P11'!J7</f>
         <v>12560</v>
       </c>
     </row>
-    <row r="38" spans="1:9" s="169" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="166"/>
-      <c r="G38" s="207">
+    <row r="38" spans="1:9" s="167" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="164"/>
+      <c r="G38" s="205">
         <f>SUM(G37:G37)</f>
         <v>12560</v>
       </c>
-      <c r="H38" s="181" t="e">
+      <c r="H38" s="179" t="e">
         <f>G30-G38</f>
         <v>#REF!</v>
       </c>
-      <c r="I38" s="181"/>
+      <c r="I38" s="179"/>
     </row>
     <row r="39" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A41" s="168" t="s">
+      <c r="A41" s="166" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43" s="169" t="s">
+      <c r="A43" s="167" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4694,7 +4450,7 @@
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="153" t="s">
+      <c r="D1" s="152" t="s">
         <v>28</v>
       </c>
     </row>
@@ -4776,9 +4532,9 @@
         <v>6</v>
       </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="123" t="e">
+      <c r="D10" s="123">
         <f>-'P09'!D17</f>
-        <v>#REF!</v>
+        <v>-163480</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -4789,9 +4545,9 @@
         <v>31</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="D12" s="119" t="e">
+      <c r="D12" s="119">
         <f>SUM(D6:D10)</f>
-        <v>#REF!</v>
+        <v>2124756</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -4816,9 +4572,9 @@
       <c r="A16" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="D16" s="124" t="e">
+      <c r="D16" s="124">
         <f>SUM(D12:D14)</f>
-        <v>#REF!</v>
+        <v>2123756</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -4875,7 +4631,7 @@
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="153" t="s">
+      <c r="E1" s="152" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4919,7 +4675,7 @@
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="145"/>
+      <c r="B6" s="144"/>
     </row>
     <row r="7" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -4927,7 +4683,7 @@
       </c>
       <c r="B7" s="1"/>
       <c r="E7" s="73"/>
-      <c r="F7" s="144"/>
+      <c r="F7" s="143"/>
     </row>
     <row r="8" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A8" s="18" t="s">
@@ -4937,22 +4693,22 @@
         <v>8</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="121" t="e">
-        <f>+'P10'!J31</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F8" s="144"/>
+      <c r="E8" s="121">
+        <f>+'P10'!J16</f>
+        <v>124812.82191780822</v>
+      </c>
+      <c r="F8" s="143"/>
     </row>
     <row r="9" spans="1:1003" x14ac:dyDescent="0.35">
-      <c r="E9" s="126" t="e">
+      <c r="E9" s="126">
         <f>SUM(E8)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F9" s="144"/>
+        <v>124812.82191780822</v>
+      </c>
+      <c r="F9" s="143"/>
     </row>
     <row r="10" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="E10" s="121"/>
-      <c r="F10" s="144"/>
+      <c r="F10" s="143"/>
     </row>
     <row r="11" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
@@ -5960,13 +5716,13 @@
       <c r="ALO11" s="13"/>
     </row>
     <row r="12" spans="1:1003" x14ac:dyDescent="0.35">
-      <c r="A12" s="143" t="s">
+      <c r="A12" s="178" t="s">
         <v>158</v>
       </c>
-      <c r="B12" s="143"/>
-      <c r="C12" s="210"/>
-      <c r="D12" s="210"/>
-      <c r="E12" s="211">
+      <c r="B12" s="178"/>
+      <c r="C12" s="240"/>
+      <c r="D12" s="240"/>
+      <c r="E12" s="73">
         <f>TB!B17</f>
         <v>112919.5</v>
       </c>
@@ -8994,9 +8750,9 @@
         <v>4</v>
       </c>
       <c r="B15" s="1"/>
-      <c r="E15" s="127" t="e">
+      <c r="E15" s="127">
         <f>SUM(E14+E9)</f>
-        <v>#REF!</v>
+        <v>250292.32191780821</v>
       </c>
       <c r="F15" s="101"/>
       <c r="G15" s="13"/>
@@ -9999,7 +9755,7 @@
     </row>
     <row r="16" spans="1:1003" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="E16" s="121"/>
-      <c r="F16" s="144"/>
+      <c r="F16" s="143"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13"/>
       <c r="L16" s="13"/>
@@ -10999,10 +10755,10 @@
       <c r="A17" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="145"/>
+      <c r="B17" s="144"/>
       <c r="E17" s="73"/>
-      <c r="F17" s="144"/>
-      <c r="I17" s="146"/>
+      <c r="F17" s="143"/>
+      <c r="I17" s="145"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13"/>
       <c r="L17" s="13"/>
@@ -12004,7 +11760,7 @@
       </c>
       <c r="B18" s="1"/>
       <c r="E18" s="73"/>
-      <c r="F18" s="144"/>
+      <c r="F18" s="143"/>
       <c r="J18" s="13"/>
       <c r="K18" s="13"/>
       <c r="L18" s="13"/>
@@ -13012,7 +12768,7 @@
         <f>+'P11'!J17</f>
         <v>6000</v>
       </c>
-      <c r="F19" s="144"/>
+      <c r="F19" s="143"/>
       <c r="J19" s="13"/>
       <c r="K19" s="13"/>
       <c r="L19" s="13"/>
@@ -14012,11 +13768,11 @@
       <c r="A20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="73" t="e">
+      <c r="E20" s="73">
         <f>+CE!G13</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F20" s="144"/>
+        <v>2123756</v>
+      </c>
+      <c r="F20" s="143"/>
       <c r="J20" s="13"/>
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
@@ -15013,11 +14769,11 @@
       <c r="ALO20" s="13"/>
     </row>
     <row r="21" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="E21" s="126" t="e">
+      <c r="E21" s="126">
         <f>SUM(E19:E20)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F21" s="144"/>
+        <v>2129756</v>
+      </c>
+      <c r="F21" s="143"/>
       <c r="J21" s="62"/>
       <c r="K21" s="13"/>
       <c r="L21" s="13"/>
@@ -16015,7 +15771,7 @@
     </row>
     <row r="22" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="E22" s="121"/>
-      <c r="F22" s="144"/>
+      <c r="F22" s="143"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
       <c r="L22" s="13"/>
@@ -17018,7 +16774,7 @@
       <c r="E23" s="121">
         <v>0</v>
       </c>
-      <c r="F23" s="144"/>
+      <c r="F23" s="143"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
@@ -18016,7 +17772,7 @@
     </row>
     <row r="24" spans="1:1012" x14ac:dyDescent="0.35">
       <c r="E24" s="73"/>
-      <c r="F24" s="144"/>
+      <c r="F24" s="143"/>
       <c r="J24" s="13"/>
       <c r="K24" s="13"/>
       <c r="L24" s="13"/>
@@ -19018,7 +18774,7 @@
       </c>
       <c r="B25" s="1"/>
       <c r="E25" s="73"/>
-      <c r="F25" s="144"/>
+      <c r="F25" s="143"/>
       <c r="J25" s="13"/>
       <c r="K25" s="13"/>
       <c r="L25" s="13"/>
@@ -20015,18 +19771,18 @@
       <c r="ALO25" s="13"/>
     </row>
     <row r="26" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A26" s="147" t="s">
+      <c r="A26" s="146" t="s">
         <v>104</v>
       </c>
       <c r="C26" s="3">
         <v>11</v>
       </c>
       <c r="D26" s="3"/>
-      <c r="E26" s="73" t="e">
+      <c r="E26" s="73">
         <f>+'P11'!J24</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F26" s="144"/>
+        <v>55750</v>
+      </c>
+      <c r="F26" s="143"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
       <c r="L26" s="13"/>
@@ -21023,15 +20779,15 @@
       <c r="ALO26" s="13"/>
     </row>
     <row r="27" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A27" s="147" t="s">
+      <c r="A27" s="146" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="148"/>
+      <c r="B27" s="147"/>
       <c r="E27" s="73">
         <f>TB!C15</f>
         <v>1000000</v>
       </c>
-      <c r="F27" s="144"/>
+      <c r="F27" s="143"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
@@ -22028,14 +21784,14 @@
       <c r="ALO27" s="13"/>
     </row>
     <row r="28" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A28" s="149" t="s">
+      <c r="A28" s="148" t="s">
         <v>41</v>
       </c>
-      <c r="E28" s="126" t="e">
+      <c r="E28" s="126">
         <f>SUM(E26:E27)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F28" s="144"/>
+        <v>1055750</v>
+      </c>
+      <c r="F28" s="143"/>
       <c r="J28" s="13"/>
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
@@ -23032,14 +22788,14 @@
       <c r="ALO28" s="13"/>
     </row>
     <row r="29" spans="1:1012" x14ac:dyDescent="0.35">
-      <c r="A29" s="149" t="s">
+      <c r="A29" s="148" t="s">
         <v>42</v>
       </c>
-      <c r="E29" s="128" t="e">
+      <c r="E29" s="128">
         <f>E28+E23</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F29" s="144"/>
+        <v>1055750</v>
+      </c>
+      <c r="F29" s="143"/>
       <c r="J29" s="13"/>
       <c r="K29" s="13"/>
       <c r="L29" s="13"/>
@@ -24040,14 +23796,14 @@
         <v>9</v>
       </c>
       <c r="B30" s="1"/>
-      <c r="E30" s="127" t="e">
+      <c r="E30" s="127">
         <f>+E21+E29</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F30" s="144"/>
-      <c r="G30" s="77" t="e">
+        <v>3185506</v>
+      </c>
+      <c r="F30" s="143"/>
+      <c r="G30" s="77">
         <f>E15-E30</f>
-        <v>#REF!</v>
+        <v>-2935213.6780821919</v>
       </c>
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
@@ -26048,9 +25804,9 @@
       </c>
       <c r="E32" s="20"/>
       <c r="F32" s="21"/>
-      <c r="G32" s="22" t="e">
+      <c r="G32" s="22">
         <f>G15-G30</f>
-        <v>#REF!</v>
+        <v>2935213.6780821919</v>
       </c>
       <c r="H32" s="23"/>
       <c r="J32" s="2"/>
@@ -30081,16 +29837,16 @@
       <c r="ALX35" s="2"/>
     </row>
     <row r="36" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="150" t="s">
+      <c r="A36" s="149" t="s">
         <v>43</v>
       </c>
-      <c r="B36" s="150"/>
-      <c r="C36" s="150"/>
-      <c r="D36" s="150"/>
+      <c r="B36" s="149"/>
+      <c r="C36" s="149"/>
+      <c r="D36" s="149"/>
       <c r="E36" s="24"/>
-      <c r="F36" s="150"/>
-      <c r="G36" s="150"/>
-      <c r="H36" s="150"/>
+      <c r="F36" s="149"/>
+      <c r="G36" s="149"/>
+      <c r="H36" s="149"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
@@ -31096,14 +30852,14 @@
       <c r="ALX36" s="2"/>
     </row>
     <row r="37" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="150"/>
-      <c r="B37" s="150"/>
-      <c r="C37" s="150"/>
-      <c r="D37" s="150"/>
+      <c r="A37" s="149"/>
+      <c r="B37" s="149"/>
+      <c r="C37" s="149"/>
+      <c r="D37" s="149"/>
       <c r="E37" s="24"/>
-      <c r="F37" s="150"/>
-      <c r="G37" s="150"/>
-      <c r="H37" s="150"/>
+      <c r="F37" s="149"/>
+      <c r="G37" s="149"/>
+      <c r="H37" s="149"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
@@ -32109,14 +31865,14 @@
       <c r="ALX37" s="2"/>
     </row>
     <row r="38" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="151"/>
-      <c r="B38" s="151"/>
-      <c r="C38" s="151"/>
-      <c r="D38" s="151"/>
+      <c r="A38" s="150"/>
+      <c r="B38" s="150"/>
+      <c r="C38" s="150"/>
+      <c r="D38" s="150"/>
       <c r="E38" s="25"/>
-      <c r="F38" s="151"/>
-      <c r="G38" s="151"/>
-      <c r="H38" s="151"/>
+      <c r="F38" s="150"/>
+      <c r="G38" s="150"/>
+      <c r="H38" s="150"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
@@ -36146,16 +35902,16 @@
       <c r="ALX41" s="2"/>
     </row>
     <row r="42" spans="1:1012" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="150" t="s">
+      <c r="A42" s="149" t="s">
         <v>46</v>
       </c>
-      <c r="B42" s="152"/>
-      <c r="C42" s="152"/>
-      <c r="D42" s="152"/>
+      <c r="B42" s="151"/>
+      <c r="C42" s="151"/>
+      <c r="D42" s="151"/>
       <c r="E42" s="26"/>
-      <c r="F42" s="152"/>
-      <c r="G42" s="152"/>
-      <c r="H42" s="152"/>
+      <c r="F42" s="151"/>
+      <c r="G42" s="151"/>
+      <c r="H42" s="151"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
@@ -37161,16 +36917,16 @@
       <c r="ALX42" s="2"/>
     </row>
     <row r="43" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="150" t="s">
+      <c r="A43" s="149" t="s">
         <v>47</v>
       </c>
-      <c r="B43" s="152"/>
-      <c r="C43" s="152"/>
-      <c r="D43" s="152"/>
+      <c r="B43" s="151"/>
+      <c r="C43" s="151"/>
+      <c r="D43" s="151"/>
       <c r="E43" s="26"/>
-      <c r="F43" s="152"/>
-      <c r="G43" s="152"/>
-      <c r="H43" s="152"/>
+      <c r="F43" s="151"/>
+      <c r="G43" s="151"/>
+      <c r="H43" s="151"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
@@ -38176,14 +37932,14 @@
       <c r="ALX43" s="2"/>
     </row>
     <row r="44" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="150"/>
-      <c r="B44" s="152"/>
-      <c r="C44" s="152"/>
-      <c r="D44" s="152"/>
+      <c r="A44" s="149"/>
+      <c r="B44" s="151"/>
+      <c r="C44" s="151"/>
+      <c r="D44" s="151"/>
       <c r="E44" s="26"/>
-      <c r="F44" s="152"/>
-      <c r="G44" s="152"/>
-      <c r="H44" s="152"/>
+      <c r="F44" s="151"/>
+      <c r="G44" s="151"/>
+      <c r="H44" s="151"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
@@ -39189,14 +38945,14 @@
       <c r="ALX44" s="2"/>
     </row>
     <row r="45" spans="1:1012" s="18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="150"/>
-      <c r="B45" s="152"/>
-      <c r="C45" s="152"/>
-      <c r="D45" s="152"/>
+      <c r="A45" s="149"/>
+      <c r="B45" s="151"/>
+      <c r="C45" s="151"/>
+      <c r="D45" s="151"/>
       <c r="E45" s="26"/>
-      <c r="F45" s="152"/>
-      <c r="G45" s="152"/>
-      <c r="H45" s="152"/>
+      <c r="F45" s="151"/>
+      <c r="G45" s="151"/>
+      <c r="H45" s="151"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
@@ -44281,7 +44037,7 @@
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
-      <c r="D1" s="153" t="s">
+      <c r="D1" s="152" t="s">
         <v>66</v>
       </c>
       <c r="E1" s="34"/>
@@ -44395,7 +44151,7 @@
       </c>
       <c r="C11" s="76"/>
       <c r="D11" s="120">
-        <f>+TB!B22</f>
+        <f>+TB!B24</f>
         <v>15000</v>
       </c>
       <c r="E11" s="1"/>
@@ -44409,7 +44165,7 @@
       </c>
       <c r="C12" s="76"/>
       <c r="D12" s="120">
-        <f>+TB!B23</f>
+        <f>+TB!B26</f>
         <v>25000</v>
       </c>
       <c r="E12" s="1"/>
@@ -44447,17 +44203,17 @@
         <v>145</v>
       </c>
       <c r="C16" s="3"/>
-      <c r="D16" s="121" t="e">
-        <f>+TB!#REF!</f>
-        <v>#REF!</v>
+      <c r="D16" s="121">
+        <f>+TB!B25</f>
+        <v>163480</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B17" s="1"/>
       <c r="C17" s="3"/>
-      <c r="D17" s="116" t="e">
+      <c r="D17" s="116">
         <f>SUM(D16)</f>
-        <v>#REF!</v>
+        <v>163480</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -44479,7 +44235,7 @@
         <v>102</v>
       </c>
       <c r="D20" s="115">
-        <f>TB!B21</f>
+        <f>TB!B23</f>
         <v>1000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement balance sheet generation and integrate into financial reports
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E1B289-3DA5-4DF2-BB49-8FD4B9871809}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A76FDB0-5174-4566-BCAF-4B26F66AAAE1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1420,9 +1420,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="43" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1431,6 +1428,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="23">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3004,10 +3004,10 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="242" t="s">
+      <c r="A6" s="241" t="s">
         <v>145</v>
       </c>
-      <c r="B6" s="243">
+      <c r="B6" s="242">
         <v>163480</v>
       </c>
     </row>
@@ -3108,25 +3108,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="239" t="s">
+      <c r="A1" s="243" t="s">
         <v>179</v>
       </c>
-      <c r="B1" s="239"/>
-      <c r="C1" s="239"/>
+      <c r="B1" s="243"/>
+      <c r="C1" s="243"/>
     </row>
     <row r="2" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="239" t="s">
+      <c r="A2" s="243" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="239"/>
-      <c r="C2" s="239"/>
+      <c r="B2" s="243"/>
+      <c r="C2" s="243"/>
     </row>
     <row r="3" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="239" t="s">
+      <c r="A3" s="243" t="s">
         <v>106</v>
       </c>
-      <c r="B3" s="239"/>
-      <c r="C3" s="239"/>
+      <c r="B3" s="243"/>
+      <c r="C3" s="243"/>
     </row>
     <row r="4" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A4" s="217" t="s">
@@ -3271,7 +3271,7 @@
       <c r="C19" s="212"/>
     </row>
     <row r="20" spans="1:3" s="202" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A20" s="241" t="s">
+      <c r="A20" s="240" t="s">
         <v>152</v>
       </c>
       <c r="B20" s="212">
@@ -3280,7 +3280,7 @@
       <c r="C20" s="212"/>
     </row>
     <row r="21" spans="1:3" s="202" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A21" s="241" t="s">
+      <c r="A21" s="240" t="s">
         <v>153</v>
       </c>
       <c r="B21" s="212">
@@ -3316,7 +3316,7 @@
       <c r="C24" s="212"/>
     </row>
     <row r="25" spans="1:3" s="202" customFormat="1" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A25" s="241" t="s">
+      <c r="A25" s="240" t="s">
         <v>145</v>
       </c>
       <c r="B25" s="212">
@@ -5720,8 +5720,8 @@
         <v>158</v>
       </c>
       <c r="B12" s="178"/>
-      <c r="C12" s="240"/>
-      <c r="D12" s="240"/>
+      <c r="C12" s="239"/>
+      <c r="D12" s="239"/>
       <c r="E12" s="73">
         <f>TB!B17</f>
         <v>112919.5</v>
@@ -23801,10 +23801,7 @@
         <v>3185506</v>
       </c>
       <c r="F30" s="143"/>
-      <c r="G30" s="77">
-        <f>E15-E30</f>
-        <v>-2935213.6780821919</v>
-      </c>
+      <c r="G30" s="77"/>
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
       <c r="L30" s="13"/>
@@ -25804,10 +25801,7 @@
       </c>
       <c r="E32" s="20"/>
       <c r="F32" s="21"/>
-      <c r="G32" s="22">
-        <f>G15-G30</f>
-        <v>2935213.6780821919</v>
-      </c>
+      <c r="G32" s="22"/>
       <c r="H32" s="23"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>

</xml_diff>

<commit_message>
feat: implement P10 worksheet generation and integrate into financial reports
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A76FDB0-5174-4566-BCAF-4B26F66AAAE1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D8D7815-81A5-4E38-B235-8F25A57F6048}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" firstSheet="3" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPE" sheetId="24" r:id="rId1"/>
@@ -2112,7 +2112,7 @@
       <c r="C6" s="44"/>
       <c r="D6" s="44"/>
       <c r="E6" s="131">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F6" s="131"/>
       <c r="G6" s="131">
@@ -2123,7 +2123,7 @@
       <c r="I6" s="119"/>
       <c r="J6" s="118">
         <f>SUM(E6:G6)</f>
-        <v>153700</v>
+        <v>154700</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2133,7 +2133,7 @@
       <c r="D7" s="44"/>
       <c r="E7" s="132">
         <f>SUM(E6:E6)</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F7" s="131"/>
       <c r="G7" s="132">
@@ -2144,7 +2144,7 @@
       <c r="I7" s="119"/>
       <c r="J7" s="132">
         <f>SUM(J6:J6)</f>
-        <v>153700</v>
+        <v>154700</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -2203,7 +2203,7 @@
       <c r="C11" s="44"/>
       <c r="D11" s="44"/>
       <c r="E11" s="131">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="F11" s="131"/>
       <c r="G11" s="118">
@@ -2214,7 +2214,7 @@
       <c r="I11" s="119"/>
       <c r="J11" s="137">
         <f>SUM(E11:G11)</f>
-        <v>28887.178082191782</v>
+        <v>29387.178082191782</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2224,7 +2224,7 @@
       <c r="D12" s="44"/>
       <c r="E12" s="132">
         <f>SUM(E11:E11)</f>
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="F12" s="131"/>
       <c r="G12" s="171">
@@ -2235,7 +2235,7 @@
       <c r="I12" s="119"/>
       <c r="J12" s="132">
         <f>SUM(J11:J11)</f>
-        <v>28887.178082191782</v>
+        <v>29387.178082191782</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -2267,14 +2267,14 @@
       </c>
       <c r="J15" s="74">
         <f>J6-J11</f>
-        <v>124812.82191780822</v>
+        <v>125312.82191780822</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2"/>
       <c r="J16" s="138">
         <f>SUM(J15:J15)</f>
-        <v>124812.82191780822</v>
+        <v>125312.82191780822</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -2349,7 +2349,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr codeName="Sheet11"/>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.109375" style="13" customWidth="1"/>
@@ -2477,9 +2477,9 @@
       <c r="F14" s="65" t="s">
         <v>134</v>
       </c>
-      <c r="H14" s="98" t="e">
-        <f>-E42</f>
-        <v>#REF!</v>
+      <c r="H14" s="98">
+        <f>-E37</f>
+        <v>-30740</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -2487,9 +2487,9 @@
         <v>87</v>
       </c>
       <c r="E15" s="21"/>
-      <c r="H15" s="100" t="e">
+      <c r="H15" s="100">
         <f>SUM(H12:H14)</f>
-        <v>#REF!</v>
+        <v>2122903.1780821919</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -2685,7 +2685,8 @@
         <v>5</v>
       </c>
       <c r="D35" s="140">
-        <v>0</v>
+        <f>'P10'!E6</f>
+        <v>1000</v>
       </c>
       <c r="E35" s="139">
         <f>B35/C35</f>
@@ -2693,214 +2694,101 @@
       </c>
       <c r="F35" s="139">
         <f>D35+E35</f>
-        <v>30740</v>
+        <v>31740</v>
       </c>
       <c r="G35" s="111"/>
       <c r="H35" s="142">
         <f>B35-F35</f>
-        <v>122960</v>
+        <v>121960</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" s="190" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
+    <row r="36" spans="1:8" s="180" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="190"/>
+      <c r="B36" s="198"/>
+      <c r="C36" s="186"/>
+      <c r="D36" s="199"/>
+      <c r="E36" s="197"/>
+      <c r="F36" s="197"/>
+      <c r="G36" s="191"/>
+      <c r="H36" s="201"/>
+    </row>
+    <row r="37" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="63" t="s">
+        <v>27</v>
       </c>
-      <c r="B36" s="165" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
+      <c r="B37" s="141">
+        <f>SUM(B35:B35)</f>
+        <v>153700</v>
       </c>
-      <c r="C36" s="65">
-        <v>5</v>
+      <c r="C37" s="113"/>
+      <c r="D37" s="200">
+        <f>SUM(D35:D35)</f>
+        <v>1000</v>
       </c>
-      <c r="D36" s="199">
+      <c r="E37" s="200">
+        <f>SUM(E35:E35)</f>
+        <v>30740</v>
+      </c>
+      <c r="F37" s="200">
+        <f>SUM(F35:F35)</f>
+        <v>31740</v>
+      </c>
+      <c r="G37" s="113"/>
+      <c r="H37" s="200">
+        <f>SUM(H35:H35)</f>
+        <v>121960</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="18"/>
+      <c r="B38" s="112"/>
+      <c r="C38" s="112"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="112"/>
+      <c r="G38" s="112"/>
+      <c r="H38" s="112"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A40" s="187" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A41" s="182" t="s">
+        <v>163</v>
+      </c>
+      <c r="H41" s="162">
         <v>0</v>
       </c>
-      <c r="E36" s="197" t="e">
-        <f t="shared" ref="E36:E40" si="0">B36/C36</f>
-        <v>#REF!</v>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A42" s="182" t="s">
+        <v>164</v>
       </c>
-      <c r="F36" s="197" t="e">
-        <f t="shared" ref="F36:F40" si="1">D36+E36</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G36" s="111"/>
-      <c r="H36" s="201" t="e">
-        <f t="shared" ref="H36:H40" si="2">B36-F36</f>
-        <v>#REF!</v>
+      <c r="H42" s="206">
+        <f>-H15</f>
+        <v>-2122903.1780821919</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" s="190" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B37" s="165" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C37" s="65">
-        <v>5</v>
-      </c>
-      <c r="D37" s="199">
-        <v>0</v>
-      </c>
-      <c r="E37" s="197" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="F37" s="197" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G37" s="111"/>
-      <c r="H37" s="201" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A43" s="182"/>
+      <c r="H43" s="162">
+        <f>SUM(H41:H42)</f>
+        <v>-2122903.1780821919</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="180" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="190" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B38" s="165" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C38" s="186">
-        <v>5</v>
-      </c>
-      <c r="D38" s="199">
-        <v>0</v>
-      </c>
-      <c r="E38" s="197" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="F38" s="197" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G38" s="191"/>
-      <c r="H38" s="201" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" s="180" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="190" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B39" s="165" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C39" s="186">
-        <v>5</v>
-      </c>
-      <c r="D39" s="199">
-        <v>0</v>
-      </c>
-      <c r="E39" s="197" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="F39" s="197" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G39" s="191"/>
-      <c r="H39" s="201" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" s="180" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="190" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B40" s="165" t="e">
-        <f>+'P10'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C40" s="186">
-        <v>5</v>
-      </c>
-      <c r="D40" s="199">
-        <v>0</v>
-      </c>
-      <c r="E40" s="197" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="F40" s="197" t="e">
-        <f t="shared" si="1"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G40" s="191"/>
-      <c r="H40" s="201" t="e">
-        <f t="shared" si="2"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" s="180" customFormat="1" ht="4.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="190"/>
-      <c r="B41" s="198"/>
-      <c r="C41" s="186"/>
-      <c r="D41" s="199"/>
-      <c r="E41" s="197"/>
-      <c r="F41" s="197"/>
-      <c r="G41" s="191"/>
-      <c r="H41" s="201"/>
-    </row>
-    <row r="42" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="B42" s="141" t="e">
-        <f>SUM(B35:B40)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C42" s="113"/>
-      <c r="D42" s="200">
-        <f>SUM(D35:D40)</f>
-        <v>0</v>
-      </c>
-      <c r="E42" s="200" t="e">
-        <f t="shared" ref="E42:H42" si="3">SUM(E35:E40)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F42" s="200" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-      <c r="G42" s="113"/>
-      <c r="H42" s="200" t="e">
-        <f t="shared" si="3"/>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="18"/>
-      <c r="B43" s="112"/>
-      <c r="C43" s="112"/>
-      <c r="D43" s="112"/>
-      <c r="E43" s="112"/>
-      <c r="F43" s="112"/>
-      <c r="G43" s="112"/>
-      <c r="H43" s="112"/>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A44" s="182"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" s="187" t="s">
-        <v>162</v>
+      <c r="A45" s="182" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="182" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="H46" s="162">
         <v>0</v>
@@ -2908,54 +2796,22 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="182" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
-      <c r="H47" s="206" t="e">
-        <f>-H15</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A48" s="182"/>
-      <c r="H48" s="162" t="e">
-        <f>SUM(H46:H47)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" s="182"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A50" s="182" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A51" s="182" t="s">
-        <v>166</v>
-      </c>
-      <c r="H51" s="162">
+      <c r="H47" s="162">
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="182" t="s">
-        <v>167</v>
+    <row r="48" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A48" s="182" t="s">
+        <v>168</v>
       </c>
-      <c r="H52" s="162">
-        <v>0</v>
+      <c r="H48" s="207">
+        <f>SUM(H43:H47)</f>
+        <v>-2122903.1780821919</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A53" s="182" t="s">
-        <v>168</v>
-      </c>
-      <c r="H53" s="207" t="e">
-        <f>SUM(H48:H52)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="49" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.85" right="0.5" top="0.75" bottom="0.17" header="0.17" footer="0.17"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4695,14 +4551,14 @@
       <c r="D8" s="3"/>
       <c r="E8" s="121">
         <f>+'P10'!J16</f>
-        <v>124812.82191780822</v>
+        <v>125312.82191780822</v>
       </c>
       <c r="F8" s="143"/>
     </row>
     <row r="9" spans="1:1003" x14ac:dyDescent="0.35">
       <c r="E9" s="126">
         <f>SUM(E8)</f>
-        <v>124812.82191780822</v>
+        <v>125312.82191780822</v>
       </c>
       <c r="F9" s="143"/>
     </row>
@@ -8752,7 +8608,7 @@
       <c r="B15" s="1"/>
       <c r="E15" s="127">
         <f>SUM(E14+E9)</f>
-        <v>250292.32191780821</v>
+        <v>250792.32191780821</v>
       </c>
       <c r="F15" s="101"/>
       <c r="G15" s="13"/>

</xml_diff>